<commit_message>
Actualiza ciclo Jul-26 con respuestas de hoteles recibidas en julio
Registra modificaciones de 8 hoteles (Arsenal, GHL Relax Club Hotel el Puente,
GHL Style Neiva, GHL Style Yopal, Hotel Tequendama Bogotá, Sonesta Cusco,
Sonesta Arequipa, Sonesta Bogotá), marca 3 hoteles sin modificaciones
(GHL Lago Titicaca, GHL Portón Medellín, GHL Style Barrancabermeja) y
refresca dashboard de cumplimiento y resumen por ciclo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -146,8 +146,28 @@
       <color rgb="00808080"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00856404"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001F4E79"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="009C0006"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00065F46"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -197,6 +217,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F4F8"/>
+        <bgColor rgb="00F0F4F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -284,7 +334,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -390,6 +440,17 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2962,18 +3023,30 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr"/>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="5" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>4 diálogos modificados: correcciones de junio no aplicadas — contacto reservas, day pass, camas twin, gimnasio</t>
+        </is>
+      </c>
       <c r="I46" s="6" t="inlineStr"/>
-      <c r="J46" s="5" t="inlineStr"/>
-      <c r="K46" s="5" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>El hotel reporta que estos 4 cambios ya se habían solicitado en junio y no se aplicaron en el chatbot; los reenvía</t>
+        </is>
+      </c>
+      <c r="K46" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
       <c r="L46" s="5" t="inlineStr"/>
@@ -3386,18 +3459,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr"/>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H56" s="5" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="n"/>
       <c r="I56" s="6" t="inlineStr"/>
-      <c r="J56" s="5" t="inlineStr"/>
-      <c r="K56" s="5" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>Envió observaciones en formato ambiguo (mixto español/inglés); se registra como sin modificaciones hasta aclarar con el hotel</t>
+        </is>
+      </c>
+      <c r="K56" s="38" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
       <c r="L56" s="5" t="inlineStr"/>
@@ -3470,18 +3551,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr"/>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="5" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="n"/>
       <c r="I58" s="6" t="inlineStr"/>
-      <c r="J58" s="5" t="inlineStr"/>
-      <c r="K58" s="5" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>Consultó sobre 2 teléfonos distintos en diálogos 10-04/10-06 vs. Reservation/Events; se registra como sin modificaciones hasta resolver la duda con el hotel</t>
+        </is>
+      </c>
+      <c r="K58" s="38" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
       <c r="L58" s="5" t="inlineStr"/>
@@ -3512,18 +3601,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F59" s="6" t="inlineStr"/>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H59" s="8" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H59" s="8" t="inlineStr">
+        <is>
+          <t>6 diálogos modificados: remodelación piscina/fechas, política menores, balcón, cajero ATM</t>
+        </is>
+      </c>
       <c r="I59" s="6" t="inlineStr"/>
-      <c r="J59" s="8" t="inlineStr"/>
-      <c r="K59" s="8" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J59" s="8" t="n"/>
+      <c r="K59" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
       <c r="L59" s="8" t="inlineStr"/>
@@ -3680,18 +3777,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F63" s="6" t="inlineStr"/>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H63" s="8" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H63" s="8" t="n"/>
       <c r="I63" s="6" t="inlineStr"/>
-      <c r="J63" s="8" t="inlineStr"/>
-      <c r="K63" s="8" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J63" s="8" t="inlineStr">
+        <is>
+          <t>Confirmó sin novedad para cambios</t>
+        </is>
+      </c>
+      <c r="K63" s="38" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
       <c r="L63" s="8" t="inlineStr"/>
@@ -3764,18 +3869,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F65" s="6" t="inlineStr"/>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H65" s="8" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H65" s="8" t="inlineStr">
+        <is>
+          <t>5 diálogos modificados: ubicación, check-in/out tardío, horario y tarifa de desayuno</t>
+        </is>
+      </c>
       <c r="I65" s="6" t="inlineStr"/>
-      <c r="J65" s="8" t="inlineStr"/>
-      <c r="K65" s="8" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J65" s="8" t="n"/>
+      <c r="K65" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
       <c r="L65" s="8" t="inlineStr"/>
@@ -3806,18 +3919,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr"/>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H66" s="5" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>2 diálogos modificados: check-in y check-out anticipado/tardío (aclaración de impuestos)</t>
+        </is>
+      </c>
       <c r="I66" s="6" t="inlineStr"/>
-      <c r="J66" s="5" t="inlineStr"/>
-      <c r="K66" s="5" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J66" s="5" t="n"/>
+      <c r="K66" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
       <c r="L66" s="5" t="inlineStr"/>
@@ -3848,18 +3969,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F67" s="6" t="inlineStr"/>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H67" s="8" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H67" s="8" t="inlineStr">
+        <is>
+          <t>2 diálogos modificados: cajero automático, horario y marcación de room service</t>
+        </is>
+      </c>
       <c r="I67" s="6" t="inlineStr"/>
-      <c r="J67" s="8" t="inlineStr"/>
-      <c r="K67" s="8" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J67" s="8" t="n"/>
+      <c r="K67" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
       <c r="L67" s="8" t="inlineStr"/>
@@ -3974,16 +4103,20 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F70" s="6" t="inlineStr"/>
+      <c r="F70" s="6" t="n"/>
       <c r="G70" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H70" s="5" t="inlineStr"/>
+      <c r="H70" s="5" t="n"/>
       <c r="I70" s="6" t="inlineStr"/>
-      <c r="J70" s="5" t="inlineStr"/>
-      <c r="K70" s="5" t="inlineStr">
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>Confirmó recibido (09/07) pero a la fecha no ha enviado la revisión</t>
+        </is>
+      </c>
+      <c r="K70" s="39" t="inlineStr">
         <is>
           <t>Sin respuesta</t>
         </is>
@@ -4268,18 +4401,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F77" s="6" t="inlineStr"/>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
       <c r="G77" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H77" s="8" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H77" s="8" t="inlineStr">
+        <is>
+          <t>4 diálogos modificados: contacto recepción, tarifas check-in/out, room service 24/7</t>
+        </is>
+      </c>
       <c r="I77" s="6" t="inlineStr"/>
-      <c r="J77" s="8" t="inlineStr"/>
-      <c r="K77" s="8" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J77" s="8" t="n"/>
+      <c r="K77" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
       <c r="L77" s="8" t="inlineStr"/>
@@ -4352,18 +4493,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F79" s="6" t="inlineStr"/>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
       <c r="G79" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H79" s="8" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H79" s="8" t="inlineStr">
+        <is>
+          <t>15 diálogos modificados: empleos, propinas, bar, spa x2, restaurante x6, brunch, san valentín, distancia al centro, celebraciones</t>
+        </is>
+      </c>
       <c r="I79" s="6" t="inlineStr"/>
-      <c r="J79" s="8" t="inlineStr"/>
-      <c r="K79" s="8" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J79" s="8" t="n"/>
+      <c r="K79" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
       <c r="L79" s="8" t="inlineStr"/>
@@ -4394,18 +4543,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F80" s="6" t="inlineStr"/>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>12/07/2026</t>
+        </is>
+      </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H80" s="5" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>8 diálogos modificados: check-in/out, desayuno horario/precio, niños, mascotas, redes, restaurante</t>
+        </is>
+      </c>
       <c r="I80" s="6" t="inlineStr"/>
-      <c r="J80" s="5" t="inlineStr"/>
-      <c r="K80" s="5" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J80" s="5" t="n"/>
+      <c r="K80" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
       <c r="L80" s="5" t="inlineStr"/>
@@ -4847,23 +5004,23 @@
         <v>42</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="I5" s="17">
@@ -4986,23 +5143,23 @@
         <v>42</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G4" s="20" t="n">
-        <v>0</v>
+        <v>0.2619047619047619</v>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>████████░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I4" s="22" t="inlineStr">
@@ -5056,23 +5213,23 @@
         <v>84</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E6" s="28" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F6" s="28" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G6" s="29" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.4047619047619048</v>
       </c>
       <c r="H6" s="30" t="inlineStr">
         <is>
-          <t>████████░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>████████████░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I6" s="28" t="inlineStr"/>
@@ -5101,7 +5258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H273"/>
+  <dimension ref="A1:H319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -15445,6 +15602,1754 @@
         </is>
       </c>
       <c r="H273" s="8" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B274" s="41" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C274" s="41" t="inlineStr">
+        <is>
+          <t>10-04</t>
+        </is>
+      </c>
+      <c r="D274" s="41" t="inlineStr">
+        <is>
+          <t>Reservation modification</t>
+        </is>
+      </c>
+      <c r="E274" s="41" t="inlineStr">
+        <is>
+          <t>Teléfono de contacto</t>
+        </is>
+      </c>
+      <c r="F274" s="41" t="inlineStr">
+        <is>
+          <t>+57 6056605831 (no se actualizó desde junio)</t>
+        </is>
+      </c>
+      <c r="G274" s="41" t="inlineStr">
+        <is>
+          <t>+57 3160107651</t>
+        </is>
+      </c>
+      <c r="H274" s="41" t="n"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B275" s="41" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C275" s="41" t="inlineStr">
+        <is>
+          <t>10-41</t>
+        </is>
+      </c>
+      <c r="D275" s="41" t="inlineStr">
+        <is>
+          <t>Day use / day pass</t>
+        </is>
+      </c>
+      <c r="E275" s="41" t="inlineStr">
+        <is>
+          <t>Precio</t>
+        </is>
+      </c>
+      <c r="F275" s="41" t="inlineStr">
+        <is>
+          <t>$150.000 COP tarifa única (no se actualizó desde junio)</t>
+        </is>
+      </c>
+      <c r="G275" s="41" t="inlineStr">
+        <is>
+          <t>$240.000 COP adultos / $120.000 COP niños</t>
+        </is>
+      </c>
+      <c r="H275" s="41" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B276" s="41" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C276" s="41" t="inlineStr">
+        <is>
+          <t>15-26</t>
+        </is>
+      </c>
+      <c r="D276" s="41" t="inlineStr">
+        <is>
+          <t>Twin beds</t>
+        </is>
+      </c>
+      <c r="E276" s="41" t="inlineStr">
+        <is>
+          <t>Teléfono de contacto</t>
+        </is>
+      </c>
+      <c r="F276" s="41" t="inlineStr">
+        <is>
+          <t>Tel +57 (605) 660 5831 (no se actualizó desde junio)</t>
+        </is>
+      </c>
+      <c r="G276" s="41" t="inlineStr">
+        <is>
+          <t>Celular +57 3160107651</t>
+        </is>
+      </c>
+      <c r="H276" s="41" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B277" s="41" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C277" s="41" t="inlineStr">
+        <is>
+          <t>17-31</t>
+        </is>
+      </c>
+      <c r="D277" s="41" t="inlineStr">
+        <is>
+          <t>Fitness gym</t>
+        </is>
+      </c>
+      <c r="E277" s="41" t="inlineStr">
+        <is>
+          <t>Instalaciones disponibles</t>
+        </is>
+      </c>
+      <c r="F277" s="41" t="inlineStr">
+        <is>
+          <t>Duchas y taquillas disponibles (no se actualizó desde junio)</t>
+        </is>
+      </c>
+      <c r="G277" s="41" t="inlineStr">
+        <is>
+          <t>No hay duchas ni taquillas; sí hay toallas y estación de agua filtrada</t>
+        </is>
+      </c>
+      <c r="H277" s="41" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B278" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C278" s="41" t="inlineStr">
+        <is>
+          <t>10-13</t>
+        </is>
+      </c>
+      <c r="D278" s="41" t="inlineStr">
+        <is>
+          <t>Opening, closing &amp; renovation</t>
+        </is>
+      </c>
+      <c r="E278" s="41" t="inlineStr">
+        <is>
+          <t>Estado de remodelación</t>
+        </is>
+      </c>
+      <c r="F278" s="41" t="inlineStr">
+        <is>
+          <t>Abrimos todo el año; sin remodelación prevista</t>
+        </is>
+      </c>
+      <c r="G278" s="41" t="inlineStr">
+        <is>
+          <t>Remodelación en curso; piscina principal, infantil y jacuzzi fuera de servicio hasta aprox. el 31 de agosto</t>
+        </is>
+      </c>
+      <c r="H278" s="41" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B279" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C279" s="41" t="inlineStr">
+        <is>
+          <t>10-42</t>
+        </is>
+      </c>
+      <c r="D279" s="41" t="inlineStr">
+        <is>
+          <t>Day use reservation</t>
+        </is>
+      </c>
+      <c r="E279" s="41" t="inlineStr">
+        <is>
+          <t>Fecha fin remodelación</t>
+        </is>
+      </c>
+      <c r="F279" s="41" t="inlineStr">
+        <is>
+          <t>Hasta aprox. el 15 de junio</t>
+        </is>
+      </c>
+      <c r="G279" s="41" t="inlineStr">
+        <is>
+          <t>Hasta aprox. el 31 de agosto</t>
+        </is>
+      </c>
+      <c r="H279" s="41" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B280" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C280" s="41" t="inlineStr">
+        <is>
+          <t>13-21</t>
+        </is>
+      </c>
+      <c r="D280" s="41" t="inlineStr">
+        <is>
+          <t>Kids</t>
+        </is>
+      </c>
+      <c r="E280" s="41" t="inlineStr">
+        <is>
+          <t>Política de ingreso de menores</t>
+        </is>
+      </c>
+      <c r="F280" s="41" t="inlineStr">
+        <is>
+          <t>Sin detalle de documentación requerida</t>
+        </is>
+      </c>
+      <c r="G280" s="41" t="inlineStr">
+        <is>
+          <t>Se agrega requisito de documento válido y autorización escrita para menores no acompañados por sus padres</t>
+        </is>
+      </c>
+      <c r="H280" s="41" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B281" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C281" s="41" t="inlineStr">
+        <is>
+          <t>15-61</t>
+        </is>
+      </c>
+      <c r="D281" s="41" t="inlineStr">
+        <is>
+          <t>Balcony &amp; windows</t>
+        </is>
+      </c>
+      <c r="E281" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad de balcón</t>
+        </is>
+      </c>
+      <c r="F281" s="41" t="inlineStr">
+        <is>
+          <t>Todas las habitaciones tienen balcón</t>
+        </is>
+      </c>
+      <c r="G281" s="41" t="inlineStr">
+        <is>
+          <t>Algunas habitaciones tienen balcón; no se reserva ubicación específica</t>
+        </is>
+      </c>
+      <c r="H281" s="41" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B282" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C282" s="41" t="inlineStr">
+        <is>
+          <t>17-61</t>
+        </is>
+      </c>
+      <c r="D282" s="41" t="inlineStr">
+        <is>
+          <t>Swimming pool</t>
+        </is>
+      </c>
+      <c r="E282" s="41" t="inlineStr">
+        <is>
+          <t>Fecha fin remodelación</t>
+        </is>
+      </c>
+      <c r="F282" s="41" t="inlineStr">
+        <is>
+          <t>Hasta aprox. el 15 de junio</t>
+        </is>
+      </c>
+      <c r="G282" s="41" t="inlineStr">
+        <is>
+          <t>Hasta aprox. el 31 de agosto</t>
+        </is>
+      </c>
+      <c r="H282" s="41" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B283" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C283" s="41" t="inlineStr">
+        <is>
+          <t>13-45</t>
+        </is>
+      </c>
+      <c r="D283" s="41" t="inlineStr">
+        <is>
+          <t>Change &amp; ATM</t>
+        </is>
+      </c>
+      <c r="E283" s="41" t="inlineStr">
+        <is>
+          <t>Cajero más cercano</t>
+        </is>
+      </c>
+      <c r="F283" s="41" t="inlineStr">
+        <is>
+          <t>Cajero ATH Eds Terpel / Banco Popular, Cra 5 #20-63, Girardot</t>
+        </is>
+      </c>
+      <c r="G283" s="41" t="inlineStr">
+        <is>
+          <t>C.cial Premier Jumbo Girardot: cajeros Bancolombia, BBVA, Servibanca, Avvillas</t>
+        </is>
+      </c>
+      <c r="H283" s="41" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B284" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Neiva</t>
+        </is>
+      </c>
+      <c r="C284" s="41" t="inlineStr">
+        <is>
+          <t>9-01</t>
+        </is>
+      </c>
+      <c r="D284" s="41" t="inlineStr">
+        <is>
+          <t>Ubicación</t>
+        </is>
+      </c>
+      <c r="E284" s="41" t="inlineStr">
+        <is>
+          <t>Dirección</t>
+        </is>
+      </c>
+      <c r="F284" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificada en el diálogo previo</t>
+        </is>
+      </c>
+      <c r="G284" s="41" t="inlineStr">
+        <is>
+          <t>Cra. 16 #42-195, Comuna 2, Neiva, Huila, Colombia</t>
+        </is>
+      </c>
+      <c r="H284" s="41" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B285" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Neiva</t>
+        </is>
+      </c>
+      <c r="C285" s="41" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="D285" s="41" t="inlineStr">
+        <is>
+          <t>Check-in time</t>
+        </is>
+      </c>
+      <c r="E285" s="41" t="inlineStr">
+        <is>
+          <t>Early check-in</t>
+        </is>
+      </c>
+      <c r="F285" s="41" t="inlineStr">
+        <is>
+          <t>Desde las 10:00, costo no especificado</t>
+        </is>
+      </c>
+      <c r="G285" s="41" t="inlineStr">
+        <is>
+          <t>Desde las 10:00, 150.000 COP por habitación, sujeto a disponibilidad</t>
+        </is>
+      </c>
+      <c r="H285" s="41" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B286" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Neiva</t>
+        </is>
+      </c>
+      <c r="C286" s="41" t="inlineStr">
+        <is>
+          <t>11-11</t>
+        </is>
+      </c>
+      <c r="D286" s="41" t="inlineStr">
+        <is>
+          <t>Check-out time</t>
+        </is>
+      </c>
+      <c r="E286" s="41" t="inlineStr">
+        <is>
+          <t>Check-out tardío</t>
+        </is>
+      </c>
+      <c r="F286" s="41" t="inlineStr">
+        <is>
+          <t>Hasta las 18:00, costo no especificado</t>
+        </is>
+      </c>
+      <c r="G286" s="41" t="inlineStr">
+        <is>
+          <t>Check-out regular hasta las 13:00; tardío hasta las 18:00 por 150.000 COP por habitación</t>
+        </is>
+      </c>
+      <c r="H286" s="41" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B287" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Neiva</t>
+        </is>
+      </c>
+      <c r="C287" s="41" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="D287" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E287" s="41" t="inlineStr">
+        <is>
+          <t>Horario desayuno</t>
+        </is>
+      </c>
+      <c r="F287" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G287" s="41" t="inlineStr">
+        <is>
+          <t>Buffet diario de 6:30 a.m. a 10:00 a.m.</t>
+        </is>
+      </c>
+      <c r="H287" s="41" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B288" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Neiva</t>
+        </is>
+      </c>
+      <c r="C288" s="41" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="D288" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E288" s="41" t="inlineStr">
+        <is>
+          <t>Precio adulto</t>
+        </is>
+      </c>
+      <c r="F288" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G288" s="41" t="inlineStr">
+        <is>
+          <t>40.000 COP por adulto; incluido en tarifa de habitación; visitantes también bienvenidos</t>
+        </is>
+      </c>
+      <c r="H288" s="41" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B289" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C289" s="41" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="D289" s="41" t="inlineStr">
+        <is>
+          <t>Check in time</t>
+        </is>
+      </c>
+      <c r="E289" s="41" t="inlineStr">
+        <is>
+          <t>Costo early check-in</t>
+        </is>
+      </c>
+      <c r="F289" s="41" t="inlineStr">
+        <is>
+          <t>70.000 COP por habitación</t>
+        </is>
+      </c>
+      <c r="G289" s="41" t="inlineStr">
+        <is>
+          <t>COP 70.000 + impuestos por habitación</t>
+        </is>
+      </c>
+      <c r="H289" s="41" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B290" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C290" s="41" t="inlineStr">
+        <is>
+          <t>11-11</t>
+        </is>
+      </c>
+      <c r="D290" s="41" t="inlineStr">
+        <is>
+          <t>Check out time</t>
+        </is>
+      </c>
+      <c r="E290" s="41" t="inlineStr">
+        <is>
+          <t>Costo late check-out</t>
+        </is>
+      </c>
+      <c r="F290" s="41" t="inlineStr">
+        <is>
+          <t>70.000 COP por habitación</t>
+        </is>
+      </c>
+      <c r="G290" s="41" t="inlineStr">
+        <is>
+          <t>COP 70.000 + impuestos por habitación</t>
+        </is>
+      </c>
+      <c r="H290" s="41" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B291" s="41" t="inlineStr">
+        <is>
+          <t>Hotel Tequendama Bogotá</t>
+        </is>
+      </c>
+      <c r="C291" s="41" t="inlineStr">
+        <is>
+          <t>13-45</t>
+        </is>
+      </c>
+      <c r="D291" s="41" t="inlineStr">
+        <is>
+          <t>Change &amp; ATM</t>
+        </is>
+      </c>
+      <c r="E291" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad de cajero automático</t>
+        </is>
+      </c>
+      <c r="F291" s="41" t="inlineStr">
+        <is>
+          <t>Sí tenemos un cajero automático en la propiedad</t>
+        </is>
+      </c>
+      <c r="G291" s="41" t="inlineStr">
+        <is>
+          <t>No tenemos un cajero automático en la propiedad</t>
+        </is>
+      </c>
+      <c r="H291" s="41" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B292" s="41" t="inlineStr">
+        <is>
+          <t>Hotel Tequendama Bogotá</t>
+        </is>
+      </c>
+      <c r="C292" s="41" t="inlineStr">
+        <is>
+          <t>13-06</t>
+        </is>
+      </c>
+      <c r="D292" s="41" t="inlineStr">
+        <is>
+          <t>Room Service</t>
+        </is>
+      </c>
+      <c r="E292" s="41" t="inlineStr">
+        <is>
+          <t>Horario y marcación</t>
+        </is>
+      </c>
+      <c r="F292" s="41" t="inlineStr">
+        <is>
+          <t>Disponible de 06:00 a 22:00; marcar 2356</t>
+        </is>
+      </c>
+      <c r="G292" s="41" t="inlineStr">
+        <is>
+          <t>Disponible de 06:00 a 00:00; marcar *2</t>
+        </is>
+      </c>
+      <c r="H292" s="41" t="n"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B293" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Cusco</t>
+        </is>
+      </c>
+      <c r="C293" s="41" t="inlineStr">
+        <is>
+          <t>16-02</t>
+        </is>
+      </c>
+      <c r="D293" s="41" t="inlineStr">
+        <is>
+          <t>Contact staff — Recepción</t>
+        </is>
+      </c>
+      <c r="E293" s="41" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
+      <c r="F293" s="41" t="inlineStr">
+        <is>
+          <t>recepcion.sonestahotelcusco@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="G293" s="41" t="inlineStr">
+        <is>
+          <t>recepcion.sonestacusco@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="H293" s="41" t="n"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B294" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Cusco</t>
+        </is>
+      </c>
+      <c r="C294" s="41" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="D294" s="41" t="inlineStr">
+        <is>
+          <t>Check-in time</t>
+        </is>
+      </c>
+      <c r="E294" s="41" t="inlineStr">
+        <is>
+          <t>Costo early check-in</t>
+        </is>
+      </c>
+      <c r="F294" s="41" t="inlineStr">
+        <is>
+          <t>40.00 USD por habitación</t>
+        </is>
+      </c>
+      <c r="G294" s="41" t="inlineStr">
+        <is>
+          <t>60.00 USD por habitación (impuestos no incluidos)</t>
+        </is>
+      </c>
+      <c r="H294" s="41" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B295" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Cusco</t>
+        </is>
+      </c>
+      <c r="C295" s="41" t="inlineStr">
+        <is>
+          <t>11-11</t>
+        </is>
+      </c>
+      <c r="D295" s="41" t="inlineStr">
+        <is>
+          <t>Check-out time</t>
+        </is>
+      </c>
+      <c r="E295" s="41" t="inlineStr">
+        <is>
+          <t>Costo late check-out</t>
+        </is>
+      </c>
+      <c r="F295" s="41" t="inlineStr">
+        <is>
+          <t>40.00 USD por habitación</t>
+        </is>
+      </c>
+      <c r="G295" s="41" t="inlineStr">
+        <is>
+          <t>60.00 USD por habitación</t>
+        </is>
+      </c>
+      <c r="H295" s="41" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B296" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Cusco</t>
+        </is>
+      </c>
+      <c r="C296" s="41" t="inlineStr">
+        <is>
+          <t>13-06</t>
+        </is>
+      </c>
+      <c r="D296" s="41" t="inlineStr">
+        <is>
+          <t>Room service</t>
+        </is>
+      </c>
+      <c r="E296" s="41" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="F296" s="41" t="inlineStr">
+        <is>
+          <t>Disponible de 06:00 a 21:00</t>
+        </is>
+      </c>
+      <c r="G296" s="41" t="inlineStr">
+        <is>
+          <t>Disponible 24/7</t>
+        </is>
+      </c>
+      <c r="H296" s="41" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B297" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C297" s="41" t="inlineStr">
+        <is>
+          <t>16-06</t>
+        </is>
+      </c>
+      <c r="D297" s="41" t="inlineStr">
+        <is>
+          <t>Jobs &amp; internships</t>
+        </is>
+      </c>
+      <c r="E297" s="41" t="inlineStr">
+        <is>
+          <t>Correo de contacto RR.HH.</t>
+        </is>
+      </c>
+      <c r="F297" s="41" t="inlineStr">
+        <is>
+          <t>contactenos@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="G297" s="41" t="inlineStr">
+        <is>
+          <t>laydy.pauca@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="H297" s="41" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B298" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C298" s="41" t="inlineStr">
+        <is>
+          <t>16-25</t>
+        </is>
+      </c>
+      <c r="D298" s="41" t="inlineStr">
+        <is>
+          <t>Tips policy</t>
+        </is>
+      </c>
+      <c r="E298" s="41" t="inlineStr">
+        <is>
+          <t>Política de propinas</t>
+        </is>
+      </c>
+      <c r="F298" s="41" t="inlineStr">
+        <is>
+          <t>Tarifa estándar incluye 19% de impuesto de servicio; propina habitual y opcional</t>
+        </is>
+      </c>
+      <c r="G298" s="41" t="inlineStr">
+        <is>
+          <t>Tarifa estándar incluye el cargo por servicio; propina opcional</t>
+        </is>
+      </c>
+      <c r="H298" s="41" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B299" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C299" s="41" t="inlineStr">
+        <is>
+          <t>17-01</t>
+        </is>
+      </c>
+      <c r="D299" s="41" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="E299" s="41" t="inlineStr">
+        <is>
+          <t>Detalles bar Arcadia</t>
+        </is>
+      </c>
+      <c r="F299" s="41" t="inlineStr">
+        <is>
+          <t>Capacidad máx. 25 pax; se sirve comida; sin happy hour listado por separado</t>
+        </is>
+      </c>
+      <c r="G299" s="41" t="inlineStr">
+        <is>
+          <t>Se retira capacidad máxima y mención de comida servida; resto de condiciones igual</t>
+        </is>
+      </c>
+      <c r="H299" s="41" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B300" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C300" s="41" t="inlineStr">
+        <is>
+          <t>17-02</t>
+        </is>
+      </c>
+      <c r="D300" s="41" t="inlineStr">
+        <is>
+          <t>Bar reservation</t>
+        </is>
+      </c>
+      <c r="E300" s="41" t="inlineStr">
+        <is>
+          <t>Reservas de bar</t>
+        </is>
+      </c>
+      <c r="F300" s="41" t="inlineStr">
+        <is>
+          <t>No se toman reservas</t>
+        </is>
+      </c>
+      <c r="G300" s="41" t="inlineStr">
+        <is>
+          <t>Para reservar, contactar al +51 945739921</t>
+        </is>
+      </c>
+      <c r="H300" s="41" t="n"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B301" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C301" s="41" t="inlineStr">
+        <is>
+          <t>17-10</t>
+        </is>
+      </c>
+      <c r="D301" s="41" t="inlineStr">
+        <is>
+          <t>Spa</t>
+        </is>
+      </c>
+      <c r="E301" s="41" t="inlineStr">
+        <is>
+          <t>Tarifas y kit obligatorio</t>
+        </is>
+      </c>
+      <c r="F301" s="41" t="inlineStr">
+        <is>
+          <t>Precio de huésped variable; obligatorio: pantuflas y vestido de baño; no obligatorio: bata y gorro</t>
+        </is>
+      </c>
+      <c r="G301" s="41" t="inlineStr">
+        <is>
+          <t>Masajes con cargo adicional; obligatorio: pantuflas, gorro y vestido de baño; no obligatorio: bata</t>
+        </is>
+      </c>
+      <c r="H301" s="41" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B302" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C302" s="41" t="inlineStr">
+        <is>
+          <t>17-15</t>
+        </is>
+      </c>
+      <c r="D302" s="41" t="inlineStr">
+        <is>
+          <t>Spa hours</t>
+        </is>
+      </c>
+      <c r="E302" s="41" t="inlineStr">
+        <is>
+          <t>Límite de tiempo</t>
+        </is>
+      </c>
+      <c r="F302" s="41" t="inlineStr">
+        <is>
+          <t>Sin límite de tiempo</t>
+        </is>
+      </c>
+      <c r="G302" s="41" t="inlineStr">
+        <is>
+          <t>Estancia máxima de 1 hora</t>
+        </is>
+      </c>
+      <c r="H302" s="41" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B303" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C303" s="41" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D303" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E303" s="41" t="inlineStr">
+        <is>
+          <t>Descripción restaurante Micaela</t>
+        </is>
+      </c>
+      <c r="F303" s="41" t="inlineStr">
+        <is>
+          <t>Descripción extensa (tipo de cocina, capacidad, niños, reservas, cajas altas, etc.)</t>
+        </is>
+      </c>
+      <c r="G303" s="41" t="inlineStr">
+        <is>
+          <t>Descripción simplificada: horario, accesibilidad, mascotas no aceptadas</t>
+        </is>
+      </c>
+      <c r="H303" s="41" t="n"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B304" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C304" s="41" t="inlineStr">
+        <is>
+          <t>18-02</t>
+        </is>
+      </c>
+      <c r="D304" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant reservation</t>
+        </is>
+      </c>
+      <c r="E304" s="41" t="inlineStr">
+        <is>
+          <t>Método de reserva</t>
+        </is>
+      </c>
+      <c r="F304" s="41" t="inlineStr">
+        <is>
+          <t>Reservar por correo a reservas.sonestaarequipa@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="G304" s="41" t="inlineStr">
+        <is>
+          <t>Contactar al +51 945739921</t>
+        </is>
+      </c>
+      <c r="H304" s="41" t="n"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B305" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C305" s="41" t="inlineStr">
+        <is>
+          <t>18-03</t>
+        </is>
+      </c>
+      <c r="D305" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant reservation cancellation</t>
+        </is>
+      </c>
+      <c r="E305" s="41" t="inlineStr">
+        <is>
+          <t>Método de cancelación</t>
+        </is>
+      </c>
+      <c r="F305" s="41" t="inlineStr">
+        <is>
+          <t>Cancelar por correo</t>
+        </is>
+      </c>
+      <c r="G305" s="41" t="inlineStr">
+        <is>
+          <t>Contactar al +51 945739921</t>
+        </is>
+      </c>
+      <c r="H305" s="41" t="n"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B306" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C306" s="41" t="inlineStr">
+        <is>
+          <t>18-04</t>
+        </is>
+      </c>
+      <c r="D306" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant reservation modification</t>
+        </is>
+      </c>
+      <c r="E306" s="41" t="inlineStr">
+        <is>
+          <t>Método de modificación</t>
+        </is>
+      </c>
+      <c r="F306" s="41" t="inlineStr">
+        <is>
+          <t>Modificar por correo</t>
+        </is>
+      </c>
+      <c r="G306" s="41" t="inlineStr">
+        <is>
+          <t>Contactar al +51 945739921</t>
+        </is>
+      </c>
+      <c r="H306" s="41" t="n"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B307" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C307" s="41" t="inlineStr">
+        <is>
+          <t>18-05</t>
+        </is>
+      </c>
+      <c r="D307" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant reservation confirmation</t>
+        </is>
+      </c>
+      <c r="E307" s="41" t="inlineStr">
+        <is>
+          <t>Método de confirmación</t>
+        </is>
+      </c>
+      <c r="F307" s="41" t="inlineStr">
+        <is>
+          <t>Confirmar por correo</t>
+        </is>
+      </c>
+      <c r="G307" s="41" t="inlineStr">
+        <is>
+          <t>Contactar al +51 945739921</t>
+        </is>
+      </c>
+      <c r="H307" s="41" t="n"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B308" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C308" s="41" t="inlineStr">
+        <is>
+          <t>18-11</t>
+        </is>
+      </c>
+      <c r="D308" s="41" t="inlineStr">
+        <is>
+          <t>Brunch</t>
+        </is>
+      </c>
+      <c r="E308" s="41" t="inlineStr">
+        <is>
+          <t>Recomendación externa</t>
+        </is>
+      </c>
+      <c r="F308" s="41" t="inlineStr">
+        <is>
+          <t>No ofrecen brunch; recomiendan Restaurante Santé como alternativa externa</t>
+        </is>
+      </c>
+      <c r="G308" s="41" t="inlineStr">
+        <is>
+          <t>No ofrecemos brunch (se retira la recomendación externa)</t>
+        </is>
+      </c>
+      <c r="H308" s="41" t="n"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B309" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C309" s="41" t="inlineStr">
+        <is>
+          <t>18-26</t>
+        </is>
+      </c>
+      <c r="D309" s="41" t="inlineStr">
+        <is>
+          <t>Valentine's day</t>
+        </is>
+      </c>
+      <c r="E309" s="41" t="inlineStr">
+        <is>
+          <t>Forma de consulta</t>
+        </is>
+      </c>
+      <c r="F309" s="41" t="inlineStr">
+        <is>
+          <t>Ver oferta mediante enlace</t>
+        </is>
+      </c>
+      <c r="G309" s="41" t="inlineStr">
+        <is>
+          <t>Escribir a reservas.sonestaarequipa@ghlhoteles.com o contactar al +51 939753285</t>
+        </is>
+      </c>
+      <c r="H309" s="41" t="n"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B310" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C310" s="41" t="inlineStr">
+        <is>
+          <t>19-03</t>
+        </is>
+      </c>
+      <c r="D310" s="41" t="inlineStr">
+        <is>
+          <t>City center</t>
+        </is>
+      </c>
+      <c r="E310" s="41" t="inlineStr">
+        <is>
+          <t>Distancia al centro</t>
+        </is>
+      </c>
+      <c r="F310" s="41" t="inlineStr">
+        <is>
+          <t>26 m, 1 min caminando</t>
+        </is>
+      </c>
+      <c r="G310" s="41" t="inlineStr">
+        <is>
+          <t>4 km</t>
+        </is>
+      </c>
+      <c r="H310" s="41" t="n"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B311" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C311" s="41" t="inlineStr">
+        <is>
+          <t>20-21</t>
+        </is>
+      </c>
+      <c r="D311" s="41" t="inlineStr">
+        <is>
+          <t>Celebration</t>
+        </is>
+      </c>
+      <c r="E311" s="41" t="inlineStr">
+        <is>
+          <t>Teléfono de eventos</t>
+        </is>
+      </c>
+      <c r="F311" s="41" t="inlineStr">
+        <is>
+          <t>+51 945 739 48</t>
+        </is>
+      </c>
+      <c r="G311" s="41" t="inlineStr">
+        <is>
+          <t>+51 945 739 484 (corrección de dígito faltante)</t>
+        </is>
+      </c>
+      <c r="H311" s="41" t="n"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B312" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C312" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D312" s="41" t="inlineStr">
+        <is>
+          <t>Check in time</t>
+        </is>
+      </c>
+      <c r="E312" s="41" t="inlineStr">
+        <is>
+          <t>Costo early check-in</t>
+        </is>
+      </c>
+      <c r="F312" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G312" s="41" t="inlineStr">
+        <is>
+          <t>$35.000, sujeto a disponibilidad</t>
+        </is>
+      </c>
+      <c r="H312" s="41" t="n"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B313" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C313" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D313" s="41" t="inlineStr">
+        <is>
+          <t>Check out time</t>
+        </is>
+      </c>
+      <c r="E313" s="41" t="inlineStr">
+        <is>
+          <t>Late check-out</t>
+        </is>
+      </c>
+      <c r="F313" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G313" s="41" t="inlineStr">
+        <is>
+          <t>$35.000 por hora; después de las 6:00 p.m. se cobra la tarifa completa</t>
+        </is>
+      </c>
+      <c r="H313" s="41" t="n"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B314" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C314" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D314" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E314" s="41" t="inlineStr">
+        <is>
+          <t>Horario sábados, domingos y festivos</t>
+        </is>
+      </c>
+      <c r="F314" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G314" s="41" t="inlineStr">
+        <is>
+          <t>6:30 a.m. a 10:30 a.m.</t>
+        </is>
+      </c>
+      <c r="H314" s="41" t="n"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B315" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C315" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D315" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E315" s="41" t="inlineStr">
+        <is>
+          <t>Precio por persona</t>
+        </is>
+      </c>
+      <c r="F315" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G315" s="41" t="inlineStr">
+        <is>
+          <t>$65.000 COP</t>
+        </is>
+      </c>
+      <c r="H315" s="41" t="n"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B316" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C316" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D316" s="41" t="inlineStr">
+        <is>
+          <t>Kids</t>
+        </is>
+      </c>
+      <c r="E316" s="41" t="inlineStr">
+        <is>
+          <t>Tarifa niños</t>
+        </is>
+      </c>
+      <c r="F316" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G316" s="41" t="inlineStr">
+        <is>
+          <t>Menores de 12 años gratis con sus padres; mayores de 12 años $80.000 por noche</t>
+        </is>
+      </c>
+      <c r="H316" s="41" t="n"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B317" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C317" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D317" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E317" s="41" t="inlineStr">
+        <is>
+          <t>Peso permitido</t>
+        </is>
+      </c>
+      <c r="F317" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G317" s="41" t="inlineStr">
+        <is>
+          <t>10 kg</t>
+        </is>
+      </c>
+      <c r="H317" s="41" t="n"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B318" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C318" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D318" s="41" t="inlineStr">
+        <is>
+          <t>Social &amp; photoshoot</t>
+        </is>
+      </c>
+      <c r="E318" s="41" t="inlineStr">
+        <is>
+          <t>Correo de contacto</t>
+        </is>
+      </c>
+      <c r="F318" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G318" s="41" t="inlineStr">
+        <is>
+          <t>cateryne.palacios@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="H318" s="41" t="n"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B319" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C319" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D319" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant Cook's Restaurante</t>
+        </is>
+      </c>
+      <c r="E319" s="41" t="inlineStr">
+        <is>
+          <t>Horario de apertura</t>
+        </is>
+      </c>
+      <c r="F319" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G319" s="41" t="inlineStr">
+        <is>
+          <t>6:00 a.m. a 12:00 p.m.</t>
+        </is>
+      </c>
+      <c r="H319" s="41" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H227"/>

</xml_diff>

<commit_message>
Confirma actualización en chatbot de los 8 hoteles con cambios de julio
Marca fecha de actualización en chatbot (15/07/2026) y cambia estado de
"Pendiente actualización" a "Actualizado" para Arsenal, GHL Relax Club Hotel
el Puente, GHL Style Neiva, GHL Style Yopal, Hotel Tequendama Bogotá,
Sonesta Cusco, Sonesta Arequipa y Sonesta Bogotá.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -166,8 +166,13 @@
       <color rgb="00065F46"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00006100"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -247,6 +252,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F0F4F8"/>
         <bgColor rgb="00F0F4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -334,7 +345,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -451,6 +462,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3038,15 +3052,19 @@
           <t>4 diálogos modificados: correcciones de junio no aplicadas — contacto reservas, day pass, camas twin, gimnasio</t>
         </is>
       </c>
-      <c r="I46" s="6" t="inlineStr"/>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
           <t>El hotel reporta que estos 4 cambios ya se habían solicitado en junio y no se aplicaron en el chatbot; los reenvía</t>
         </is>
       </c>
-      <c r="K46" s="37" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K46" s="42" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
       <c r="L46" s="5" t="inlineStr"/>
@@ -3616,11 +3634,15 @@
           <t>6 diálogos modificados: remodelación piscina/fechas, política menores, balcón, cajero ATM</t>
         </is>
       </c>
-      <c r="I59" s="6" t="inlineStr"/>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="J59" s="8" t="n"/>
-      <c r="K59" s="37" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K59" s="42" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
       <c r="L59" s="8" t="inlineStr"/>
@@ -3884,11 +3906,15 @@
           <t>5 diálogos modificados: ubicación, check-in/out tardío, horario y tarifa de desayuno</t>
         </is>
       </c>
-      <c r="I65" s="6" t="inlineStr"/>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="J65" s="8" t="n"/>
-      <c r="K65" s="37" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K65" s="42" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
       <c r="L65" s="8" t="inlineStr"/>
@@ -3934,11 +3960,15 @@
           <t>2 diálogos modificados: check-in y check-out anticipado/tardío (aclaración de impuestos)</t>
         </is>
       </c>
-      <c r="I66" s="6" t="inlineStr"/>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="J66" s="5" t="n"/>
-      <c r="K66" s="37" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K66" s="42" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
       <c r="L66" s="5" t="inlineStr"/>
@@ -3984,11 +4014,15 @@
           <t>2 diálogos modificados: cajero automático, horario y marcación de room service</t>
         </is>
       </c>
-      <c r="I67" s="6" t="inlineStr"/>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="J67" s="8" t="n"/>
-      <c r="K67" s="37" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K67" s="42" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
       <c r="L67" s="8" t="inlineStr"/>
@@ -4416,11 +4450,15 @@
           <t>4 diálogos modificados: contacto recepción, tarifas check-in/out, room service 24/7</t>
         </is>
       </c>
-      <c r="I77" s="6" t="inlineStr"/>
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="J77" s="8" t="n"/>
-      <c r="K77" s="37" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K77" s="42" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
       <c r="L77" s="8" t="inlineStr"/>
@@ -4508,11 +4546,15 @@
           <t>15 diálogos modificados: empleos, propinas, bar, spa x2, restaurante x6, brunch, san valentín, distancia al centro, celebraciones</t>
         </is>
       </c>
-      <c r="I79" s="6" t="inlineStr"/>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="J79" s="8" t="n"/>
-      <c r="K79" s="37" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K79" s="42" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
       <c r="L79" s="8" t="inlineStr"/>
@@ -4558,11 +4600,15 @@
           <t>8 diálogos modificados: check-in/out, desayuno horario/precio, niños, mascotas, redes, restaurante</t>
         </is>
       </c>
-      <c r="I80" s="6" t="inlineStr"/>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="J80" s="5" t="n"/>
-      <c r="K80" s="37" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K80" s="42" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
       <c r="L80" s="5" t="inlineStr"/>
@@ -5016,7 +5062,7 @@
         <v>3</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Registra sin cambios de julio para Armeria Real, Hamilton y Villavicencio
Armeria Real, GHL Collection Hamilton y GHL Grand Villavicencio confirman
que no tienen modificaciones para el ciclo Jul-26. Se marcan como "Sin
modificaciones" y se refrescan los totales de Dashboard cumplimiento y
Resumen por ciclo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -3309,18 +3309,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr"/>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="6" t="inlineStr"/>
-      <c r="J52" s="5" t="inlineStr"/>
-      <c r="K52" s="5" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para julio</t>
+        </is>
+      </c>
+      <c r="K52" s="38" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
       <c r="L52" s="5" t="inlineStr"/>
@@ -3351,18 +3359,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H53" s="8" t="inlineStr"/>
       <c r="I53" s="6" t="inlineStr"/>
-      <c r="J53" s="8" t="inlineStr"/>
-      <c r="K53" s="8" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J53" s="8" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para julio</t>
+        </is>
+      </c>
+      <c r="K53" s="38" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
       <c r="L53" s="8" t="inlineStr"/>
@@ -3393,18 +3409,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr"/>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="6" t="inlineStr"/>
-      <c r="J54" s="5" t="inlineStr"/>
-      <c r="K54" s="5" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para julio</t>
+        </is>
+      </c>
+      <c r="K54" s="38" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
       <c r="L54" s="5" t="inlineStr"/>
@@ -5050,23 +5074,23 @@
         <v>42</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>8</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G5" s="12" t="n">
         <v>8</v>
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="I5" s="17">
@@ -5189,23 +5213,23 @@
         <v>42</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E4" s="19" t="n">
         <v>8</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G4" s="20" t="n">
-        <v>0.2619047619047619</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>████████░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>██████████░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I4" s="22" t="inlineStr">
@@ -5259,23 +5283,23 @@
         <v>84</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E6" s="28" t="n">
         <v>31</v>
       </c>
       <c r="F6" s="28" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G6" s="29" t="n">
-        <v>0.4047619047619048</v>
+        <v>0.4404761904761905</v>
       </c>
       <c r="H6" s="30" t="inlineStr">
         <is>
-          <t>████████████░░░░░░░░░░░░░░░░░░</t>
+          <t>█████████████░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I6" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Registra sin cambios de julio para GHL Hotel Abadía Plaza y Costa Azul
GHL Hotel Abadía Plaza y GHL Relax Hotel Costa Azul confirman que no
tienen modificaciones para el ciclo Jul-26. Se marcan como "Sin
modificaciones" y se refrescan los totales de Dashboard cumplimiento y
Resumen por ciclo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -3739,18 +3739,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F61" s="6" t="inlineStr"/>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr"/>
       <c r="I61" s="6" t="inlineStr"/>
-      <c r="J61" s="8" t="inlineStr"/>
-      <c r="K61" s="8" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J61" s="8" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para julio</t>
+        </is>
+      </c>
+      <c r="K61" s="38" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
       <c r="L61" s="8" t="inlineStr"/>
@@ -4077,18 +4085,26 @@
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F68" s="6" t="inlineStr"/>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr"/>
       <c r="I68" s="6" t="inlineStr"/>
-      <c r="J68" s="5" t="inlineStr"/>
-      <c r="K68" s="5" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para julio</t>
+        </is>
+      </c>
+      <c r="K68" s="38" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
       <c r="L68" s="5" t="inlineStr"/>
@@ -5074,23 +5090,23 @@
         <v>42</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>8</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G5" s="12" t="n">
         <v>8</v>
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="I5" s="17">
@@ -5213,23 +5229,23 @@
         <v>42</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E4" s="19" t="n">
         <v>8</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G4" s="20" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>██████████░░░░░░░░░░░░░░░░░░░░</t>
+          <t>███████████░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I4" s="22" t="inlineStr">
@@ -5283,23 +5299,23 @@
         <v>84</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E6" s="28" t="n">
         <v>31</v>
       </c>
       <c r="F6" s="28" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G6" s="29" t="n">
-        <v>0.4404761904761905</v>
+        <v>0.4642857142857143</v>
       </c>
       <c r="H6" s="30" t="inlineStr">
         <is>
-          <t>█████████████░░░░░░░░░░░░░░░░░</t>
+          <t>██████████████░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I6" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Actualiza correo de contacto de Bioxury
Reemplaza el correo compartido con Sonesta Bogotá (catalina.rojas@ghlhoteles.com)
por el correo propio de Bioxury: calidad.bioxury@ghlhoteles.com, en los ciclos
Jun-26 y Jul-26. Aún no se tiene nombre de contacto.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -1040,12 +1040,12 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Andrea Rojas</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>catalina.rojas@ghlhoteles.com</t>
+          <t>calidad.bioxury@ghlhoteles.com</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1063,7 +1063,7 @@
       <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>⚠ El correo catalina.rojas@ghlhoteles.com ahora corresponde a Sonesta Bogotá (Catalina Rojas) — verificar/definir contacto propio de Bioxury</t>
+          <t>Correo actualizado a calidad.bioxury@ghlhoteles.com; sin nombre de contacto</t>
         </is>
       </c>
       <c r="K6" s="22" t="inlineStr">
@@ -3124,12 +3124,12 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Andrea Rojas</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>catalina.rojas@ghlhoteles.com</t>
+          <t>calidad.bioxury@ghlhoteles.com</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
@@ -3147,7 +3147,7 @@
       <c r="I48" s="6" t="inlineStr"/>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>⚠ El correo catalina.rojas@ghlhoteles.com ahora corresponde a Sonesta Bogotá (Catalina Rojas) — verificar/definir contacto propio de Bioxury</t>
+          <t>Correo actualizado a calidad.bioxury@ghlhoteles.com; sin nombre de contacto</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Corrige fecha de actualización de 15/07 a 30/07/2026
La fecha usada como "hoy" en los registros de confirmación de julio estaba
mal (15/07 en vez de 30/07). Corrige fechaChatbot de los 8 hoteles
actualizados y fecha de respuesta de los 5 hoteles sin modificaciones.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -3054,7 +3054,7 @@
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
@@ -3311,7 +3311,7 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -3361,7 +3361,7 @@
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="I59" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="J59" s="8" t="n"/>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="I65" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="J65" s="8" t="n"/>
@@ -3994,7 +3994,7 @@
       </c>
       <c r="I66" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="J66" s="5" t="n"/>
@@ -4048,7 +4048,7 @@
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="J67" s="8" t="n"/>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
@@ -4492,7 +4492,7 @@
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="J77" s="8" t="n"/>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="I79" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="J79" s="8" t="n"/>
@@ -4642,7 +4642,7 @@
       </c>
       <c r="I80" s="6" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="J80" s="5" t="n"/>
@@ -17767,6 +17767,8 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Corrige registros de Sonesta Bogotá y GHL Style Neiva usando PDFs de julio
Al comparar contra los PDFs reales enviados en julio (carpeta JULIO), se
detectó que los 8 "cambios" de Sonesta Bogotá y 2 de los 5 de GHL Style
Neiva (horario/tarifa desayuno) ya coincidían con el contenido vigente del
chatbot — no eran modificaciones reales, solo confirmaciones del hotel.

- Sonesta Bogotá: pasa de "Actualizado" a "Sin modificaciones".
- GHL Style Neiva: se retiran los 2 diálogos de desayuno; se corrige el
  diálogo de ubicación de "9-01" a "19-01 - Location" con la dirección
  anterior real (Cra. 8a) tomada del PDF.
- Se refrescan Dashboard cumplimiento y Resumen por ciclo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -3935,7 +3935,7 @@
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>5 diálogos modificados: ubicación, check-in/out tardío, horario y tarifa de desayuno</t>
+          <t>3 diálogos modificados: ubicación, check-in/out tardío</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -3943,7 +3943,11 @@
           <t>30/07/2026</t>
         </is>
       </c>
-      <c r="J65" s="8" t="n"/>
+      <c r="J65" s="8" t="inlineStr">
+        <is>
+          <t>Se retiran horario y tarifa de desayuno del listado: coinciden con el PDF de julio vigente, no eran cambios reales</t>
+        </is>
+      </c>
       <c r="K65" s="42" t="inlineStr">
         <is>
           <t>Actualizado</t>
@@ -4632,23 +4636,19 @@
       </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H80" s="5" t="inlineStr">
-        <is>
-          <t>8 diálogos modificados: check-in/out, desayuno horario/precio, niños, mascotas, redes, restaurante</t>
-        </is>
-      </c>
-      <c r="I80" s="6" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="J80" s="5" t="n"/>
-      <c r="K80" s="42" t="inlineStr">
-        <is>
-          <t>Actualizado</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="n"/>
+      <c r="I80" s="6" t="n"/>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>Los 8 puntos que reportó ya coinciden con el PDF de julio vigente — no eran cambios reales, solo confirmó valores ya correctos</t>
+        </is>
+      </c>
+      <c r="K80" s="38" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
       <c r="L80" s="5" t="inlineStr"/>
@@ -5096,13 +5096,13 @@
         <v>26</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
@@ -5235,10 +5235,10 @@
         <v>26</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G4" s="20" t="n">
         <v>0.3809523809523809</v>
@@ -5305,10 +5305,10 @@
         <v>45</v>
       </c>
       <c r="E6" s="28" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F6" s="28" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G6" s="29" t="n">
         <v>0.4642857142857143</v>
@@ -5344,7 +5344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H319"/>
+  <dimension ref="A1:H309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16082,7 +16082,7 @@
       </c>
       <c r="C284" s="41" t="inlineStr">
         <is>
-          <t>9-01</t>
+          <t>19-01</t>
         </is>
       </c>
       <c r="D284" s="41" t="inlineStr">
@@ -16097,7 +16097,7 @@
       </c>
       <c r="F284" s="41" t="inlineStr">
         <is>
-          <t>⚠ No especificada en el diálogo previo</t>
+          <t>Cra. 8a #38-42, Comuna 2, Neiva, Huila, Colombia</t>
         </is>
       </c>
       <c r="G284" s="41" t="inlineStr">
@@ -16191,32 +16191,32 @@
       </c>
       <c r="B287" s="41" t="inlineStr">
         <is>
-          <t>GHL Style Neiva</t>
+          <t>GHL Style Yopal</t>
         </is>
       </c>
       <c r="C287" s="41" t="inlineStr">
         <is>
-          <t>12-01</t>
+          <t>11-01</t>
         </is>
       </c>
       <c r="D287" s="41" t="inlineStr">
         <is>
-          <t>Breakfast time</t>
+          <t>Check in time</t>
         </is>
       </c>
       <c r="E287" s="41" t="inlineStr">
         <is>
-          <t>Horario desayuno</t>
+          <t>Costo early check-in</t>
         </is>
       </c>
       <c r="F287" s="41" t="inlineStr">
         <is>
-          <t>⚠ No especificado</t>
+          <t>70.000 COP por habitación</t>
         </is>
       </c>
       <c r="G287" s="41" t="inlineStr">
         <is>
-          <t>Buffet diario de 6:30 a.m. a 10:00 a.m.</t>
+          <t>COP 70.000 + impuestos por habitación</t>
         </is>
       </c>
       <c r="H287" s="41" t="n"/>
@@ -16229,32 +16229,32 @@
       </c>
       <c r="B288" s="41" t="inlineStr">
         <is>
-          <t>GHL Style Neiva</t>
+          <t>GHL Style Yopal</t>
         </is>
       </c>
       <c r="C288" s="41" t="inlineStr">
         <is>
-          <t>12-02</t>
+          <t>11-11</t>
         </is>
       </c>
       <c r="D288" s="41" t="inlineStr">
         <is>
-          <t>Breakfast rates</t>
+          <t>Check out time</t>
         </is>
       </c>
       <c r="E288" s="41" t="inlineStr">
         <is>
-          <t>Precio adulto</t>
+          <t>Costo late check-out</t>
         </is>
       </c>
       <c r="F288" s="41" t="inlineStr">
         <is>
-          <t>⚠ No especificado</t>
+          <t>70.000 COP por habitación</t>
         </is>
       </c>
       <c r="G288" s="41" t="inlineStr">
         <is>
-          <t>40.000 COP por adulto; incluido en tarifa de habitación; visitantes también bienvenidos</t>
+          <t>COP 70.000 + impuestos por habitación</t>
         </is>
       </c>
       <c r="H288" s="41" t="n"/>
@@ -16267,32 +16267,32 @@
       </c>
       <c r="B289" s="41" t="inlineStr">
         <is>
-          <t>GHL Style Yopal</t>
+          <t>Hotel Tequendama Bogotá</t>
         </is>
       </c>
       <c r="C289" s="41" t="inlineStr">
         <is>
-          <t>11-01</t>
+          <t>13-45</t>
         </is>
       </c>
       <c r="D289" s="41" t="inlineStr">
         <is>
-          <t>Check in time</t>
+          <t>Change &amp; ATM</t>
         </is>
       </c>
       <c r="E289" s="41" t="inlineStr">
         <is>
-          <t>Costo early check-in</t>
+          <t>Disponibilidad de cajero automático</t>
         </is>
       </c>
       <c r="F289" s="41" t="inlineStr">
         <is>
-          <t>70.000 COP por habitación</t>
+          <t>Sí tenemos un cajero automático en la propiedad</t>
         </is>
       </c>
       <c r="G289" s="41" t="inlineStr">
         <is>
-          <t>COP 70.000 + impuestos por habitación</t>
+          <t>No tenemos un cajero automático en la propiedad</t>
         </is>
       </c>
       <c r="H289" s="41" t="n"/>
@@ -16305,32 +16305,32 @@
       </c>
       <c r="B290" s="41" t="inlineStr">
         <is>
-          <t>GHL Style Yopal</t>
+          <t>Hotel Tequendama Bogotá</t>
         </is>
       </c>
       <c r="C290" s="41" t="inlineStr">
         <is>
-          <t>11-11</t>
+          <t>13-06</t>
         </is>
       </c>
       <c r="D290" s="41" t="inlineStr">
         <is>
-          <t>Check out time</t>
+          <t>Room Service</t>
         </is>
       </c>
       <c r="E290" s="41" t="inlineStr">
         <is>
-          <t>Costo late check-out</t>
+          <t>Horario y marcación</t>
         </is>
       </c>
       <c r="F290" s="41" t="inlineStr">
         <is>
-          <t>70.000 COP por habitación</t>
+          <t>Disponible de 06:00 a 22:00; marcar 2356</t>
         </is>
       </c>
       <c r="G290" s="41" t="inlineStr">
         <is>
-          <t>COP 70.000 + impuestos por habitación</t>
+          <t>Disponible de 06:00 a 00:00; marcar *2</t>
         </is>
       </c>
       <c r="H290" s="41" t="n"/>
@@ -16343,32 +16343,32 @@
       </c>
       <c r="B291" s="41" t="inlineStr">
         <is>
-          <t>Hotel Tequendama Bogotá</t>
+          <t>Sonesta Cusco</t>
         </is>
       </c>
       <c r="C291" s="41" t="inlineStr">
         <is>
-          <t>13-45</t>
+          <t>16-02</t>
         </is>
       </c>
       <c r="D291" s="41" t="inlineStr">
         <is>
-          <t>Change &amp; ATM</t>
+          <t>Contact staff — Recepción</t>
         </is>
       </c>
       <c r="E291" s="41" t="inlineStr">
         <is>
-          <t>Disponibilidad de cajero automático</t>
+          <t>Correo</t>
         </is>
       </c>
       <c r="F291" s="41" t="inlineStr">
         <is>
-          <t>Sí tenemos un cajero automático en la propiedad</t>
+          <t>recepcion.sonestahotelcusco@ghlhoteles.com</t>
         </is>
       </c>
       <c r="G291" s="41" t="inlineStr">
         <is>
-          <t>No tenemos un cajero automático en la propiedad</t>
+          <t>recepcion.sonestacusco@ghlhoteles.com</t>
         </is>
       </c>
       <c r="H291" s="41" t="n"/>
@@ -16381,32 +16381,32 @@
       </c>
       <c r="B292" s="41" t="inlineStr">
         <is>
-          <t>Hotel Tequendama Bogotá</t>
+          <t>Sonesta Cusco</t>
         </is>
       </c>
       <c r="C292" s="41" t="inlineStr">
         <is>
-          <t>13-06</t>
+          <t>11-01</t>
         </is>
       </c>
       <c r="D292" s="41" t="inlineStr">
         <is>
-          <t>Room Service</t>
+          <t>Check-in time</t>
         </is>
       </c>
       <c r="E292" s="41" t="inlineStr">
         <is>
-          <t>Horario y marcación</t>
+          <t>Costo early check-in</t>
         </is>
       </c>
       <c r="F292" s="41" t="inlineStr">
         <is>
-          <t>Disponible de 06:00 a 22:00; marcar 2356</t>
+          <t>40.00 USD por habitación</t>
         </is>
       </c>
       <c r="G292" s="41" t="inlineStr">
         <is>
-          <t>Disponible de 06:00 a 00:00; marcar *2</t>
+          <t>60.00 USD por habitación (impuestos no incluidos)</t>
         </is>
       </c>
       <c r="H292" s="41" t="n"/>
@@ -16424,27 +16424,27 @@
       </c>
       <c r="C293" s="41" t="inlineStr">
         <is>
-          <t>16-02</t>
+          <t>11-11</t>
         </is>
       </c>
       <c r="D293" s="41" t="inlineStr">
         <is>
-          <t>Contact staff — Recepción</t>
+          <t>Check-out time</t>
         </is>
       </c>
       <c r="E293" s="41" t="inlineStr">
         <is>
-          <t>Correo</t>
+          <t>Costo late check-out</t>
         </is>
       </c>
       <c r="F293" s="41" t="inlineStr">
         <is>
-          <t>recepcion.sonestahotelcusco@ghlhoteles.com</t>
+          <t>40.00 USD por habitación</t>
         </is>
       </c>
       <c r="G293" s="41" t="inlineStr">
         <is>
-          <t>recepcion.sonestacusco@ghlhoteles.com</t>
+          <t>60.00 USD por habitación</t>
         </is>
       </c>
       <c r="H293" s="41" t="n"/>
@@ -16462,27 +16462,27 @@
       </c>
       <c r="C294" s="41" t="inlineStr">
         <is>
-          <t>11-01</t>
+          <t>13-06</t>
         </is>
       </c>
       <c r="D294" s="41" t="inlineStr">
         <is>
-          <t>Check-in time</t>
+          <t>Room service</t>
         </is>
       </c>
       <c r="E294" s="41" t="inlineStr">
         <is>
-          <t>Costo early check-in</t>
+          <t>Horario</t>
         </is>
       </c>
       <c r="F294" s="41" t="inlineStr">
         <is>
-          <t>40.00 USD por habitación</t>
+          <t>Disponible de 06:00 a 21:00</t>
         </is>
       </c>
       <c r="G294" s="41" t="inlineStr">
         <is>
-          <t>60.00 USD por habitación (impuestos no incluidos)</t>
+          <t>Disponible 24/7</t>
         </is>
       </c>
       <c r="H294" s="41" t="n"/>
@@ -16495,32 +16495,32 @@
       </c>
       <c r="B295" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Cusco</t>
+          <t>Sonesta Arequipa</t>
         </is>
       </c>
       <c r="C295" s="41" t="inlineStr">
         <is>
-          <t>11-11</t>
+          <t>16-06</t>
         </is>
       </c>
       <c r="D295" s="41" t="inlineStr">
         <is>
-          <t>Check-out time</t>
+          <t>Jobs &amp; internships</t>
         </is>
       </c>
       <c r="E295" s="41" t="inlineStr">
         <is>
-          <t>Costo late check-out</t>
+          <t>Correo de contacto RR.HH.</t>
         </is>
       </c>
       <c r="F295" s="41" t="inlineStr">
         <is>
-          <t>40.00 USD por habitación</t>
+          <t>contactenos@ghlhoteles.com</t>
         </is>
       </c>
       <c r="G295" s="41" t="inlineStr">
         <is>
-          <t>60.00 USD por habitación</t>
+          <t>laydy.pauca@ghlhoteles.com</t>
         </is>
       </c>
       <c r="H295" s="41" t="n"/>
@@ -16533,32 +16533,32 @@
       </c>
       <c r="B296" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Cusco</t>
+          <t>Sonesta Arequipa</t>
         </is>
       </c>
       <c r="C296" s="41" t="inlineStr">
         <is>
-          <t>13-06</t>
+          <t>16-25</t>
         </is>
       </c>
       <c r="D296" s="41" t="inlineStr">
         <is>
-          <t>Room service</t>
+          <t>Tips policy</t>
         </is>
       </c>
       <c r="E296" s="41" t="inlineStr">
         <is>
-          <t>Horario</t>
+          <t>Política de propinas</t>
         </is>
       </c>
       <c r="F296" s="41" t="inlineStr">
         <is>
-          <t>Disponible de 06:00 a 21:00</t>
+          <t>Tarifa estándar incluye 19% de impuesto de servicio; propina habitual y opcional</t>
         </is>
       </c>
       <c r="G296" s="41" t="inlineStr">
         <is>
-          <t>Disponible 24/7</t>
+          <t>Tarifa estándar incluye el cargo por servicio; propina opcional</t>
         </is>
       </c>
       <c r="H296" s="41" t="n"/>
@@ -16576,27 +16576,27 @@
       </c>
       <c r="C297" s="41" t="inlineStr">
         <is>
-          <t>16-06</t>
+          <t>17-01</t>
         </is>
       </c>
       <c r="D297" s="41" t="inlineStr">
         <is>
-          <t>Jobs &amp; internships</t>
+          <t>Bar</t>
         </is>
       </c>
       <c r="E297" s="41" t="inlineStr">
         <is>
-          <t>Correo de contacto RR.HH.</t>
+          <t>Detalles bar Arcadia</t>
         </is>
       </c>
       <c r="F297" s="41" t="inlineStr">
         <is>
-          <t>contactenos@ghlhoteles.com</t>
+          <t>Capacidad máx. 25 pax; se sirve comida; sin happy hour listado por separado</t>
         </is>
       </c>
       <c r="G297" s="41" t="inlineStr">
         <is>
-          <t>laydy.pauca@ghlhoteles.com</t>
+          <t>Se retira capacidad máxima y mención de comida servida; resto de condiciones igual</t>
         </is>
       </c>
       <c r="H297" s="41" t="n"/>
@@ -16614,27 +16614,27 @@
       </c>
       <c r="C298" s="41" t="inlineStr">
         <is>
-          <t>16-25</t>
+          <t>17-02</t>
         </is>
       </c>
       <c r="D298" s="41" t="inlineStr">
         <is>
-          <t>Tips policy</t>
+          <t>Bar reservation</t>
         </is>
       </c>
       <c r="E298" s="41" t="inlineStr">
         <is>
-          <t>Política de propinas</t>
+          <t>Reservas de bar</t>
         </is>
       </c>
       <c r="F298" s="41" t="inlineStr">
         <is>
-          <t>Tarifa estándar incluye 19% de impuesto de servicio; propina habitual y opcional</t>
+          <t>No se toman reservas</t>
         </is>
       </c>
       <c r="G298" s="41" t="inlineStr">
         <is>
-          <t>Tarifa estándar incluye el cargo por servicio; propina opcional</t>
+          <t>Para reservar, contactar al +51 945739921</t>
         </is>
       </c>
       <c r="H298" s="41" t="n"/>
@@ -16652,27 +16652,27 @@
       </c>
       <c r="C299" s="41" t="inlineStr">
         <is>
-          <t>17-01</t>
+          <t>17-10</t>
         </is>
       </c>
       <c r="D299" s="41" t="inlineStr">
         <is>
-          <t>Bar</t>
+          <t>Spa</t>
         </is>
       </c>
       <c r="E299" s="41" t="inlineStr">
         <is>
-          <t>Detalles bar Arcadia</t>
+          <t>Tarifas y kit obligatorio</t>
         </is>
       </c>
       <c r="F299" s="41" t="inlineStr">
         <is>
-          <t>Capacidad máx. 25 pax; se sirve comida; sin happy hour listado por separado</t>
+          <t>Precio de huésped variable; obligatorio: pantuflas y vestido de baño; no obligatorio: bata y gorro</t>
         </is>
       </c>
       <c r="G299" s="41" t="inlineStr">
         <is>
-          <t>Se retira capacidad máxima y mención de comida servida; resto de condiciones igual</t>
+          <t>Masajes con cargo adicional; obligatorio: pantuflas, gorro y vestido de baño; no obligatorio: bata</t>
         </is>
       </c>
       <c r="H299" s="41" t="n"/>
@@ -16690,27 +16690,27 @@
       </c>
       <c r="C300" s="41" t="inlineStr">
         <is>
-          <t>17-02</t>
+          <t>17-15</t>
         </is>
       </c>
       <c r="D300" s="41" t="inlineStr">
         <is>
-          <t>Bar reservation</t>
+          <t>Spa hours</t>
         </is>
       </c>
       <c r="E300" s="41" t="inlineStr">
         <is>
-          <t>Reservas de bar</t>
+          <t>Límite de tiempo</t>
         </is>
       </c>
       <c r="F300" s="41" t="inlineStr">
         <is>
-          <t>No se toman reservas</t>
+          <t>Sin límite de tiempo</t>
         </is>
       </c>
       <c r="G300" s="41" t="inlineStr">
         <is>
-          <t>Para reservar, contactar al +51 945739921</t>
+          <t>Estancia máxima de 1 hora</t>
         </is>
       </c>
       <c r="H300" s="41" t="n"/>
@@ -16728,27 +16728,27 @@
       </c>
       <c r="C301" s="41" t="inlineStr">
         <is>
-          <t>17-10</t>
+          <t>18-01</t>
         </is>
       </c>
       <c r="D301" s="41" t="inlineStr">
         <is>
-          <t>Spa</t>
+          <t>Restaurant</t>
         </is>
       </c>
       <c r="E301" s="41" t="inlineStr">
         <is>
-          <t>Tarifas y kit obligatorio</t>
+          <t>Descripción restaurante Micaela</t>
         </is>
       </c>
       <c r="F301" s="41" t="inlineStr">
         <is>
-          <t>Precio de huésped variable; obligatorio: pantuflas y vestido de baño; no obligatorio: bata y gorro</t>
+          <t>Descripción extensa (tipo de cocina, capacidad, niños, reservas, cajas altas, etc.)</t>
         </is>
       </c>
       <c r="G301" s="41" t="inlineStr">
         <is>
-          <t>Masajes con cargo adicional; obligatorio: pantuflas, gorro y vestido de baño; no obligatorio: bata</t>
+          <t>Descripción simplificada: horario, accesibilidad, mascotas no aceptadas</t>
         </is>
       </c>
       <c r="H301" s="41" t="n"/>
@@ -16766,27 +16766,27 @@
       </c>
       <c r="C302" s="41" t="inlineStr">
         <is>
-          <t>17-15</t>
+          <t>18-02</t>
         </is>
       </c>
       <c r="D302" s="41" t="inlineStr">
         <is>
-          <t>Spa hours</t>
+          <t>Restaurant reservation</t>
         </is>
       </c>
       <c r="E302" s="41" t="inlineStr">
         <is>
-          <t>Límite de tiempo</t>
+          <t>Método de reserva</t>
         </is>
       </c>
       <c r="F302" s="41" t="inlineStr">
         <is>
-          <t>Sin límite de tiempo</t>
+          <t>Reservar por correo a reservas.sonestaarequipa@ghlhoteles.com</t>
         </is>
       </c>
       <c r="G302" s="41" t="inlineStr">
         <is>
-          <t>Estancia máxima de 1 hora</t>
+          <t>Contactar al +51 945739921</t>
         </is>
       </c>
       <c r="H302" s="41" t="n"/>
@@ -16804,27 +16804,27 @@
       </c>
       <c r="C303" s="41" t="inlineStr">
         <is>
-          <t>18-01</t>
+          <t>18-03</t>
         </is>
       </c>
       <c r="D303" s="41" t="inlineStr">
         <is>
-          <t>Restaurant</t>
+          <t>Restaurant reservation cancellation</t>
         </is>
       </c>
       <c r="E303" s="41" t="inlineStr">
         <is>
-          <t>Descripción restaurante Micaela</t>
+          <t>Método de cancelación</t>
         </is>
       </c>
       <c r="F303" s="41" t="inlineStr">
         <is>
-          <t>Descripción extensa (tipo de cocina, capacidad, niños, reservas, cajas altas, etc.)</t>
+          <t>Cancelar por correo</t>
         </is>
       </c>
       <c r="G303" s="41" t="inlineStr">
         <is>
-          <t>Descripción simplificada: horario, accesibilidad, mascotas no aceptadas</t>
+          <t>Contactar al +51 945739921</t>
         </is>
       </c>
       <c r="H303" s="41" t="n"/>
@@ -16842,22 +16842,22 @@
       </c>
       <c r="C304" s="41" t="inlineStr">
         <is>
-          <t>18-02</t>
+          <t>18-04</t>
         </is>
       </c>
       <c r="D304" s="41" t="inlineStr">
         <is>
-          <t>Restaurant reservation</t>
+          <t>Restaurant reservation modification</t>
         </is>
       </c>
       <c r="E304" s="41" t="inlineStr">
         <is>
-          <t>Método de reserva</t>
+          <t>Método de modificación</t>
         </is>
       </c>
       <c r="F304" s="41" t="inlineStr">
         <is>
-          <t>Reservar por correo a reservas.sonestaarequipa@ghlhoteles.com</t>
+          <t>Modificar por correo</t>
         </is>
       </c>
       <c r="G304" s="41" t="inlineStr">
@@ -16880,22 +16880,22 @@
       </c>
       <c r="C305" s="41" t="inlineStr">
         <is>
-          <t>18-03</t>
+          <t>18-05</t>
         </is>
       </c>
       <c r="D305" s="41" t="inlineStr">
         <is>
-          <t>Restaurant reservation cancellation</t>
+          <t>Restaurant reservation confirmation</t>
         </is>
       </c>
       <c r="E305" s="41" t="inlineStr">
         <is>
-          <t>Método de cancelación</t>
+          <t>Método de confirmación</t>
         </is>
       </c>
       <c r="F305" s="41" t="inlineStr">
         <is>
-          <t>Cancelar por correo</t>
+          <t>Confirmar por correo</t>
         </is>
       </c>
       <c r="G305" s="41" t="inlineStr">
@@ -16918,27 +16918,27 @@
       </c>
       <c r="C306" s="41" t="inlineStr">
         <is>
-          <t>18-04</t>
+          <t>18-11</t>
         </is>
       </c>
       <c r="D306" s="41" t="inlineStr">
         <is>
-          <t>Restaurant reservation modification</t>
+          <t>Brunch</t>
         </is>
       </c>
       <c r="E306" s="41" t="inlineStr">
         <is>
-          <t>Método de modificación</t>
+          <t>Recomendación externa</t>
         </is>
       </c>
       <c r="F306" s="41" t="inlineStr">
         <is>
-          <t>Modificar por correo</t>
+          <t>No ofrecen brunch; recomiendan Restaurante Santé como alternativa externa</t>
         </is>
       </c>
       <c r="G306" s="41" t="inlineStr">
         <is>
-          <t>Contactar al +51 945739921</t>
+          <t>No ofrecemos brunch (se retira la recomendación externa)</t>
         </is>
       </c>
       <c r="H306" s="41" t="n"/>
@@ -16956,27 +16956,27 @@
       </c>
       <c r="C307" s="41" t="inlineStr">
         <is>
-          <t>18-05</t>
+          <t>18-26</t>
         </is>
       </c>
       <c r="D307" s="41" t="inlineStr">
         <is>
-          <t>Restaurant reservation confirmation</t>
+          <t>Valentine's day</t>
         </is>
       </c>
       <c r="E307" s="41" t="inlineStr">
         <is>
-          <t>Método de confirmación</t>
+          <t>Forma de consulta</t>
         </is>
       </c>
       <c r="F307" s="41" t="inlineStr">
         <is>
-          <t>Confirmar por correo</t>
+          <t>Ver oferta mediante enlace</t>
         </is>
       </c>
       <c r="G307" s="41" t="inlineStr">
         <is>
-          <t>Contactar al +51 945739921</t>
+          <t>Escribir a reservas.sonestaarequipa@ghlhoteles.com o contactar al +51 939753285</t>
         </is>
       </c>
       <c r="H307" s="41" t="n"/>
@@ -16994,27 +16994,27 @@
       </c>
       <c r="C308" s="41" t="inlineStr">
         <is>
-          <t>18-11</t>
+          <t>19-03</t>
         </is>
       </c>
       <c r="D308" s="41" t="inlineStr">
         <is>
-          <t>Brunch</t>
+          <t>City center</t>
         </is>
       </c>
       <c r="E308" s="41" t="inlineStr">
         <is>
-          <t>Recomendación externa</t>
+          <t>Distancia al centro</t>
         </is>
       </c>
       <c r="F308" s="41" t="inlineStr">
         <is>
-          <t>No ofrecen brunch; recomiendan Restaurante Santé como alternativa externa</t>
+          <t>26 m, 1 min caminando</t>
         </is>
       </c>
       <c r="G308" s="41" t="inlineStr">
         <is>
-          <t>No ofrecemos brunch (se retira la recomendación externa)</t>
+          <t>4 km</t>
         </is>
       </c>
       <c r="H308" s="41" t="n"/>
@@ -17032,410 +17032,30 @@
       </c>
       <c r="C309" s="41" t="inlineStr">
         <is>
-          <t>18-26</t>
+          <t>20-21</t>
         </is>
       </c>
       <c r="D309" s="41" t="inlineStr">
         <is>
-          <t>Valentine's day</t>
+          <t>Celebration</t>
         </is>
       </c>
       <c r="E309" s="41" t="inlineStr">
         <is>
-          <t>Forma de consulta</t>
+          <t>Teléfono de eventos</t>
         </is>
       </c>
       <c r="F309" s="41" t="inlineStr">
         <is>
-          <t>Ver oferta mediante enlace</t>
+          <t>+51 945 739 48</t>
         </is>
       </c>
       <c r="G309" s="41" t="inlineStr">
         <is>
-          <t>Escribir a reservas.sonestaarequipa@ghlhoteles.com o contactar al +51 939753285</t>
+          <t>+51 945 739 484 (corrección de dígito faltante)</t>
         </is>
       </c>
       <c r="H309" s="41" t="n"/>
-    </row>
-    <row r="310">
-      <c r="A310" s="40" t="inlineStr">
-        <is>
-          <t>Jul-26</t>
-        </is>
-      </c>
-      <c r="B310" s="41" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C310" s="41" t="inlineStr">
-        <is>
-          <t>19-03</t>
-        </is>
-      </c>
-      <c r="D310" s="41" t="inlineStr">
-        <is>
-          <t>City center</t>
-        </is>
-      </c>
-      <c r="E310" s="41" t="inlineStr">
-        <is>
-          <t>Distancia al centro</t>
-        </is>
-      </c>
-      <c r="F310" s="41" t="inlineStr">
-        <is>
-          <t>26 m, 1 min caminando</t>
-        </is>
-      </c>
-      <c r="G310" s="41" t="inlineStr">
-        <is>
-          <t>4 km</t>
-        </is>
-      </c>
-      <c r="H310" s="41" t="n"/>
-    </row>
-    <row r="311">
-      <c r="A311" s="40" t="inlineStr">
-        <is>
-          <t>Jul-26</t>
-        </is>
-      </c>
-      <c r="B311" s="41" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C311" s="41" t="inlineStr">
-        <is>
-          <t>20-21</t>
-        </is>
-      </c>
-      <c r="D311" s="41" t="inlineStr">
-        <is>
-          <t>Celebration</t>
-        </is>
-      </c>
-      <c r="E311" s="41" t="inlineStr">
-        <is>
-          <t>Teléfono de eventos</t>
-        </is>
-      </c>
-      <c r="F311" s="41" t="inlineStr">
-        <is>
-          <t>+51 945 739 48</t>
-        </is>
-      </c>
-      <c r="G311" s="41" t="inlineStr">
-        <is>
-          <t>+51 945 739 484 (corrección de dígito faltante)</t>
-        </is>
-      </c>
-      <c r="H311" s="41" t="n"/>
-    </row>
-    <row r="312">
-      <c r="A312" s="40" t="inlineStr">
-        <is>
-          <t>Jul-26</t>
-        </is>
-      </c>
-      <c r="B312" s="41" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C312" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D312" s="41" t="inlineStr">
-        <is>
-          <t>Check in time</t>
-        </is>
-      </c>
-      <c r="E312" s="41" t="inlineStr">
-        <is>
-          <t>Costo early check-in</t>
-        </is>
-      </c>
-      <c r="F312" s="41" t="inlineStr">
-        <is>
-          <t>Versión anterior</t>
-        </is>
-      </c>
-      <c r="G312" s="41" t="inlineStr">
-        <is>
-          <t>$35.000, sujeto a disponibilidad</t>
-        </is>
-      </c>
-      <c r="H312" s="41" t="n"/>
-    </row>
-    <row r="313">
-      <c r="A313" s="40" t="inlineStr">
-        <is>
-          <t>Jul-26</t>
-        </is>
-      </c>
-      <c r="B313" s="41" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C313" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D313" s="41" t="inlineStr">
-        <is>
-          <t>Check out time</t>
-        </is>
-      </c>
-      <c r="E313" s="41" t="inlineStr">
-        <is>
-          <t>Late check-out</t>
-        </is>
-      </c>
-      <c r="F313" s="41" t="inlineStr">
-        <is>
-          <t>Versión anterior</t>
-        </is>
-      </c>
-      <c r="G313" s="41" t="inlineStr">
-        <is>
-          <t>$35.000 por hora; después de las 6:00 p.m. se cobra la tarifa completa</t>
-        </is>
-      </c>
-      <c r="H313" s="41" t="n"/>
-    </row>
-    <row r="314">
-      <c r="A314" s="40" t="inlineStr">
-        <is>
-          <t>Jul-26</t>
-        </is>
-      </c>
-      <c r="B314" s="41" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C314" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D314" s="41" t="inlineStr">
-        <is>
-          <t>Breakfast time</t>
-        </is>
-      </c>
-      <c r="E314" s="41" t="inlineStr">
-        <is>
-          <t>Horario sábados, domingos y festivos</t>
-        </is>
-      </c>
-      <c r="F314" s="41" t="inlineStr">
-        <is>
-          <t>Versión anterior</t>
-        </is>
-      </c>
-      <c r="G314" s="41" t="inlineStr">
-        <is>
-          <t>6:30 a.m. a 10:30 a.m.</t>
-        </is>
-      </c>
-      <c r="H314" s="41" t="n"/>
-    </row>
-    <row r="315">
-      <c r="A315" s="40" t="inlineStr">
-        <is>
-          <t>Jul-26</t>
-        </is>
-      </c>
-      <c r="B315" s="41" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C315" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D315" s="41" t="inlineStr">
-        <is>
-          <t>Breakfast rates</t>
-        </is>
-      </c>
-      <c r="E315" s="41" t="inlineStr">
-        <is>
-          <t>Precio por persona</t>
-        </is>
-      </c>
-      <c r="F315" s="41" t="inlineStr">
-        <is>
-          <t>Versión anterior</t>
-        </is>
-      </c>
-      <c r="G315" s="41" t="inlineStr">
-        <is>
-          <t>$65.000 COP</t>
-        </is>
-      </c>
-      <c r="H315" s="41" t="n"/>
-    </row>
-    <row r="316">
-      <c r="A316" s="40" t="inlineStr">
-        <is>
-          <t>Jul-26</t>
-        </is>
-      </c>
-      <c r="B316" s="41" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C316" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D316" s="41" t="inlineStr">
-        <is>
-          <t>Kids</t>
-        </is>
-      </c>
-      <c r="E316" s="41" t="inlineStr">
-        <is>
-          <t>Tarifa niños</t>
-        </is>
-      </c>
-      <c r="F316" s="41" t="inlineStr">
-        <is>
-          <t>Versión anterior</t>
-        </is>
-      </c>
-      <c r="G316" s="41" t="inlineStr">
-        <is>
-          <t>Menores de 12 años gratis con sus padres; mayores de 12 años $80.000 por noche</t>
-        </is>
-      </c>
-      <c r="H316" s="41" t="n"/>
-    </row>
-    <row r="317">
-      <c r="A317" s="40" t="inlineStr">
-        <is>
-          <t>Jul-26</t>
-        </is>
-      </c>
-      <c r="B317" s="41" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C317" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D317" s="41" t="inlineStr">
-        <is>
-          <t>Pets</t>
-        </is>
-      </c>
-      <c r="E317" s="41" t="inlineStr">
-        <is>
-          <t>Peso permitido</t>
-        </is>
-      </c>
-      <c r="F317" s="41" t="inlineStr">
-        <is>
-          <t>Versión anterior</t>
-        </is>
-      </c>
-      <c r="G317" s="41" t="inlineStr">
-        <is>
-          <t>10 kg</t>
-        </is>
-      </c>
-      <c r="H317" s="41" t="n"/>
-    </row>
-    <row r="318">
-      <c r="A318" s="40" t="inlineStr">
-        <is>
-          <t>Jul-26</t>
-        </is>
-      </c>
-      <c r="B318" s="41" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C318" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D318" s="41" t="inlineStr">
-        <is>
-          <t>Social &amp; photoshoot</t>
-        </is>
-      </c>
-      <c r="E318" s="41" t="inlineStr">
-        <is>
-          <t>Correo de contacto</t>
-        </is>
-      </c>
-      <c r="F318" s="41" t="inlineStr">
-        <is>
-          <t>Versión anterior</t>
-        </is>
-      </c>
-      <c r="G318" s="41" t="inlineStr">
-        <is>
-          <t>cateryne.palacios@ghlhoteles.com</t>
-        </is>
-      </c>
-      <c r="H318" s="41" t="n"/>
-    </row>
-    <row r="319">
-      <c r="A319" s="40" t="inlineStr">
-        <is>
-          <t>Jul-26</t>
-        </is>
-      </c>
-      <c r="B319" s="41" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C319" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D319" s="41" t="inlineStr">
-        <is>
-          <t>Restaurant Cook's Restaurante</t>
-        </is>
-      </c>
-      <c r="E319" s="41" t="inlineStr">
-        <is>
-          <t>Horario de apertura</t>
-        </is>
-      </c>
-      <c r="F319" s="41" t="inlineStr">
-        <is>
-          <t>Versión anterior</t>
-        </is>
-      </c>
-      <c r="G319" s="41" t="inlineStr">
-        <is>
-          <t>6:00 a.m. a 12:00 p.m.</t>
-        </is>
-      </c>
-      <c r="H319" s="41" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H227"/>
@@ -17767,8 +17387,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Revert "Corrige registros de Sonesta Bogotá y GHL Style Neiva usando PDFs de julio"
This reverts commit da65c6778d8ce4d8eadfe9fa6701bae533ec19b8.
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -3935,7 +3935,7 @@
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>3 diálogos modificados: ubicación, check-in/out tardío</t>
+          <t>5 diálogos modificados: ubicación, check-in/out tardío, horario y tarifa de desayuno</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -3943,11 +3943,7 @@
           <t>30/07/2026</t>
         </is>
       </c>
-      <c r="J65" s="8" t="inlineStr">
-        <is>
-          <t>Se retiran horario y tarifa de desayuno del listado: coinciden con el PDF de julio vigente, no eran cambios reales</t>
-        </is>
-      </c>
+      <c r="J65" s="8" t="n"/>
       <c r="K65" s="42" t="inlineStr">
         <is>
           <t>Actualizado</t>
@@ -4636,19 +4632,23 @@
       </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H80" s="5" t="n"/>
-      <c r="I80" s="6" t="n"/>
-      <c r="J80" s="5" t="inlineStr">
-        <is>
-          <t>Los 8 puntos que reportó ya coinciden con el PDF de julio vigente — no eran cambios reales, solo confirmó valores ya correctos</t>
-        </is>
-      </c>
-      <c r="K80" s="38" t="inlineStr">
-        <is>
-          <t>Sin modificaciones</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>8 diálogos modificados: check-in/out, desayuno horario/precio, niños, mascotas, redes, restaurante</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="n"/>
+      <c r="K80" s="42" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
       <c r="L80" s="5" t="inlineStr"/>
@@ -5096,13 +5096,13 @@
         <v>26</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
@@ -5235,10 +5235,10 @@
         <v>26</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G4" s="20" t="n">
         <v>0.3809523809523809</v>
@@ -5305,10 +5305,10 @@
         <v>45</v>
       </c>
       <c r="E6" s="28" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F6" s="28" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G6" s="29" t="n">
         <v>0.4642857142857143</v>
@@ -5344,7 +5344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H309"/>
+  <dimension ref="A1:H319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16082,7 +16082,7 @@
       </c>
       <c r="C284" s="41" t="inlineStr">
         <is>
-          <t>19-01</t>
+          <t>9-01</t>
         </is>
       </c>
       <c r="D284" s="41" t="inlineStr">
@@ -16097,7 +16097,7 @@
       </c>
       <c r="F284" s="41" t="inlineStr">
         <is>
-          <t>Cra. 8a #38-42, Comuna 2, Neiva, Huila, Colombia</t>
+          <t>⚠ No especificada en el diálogo previo</t>
         </is>
       </c>
       <c r="G284" s="41" t="inlineStr">
@@ -16191,32 +16191,32 @@
       </c>
       <c r="B287" s="41" t="inlineStr">
         <is>
-          <t>GHL Style Yopal</t>
+          <t>GHL Style Neiva</t>
         </is>
       </c>
       <c r="C287" s="41" t="inlineStr">
         <is>
-          <t>11-01</t>
+          <t>12-01</t>
         </is>
       </c>
       <c r="D287" s="41" t="inlineStr">
         <is>
-          <t>Check in time</t>
+          <t>Breakfast time</t>
         </is>
       </c>
       <c r="E287" s="41" t="inlineStr">
         <is>
-          <t>Costo early check-in</t>
+          <t>Horario desayuno</t>
         </is>
       </c>
       <c r="F287" s="41" t="inlineStr">
         <is>
-          <t>70.000 COP por habitación</t>
+          <t>⚠ No especificado</t>
         </is>
       </c>
       <c r="G287" s="41" t="inlineStr">
         <is>
-          <t>COP 70.000 + impuestos por habitación</t>
+          <t>Buffet diario de 6:30 a.m. a 10:00 a.m.</t>
         </is>
       </c>
       <c r="H287" s="41" t="n"/>
@@ -16229,32 +16229,32 @@
       </c>
       <c r="B288" s="41" t="inlineStr">
         <is>
-          <t>GHL Style Yopal</t>
+          <t>GHL Style Neiva</t>
         </is>
       </c>
       <c r="C288" s="41" t="inlineStr">
         <is>
-          <t>11-11</t>
+          <t>12-02</t>
         </is>
       </c>
       <c r="D288" s="41" t="inlineStr">
         <is>
-          <t>Check out time</t>
+          <t>Breakfast rates</t>
         </is>
       </c>
       <c r="E288" s="41" t="inlineStr">
         <is>
-          <t>Costo late check-out</t>
+          <t>Precio adulto</t>
         </is>
       </c>
       <c r="F288" s="41" t="inlineStr">
         <is>
-          <t>70.000 COP por habitación</t>
+          <t>⚠ No especificado</t>
         </is>
       </c>
       <c r="G288" s="41" t="inlineStr">
         <is>
-          <t>COP 70.000 + impuestos por habitación</t>
+          <t>40.000 COP por adulto; incluido en tarifa de habitación; visitantes también bienvenidos</t>
         </is>
       </c>
       <c r="H288" s="41" t="n"/>
@@ -16267,32 +16267,32 @@
       </c>
       <c r="B289" s="41" t="inlineStr">
         <is>
-          <t>Hotel Tequendama Bogotá</t>
+          <t>GHL Style Yopal</t>
         </is>
       </c>
       <c r="C289" s="41" t="inlineStr">
         <is>
-          <t>13-45</t>
+          <t>11-01</t>
         </is>
       </c>
       <c r="D289" s="41" t="inlineStr">
         <is>
-          <t>Change &amp; ATM</t>
+          <t>Check in time</t>
         </is>
       </c>
       <c r="E289" s="41" t="inlineStr">
         <is>
-          <t>Disponibilidad de cajero automático</t>
+          <t>Costo early check-in</t>
         </is>
       </c>
       <c r="F289" s="41" t="inlineStr">
         <is>
-          <t>Sí tenemos un cajero automático en la propiedad</t>
+          <t>70.000 COP por habitación</t>
         </is>
       </c>
       <c r="G289" s="41" t="inlineStr">
         <is>
-          <t>No tenemos un cajero automático en la propiedad</t>
+          <t>COP 70.000 + impuestos por habitación</t>
         </is>
       </c>
       <c r="H289" s="41" t="n"/>
@@ -16305,32 +16305,32 @@
       </c>
       <c r="B290" s="41" t="inlineStr">
         <is>
-          <t>Hotel Tequendama Bogotá</t>
+          <t>GHL Style Yopal</t>
         </is>
       </c>
       <c r="C290" s="41" t="inlineStr">
         <is>
-          <t>13-06</t>
+          <t>11-11</t>
         </is>
       </c>
       <c r="D290" s="41" t="inlineStr">
         <is>
-          <t>Room Service</t>
+          <t>Check out time</t>
         </is>
       </c>
       <c r="E290" s="41" t="inlineStr">
         <is>
-          <t>Horario y marcación</t>
+          <t>Costo late check-out</t>
         </is>
       </c>
       <c r="F290" s="41" t="inlineStr">
         <is>
-          <t>Disponible de 06:00 a 22:00; marcar 2356</t>
+          <t>70.000 COP por habitación</t>
         </is>
       </c>
       <c r="G290" s="41" t="inlineStr">
         <is>
-          <t>Disponible de 06:00 a 00:00; marcar *2</t>
+          <t>COP 70.000 + impuestos por habitación</t>
         </is>
       </c>
       <c r="H290" s="41" t="n"/>
@@ -16343,32 +16343,32 @@
       </c>
       <c r="B291" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Cusco</t>
+          <t>Hotel Tequendama Bogotá</t>
         </is>
       </c>
       <c r="C291" s="41" t="inlineStr">
         <is>
-          <t>16-02</t>
+          <t>13-45</t>
         </is>
       </c>
       <c r="D291" s="41" t="inlineStr">
         <is>
-          <t>Contact staff — Recepción</t>
+          <t>Change &amp; ATM</t>
         </is>
       </c>
       <c r="E291" s="41" t="inlineStr">
         <is>
-          <t>Correo</t>
+          <t>Disponibilidad de cajero automático</t>
         </is>
       </c>
       <c r="F291" s="41" t="inlineStr">
         <is>
-          <t>recepcion.sonestahotelcusco@ghlhoteles.com</t>
+          <t>Sí tenemos un cajero automático en la propiedad</t>
         </is>
       </c>
       <c r="G291" s="41" t="inlineStr">
         <is>
-          <t>recepcion.sonestacusco@ghlhoteles.com</t>
+          <t>No tenemos un cajero automático en la propiedad</t>
         </is>
       </c>
       <c r="H291" s="41" t="n"/>
@@ -16381,32 +16381,32 @@
       </c>
       <c r="B292" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Cusco</t>
+          <t>Hotel Tequendama Bogotá</t>
         </is>
       </c>
       <c r="C292" s="41" t="inlineStr">
         <is>
-          <t>11-01</t>
+          <t>13-06</t>
         </is>
       </c>
       <c r="D292" s="41" t="inlineStr">
         <is>
-          <t>Check-in time</t>
+          <t>Room Service</t>
         </is>
       </c>
       <c r="E292" s="41" t="inlineStr">
         <is>
-          <t>Costo early check-in</t>
+          <t>Horario y marcación</t>
         </is>
       </c>
       <c r="F292" s="41" t="inlineStr">
         <is>
-          <t>40.00 USD por habitación</t>
+          <t>Disponible de 06:00 a 22:00; marcar 2356</t>
         </is>
       </c>
       <c r="G292" s="41" t="inlineStr">
         <is>
-          <t>60.00 USD por habitación (impuestos no incluidos)</t>
+          <t>Disponible de 06:00 a 00:00; marcar *2</t>
         </is>
       </c>
       <c r="H292" s="41" t="n"/>
@@ -16424,27 +16424,27 @@
       </c>
       <c r="C293" s="41" t="inlineStr">
         <is>
-          <t>11-11</t>
+          <t>16-02</t>
         </is>
       </c>
       <c r="D293" s="41" t="inlineStr">
         <is>
-          <t>Check-out time</t>
+          <t>Contact staff — Recepción</t>
         </is>
       </c>
       <c r="E293" s="41" t="inlineStr">
         <is>
-          <t>Costo late check-out</t>
+          <t>Correo</t>
         </is>
       </c>
       <c r="F293" s="41" t="inlineStr">
         <is>
-          <t>40.00 USD por habitación</t>
+          <t>recepcion.sonestahotelcusco@ghlhoteles.com</t>
         </is>
       </c>
       <c r="G293" s="41" t="inlineStr">
         <is>
-          <t>60.00 USD por habitación</t>
+          <t>recepcion.sonestacusco@ghlhoteles.com</t>
         </is>
       </c>
       <c r="H293" s="41" t="n"/>
@@ -16462,27 +16462,27 @@
       </c>
       <c r="C294" s="41" t="inlineStr">
         <is>
-          <t>13-06</t>
+          <t>11-01</t>
         </is>
       </c>
       <c r="D294" s="41" t="inlineStr">
         <is>
-          <t>Room service</t>
+          <t>Check-in time</t>
         </is>
       </c>
       <c r="E294" s="41" t="inlineStr">
         <is>
-          <t>Horario</t>
+          <t>Costo early check-in</t>
         </is>
       </c>
       <c r="F294" s="41" t="inlineStr">
         <is>
-          <t>Disponible de 06:00 a 21:00</t>
+          <t>40.00 USD por habitación</t>
         </is>
       </c>
       <c r="G294" s="41" t="inlineStr">
         <is>
-          <t>Disponible 24/7</t>
+          <t>60.00 USD por habitación (impuestos no incluidos)</t>
         </is>
       </c>
       <c r="H294" s="41" t="n"/>
@@ -16495,32 +16495,32 @@
       </c>
       <c r="B295" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Arequipa</t>
+          <t>Sonesta Cusco</t>
         </is>
       </c>
       <c r="C295" s="41" t="inlineStr">
         <is>
-          <t>16-06</t>
+          <t>11-11</t>
         </is>
       </c>
       <c r="D295" s="41" t="inlineStr">
         <is>
-          <t>Jobs &amp; internships</t>
+          <t>Check-out time</t>
         </is>
       </c>
       <c r="E295" s="41" t="inlineStr">
         <is>
-          <t>Correo de contacto RR.HH.</t>
+          <t>Costo late check-out</t>
         </is>
       </c>
       <c r="F295" s="41" t="inlineStr">
         <is>
-          <t>contactenos@ghlhoteles.com</t>
+          <t>40.00 USD por habitación</t>
         </is>
       </c>
       <c r="G295" s="41" t="inlineStr">
         <is>
-          <t>laydy.pauca@ghlhoteles.com</t>
+          <t>60.00 USD por habitación</t>
         </is>
       </c>
       <c r="H295" s="41" t="n"/>
@@ -16533,32 +16533,32 @@
       </c>
       <c r="B296" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Arequipa</t>
+          <t>Sonesta Cusco</t>
         </is>
       </c>
       <c r="C296" s="41" t="inlineStr">
         <is>
-          <t>16-25</t>
+          <t>13-06</t>
         </is>
       </c>
       <c r="D296" s="41" t="inlineStr">
         <is>
-          <t>Tips policy</t>
+          <t>Room service</t>
         </is>
       </c>
       <c r="E296" s="41" t="inlineStr">
         <is>
-          <t>Política de propinas</t>
+          <t>Horario</t>
         </is>
       </c>
       <c r="F296" s="41" t="inlineStr">
         <is>
-          <t>Tarifa estándar incluye 19% de impuesto de servicio; propina habitual y opcional</t>
+          <t>Disponible de 06:00 a 21:00</t>
         </is>
       </c>
       <c r="G296" s="41" t="inlineStr">
         <is>
-          <t>Tarifa estándar incluye el cargo por servicio; propina opcional</t>
+          <t>Disponible 24/7</t>
         </is>
       </c>
       <c r="H296" s="41" t="n"/>
@@ -16576,27 +16576,27 @@
       </c>
       <c r="C297" s="41" t="inlineStr">
         <is>
-          <t>17-01</t>
+          <t>16-06</t>
         </is>
       </c>
       <c r="D297" s="41" t="inlineStr">
         <is>
-          <t>Bar</t>
+          <t>Jobs &amp; internships</t>
         </is>
       </c>
       <c r="E297" s="41" t="inlineStr">
         <is>
-          <t>Detalles bar Arcadia</t>
+          <t>Correo de contacto RR.HH.</t>
         </is>
       </c>
       <c r="F297" s="41" t="inlineStr">
         <is>
-          <t>Capacidad máx. 25 pax; se sirve comida; sin happy hour listado por separado</t>
+          <t>contactenos@ghlhoteles.com</t>
         </is>
       </c>
       <c r="G297" s="41" t="inlineStr">
         <is>
-          <t>Se retira capacidad máxima y mención de comida servida; resto de condiciones igual</t>
+          <t>laydy.pauca@ghlhoteles.com</t>
         </is>
       </c>
       <c r="H297" s="41" t="n"/>
@@ -16614,27 +16614,27 @@
       </c>
       <c r="C298" s="41" t="inlineStr">
         <is>
-          <t>17-02</t>
+          <t>16-25</t>
         </is>
       </c>
       <c r="D298" s="41" t="inlineStr">
         <is>
-          <t>Bar reservation</t>
+          <t>Tips policy</t>
         </is>
       </c>
       <c r="E298" s="41" t="inlineStr">
         <is>
-          <t>Reservas de bar</t>
+          <t>Política de propinas</t>
         </is>
       </c>
       <c r="F298" s="41" t="inlineStr">
         <is>
-          <t>No se toman reservas</t>
+          <t>Tarifa estándar incluye 19% de impuesto de servicio; propina habitual y opcional</t>
         </is>
       </c>
       <c r="G298" s="41" t="inlineStr">
         <is>
-          <t>Para reservar, contactar al +51 945739921</t>
+          <t>Tarifa estándar incluye el cargo por servicio; propina opcional</t>
         </is>
       </c>
       <c r="H298" s="41" t="n"/>
@@ -16652,27 +16652,27 @@
       </c>
       <c r="C299" s="41" t="inlineStr">
         <is>
-          <t>17-10</t>
+          <t>17-01</t>
         </is>
       </c>
       <c r="D299" s="41" t="inlineStr">
         <is>
-          <t>Spa</t>
+          <t>Bar</t>
         </is>
       </c>
       <c r="E299" s="41" t="inlineStr">
         <is>
-          <t>Tarifas y kit obligatorio</t>
+          <t>Detalles bar Arcadia</t>
         </is>
       </c>
       <c r="F299" s="41" t="inlineStr">
         <is>
-          <t>Precio de huésped variable; obligatorio: pantuflas y vestido de baño; no obligatorio: bata y gorro</t>
+          <t>Capacidad máx. 25 pax; se sirve comida; sin happy hour listado por separado</t>
         </is>
       </c>
       <c r="G299" s="41" t="inlineStr">
         <is>
-          <t>Masajes con cargo adicional; obligatorio: pantuflas, gorro y vestido de baño; no obligatorio: bata</t>
+          <t>Se retira capacidad máxima y mención de comida servida; resto de condiciones igual</t>
         </is>
       </c>
       <c r="H299" s="41" t="n"/>
@@ -16690,27 +16690,27 @@
       </c>
       <c r="C300" s="41" t="inlineStr">
         <is>
-          <t>17-15</t>
+          <t>17-02</t>
         </is>
       </c>
       <c r="D300" s="41" t="inlineStr">
         <is>
-          <t>Spa hours</t>
+          <t>Bar reservation</t>
         </is>
       </c>
       <c r="E300" s="41" t="inlineStr">
         <is>
-          <t>Límite de tiempo</t>
+          <t>Reservas de bar</t>
         </is>
       </c>
       <c r="F300" s="41" t="inlineStr">
         <is>
-          <t>Sin límite de tiempo</t>
+          <t>No se toman reservas</t>
         </is>
       </c>
       <c r="G300" s="41" t="inlineStr">
         <is>
-          <t>Estancia máxima de 1 hora</t>
+          <t>Para reservar, contactar al +51 945739921</t>
         </is>
       </c>
       <c r="H300" s="41" t="n"/>
@@ -16728,27 +16728,27 @@
       </c>
       <c r="C301" s="41" t="inlineStr">
         <is>
-          <t>18-01</t>
+          <t>17-10</t>
         </is>
       </c>
       <c r="D301" s="41" t="inlineStr">
         <is>
-          <t>Restaurant</t>
+          <t>Spa</t>
         </is>
       </c>
       <c r="E301" s="41" t="inlineStr">
         <is>
-          <t>Descripción restaurante Micaela</t>
+          <t>Tarifas y kit obligatorio</t>
         </is>
       </c>
       <c r="F301" s="41" t="inlineStr">
         <is>
-          <t>Descripción extensa (tipo de cocina, capacidad, niños, reservas, cajas altas, etc.)</t>
+          <t>Precio de huésped variable; obligatorio: pantuflas y vestido de baño; no obligatorio: bata y gorro</t>
         </is>
       </c>
       <c r="G301" s="41" t="inlineStr">
         <is>
-          <t>Descripción simplificada: horario, accesibilidad, mascotas no aceptadas</t>
+          <t>Masajes con cargo adicional; obligatorio: pantuflas, gorro y vestido de baño; no obligatorio: bata</t>
         </is>
       </c>
       <c r="H301" s="41" t="n"/>
@@ -16766,27 +16766,27 @@
       </c>
       <c r="C302" s="41" t="inlineStr">
         <is>
-          <t>18-02</t>
+          <t>17-15</t>
         </is>
       </c>
       <c r="D302" s="41" t="inlineStr">
         <is>
-          <t>Restaurant reservation</t>
+          <t>Spa hours</t>
         </is>
       </c>
       <c r="E302" s="41" t="inlineStr">
         <is>
-          <t>Método de reserva</t>
+          <t>Límite de tiempo</t>
         </is>
       </c>
       <c r="F302" s="41" t="inlineStr">
         <is>
-          <t>Reservar por correo a reservas.sonestaarequipa@ghlhoteles.com</t>
+          <t>Sin límite de tiempo</t>
         </is>
       </c>
       <c r="G302" s="41" t="inlineStr">
         <is>
-          <t>Contactar al +51 945739921</t>
+          <t>Estancia máxima de 1 hora</t>
         </is>
       </c>
       <c r="H302" s="41" t="n"/>
@@ -16804,27 +16804,27 @@
       </c>
       <c r="C303" s="41" t="inlineStr">
         <is>
-          <t>18-03</t>
+          <t>18-01</t>
         </is>
       </c>
       <c r="D303" s="41" t="inlineStr">
         <is>
-          <t>Restaurant reservation cancellation</t>
+          <t>Restaurant</t>
         </is>
       </c>
       <c r="E303" s="41" t="inlineStr">
         <is>
-          <t>Método de cancelación</t>
+          <t>Descripción restaurante Micaela</t>
         </is>
       </c>
       <c r="F303" s="41" t="inlineStr">
         <is>
-          <t>Cancelar por correo</t>
+          <t>Descripción extensa (tipo de cocina, capacidad, niños, reservas, cajas altas, etc.)</t>
         </is>
       </c>
       <c r="G303" s="41" t="inlineStr">
         <is>
-          <t>Contactar al +51 945739921</t>
+          <t>Descripción simplificada: horario, accesibilidad, mascotas no aceptadas</t>
         </is>
       </c>
       <c r="H303" s="41" t="n"/>
@@ -16842,22 +16842,22 @@
       </c>
       <c r="C304" s="41" t="inlineStr">
         <is>
-          <t>18-04</t>
+          <t>18-02</t>
         </is>
       </c>
       <c r="D304" s="41" t="inlineStr">
         <is>
-          <t>Restaurant reservation modification</t>
+          <t>Restaurant reservation</t>
         </is>
       </c>
       <c r="E304" s="41" t="inlineStr">
         <is>
-          <t>Método de modificación</t>
+          <t>Método de reserva</t>
         </is>
       </c>
       <c r="F304" s="41" t="inlineStr">
         <is>
-          <t>Modificar por correo</t>
+          <t>Reservar por correo a reservas.sonestaarequipa@ghlhoteles.com</t>
         </is>
       </c>
       <c r="G304" s="41" t="inlineStr">
@@ -16880,22 +16880,22 @@
       </c>
       <c r="C305" s="41" t="inlineStr">
         <is>
-          <t>18-05</t>
+          <t>18-03</t>
         </is>
       </c>
       <c r="D305" s="41" t="inlineStr">
         <is>
-          <t>Restaurant reservation confirmation</t>
+          <t>Restaurant reservation cancellation</t>
         </is>
       </c>
       <c r="E305" s="41" t="inlineStr">
         <is>
-          <t>Método de confirmación</t>
+          <t>Método de cancelación</t>
         </is>
       </c>
       <c r="F305" s="41" t="inlineStr">
         <is>
-          <t>Confirmar por correo</t>
+          <t>Cancelar por correo</t>
         </is>
       </c>
       <c r="G305" s="41" t="inlineStr">
@@ -16918,27 +16918,27 @@
       </c>
       <c r="C306" s="41" t="inlineStr">
         <is>
-          <t>18-11</t>
+          <t>18-04</t>
         </is>
       </c>
       <c r="D306" s="41" t="inlineStr">
         <is>
-          <t>Brunch</t>
+          <t>Restaurant reservation modification</t>
         </is>
       </c>
       <c r="E306" s="41" t="inlineStr">
         <is>
-          <t>Recomendación externa</t>
+          <t>Método de modificación</t>
         </is>
       </c>
       <c r="F306" s="41" t="inlineStr">
         <is>
-          <t>No ofrecen brunch; recomiendan Restaurante Santé como alternativa externa</t>
+          <t>Modificar por correo</t>
         </is>
       </c>
       <c r="G306" s="41" t="inlineStr">
         <is>
-          <t>No ofrecemos brunch (se retira la recomendación externa)</t>
+          <t>Contactar al +51 945739921</t>
         </is>
       </c>
       <c r="H306" s="41" t="n"/>
@@ -16956,27 +16956,27 @@
       </c>
       <c r="C307" s="41" t="inlineStr">
         <is>
-          <t>18-26</t>
+          <t>18-05</t>
         </is>
       </c>
       <c r="D307" s="41" t="inlineStr">
         <is>
-          <t>Valentine's day</t>
+          <t>Restaurant reservation confirmation</t>
         </is>
       </c>
       <c r="E307" s="41" t="inlineStr">
         <is>
-          <t>Forma de consulta</t>
+          <t>Método de confirmación</t>
         </is>
       </c>
       <c r="F307" s="41" t="inlineStr">
         <is>
-          <t>Ver oferta mediante enlace</t>
+          <t>Confirmar por correo</t>
         </is>
       </c>
       <c r="G307" s="41" t="inlineStr">
         <is>
-          <t>Escribir a reservas.sonestaarequipa@ghlhoteles.com o contactar al +51 939753285</t>
+          <t>Contactar al +51 945739921</t>
         </is>
       </c>
       <c r="H307" s="41" t="n"/>
@@ -16994,27 +16994,27 @@
       </c>
       <c r="C308" s="41" t="inlineStr">
         <is>
-          <t>19-03</t>
+          <t>18-11</t>
         </is>
       </c>
       <c r="D308" s="41" t="inlineStr">
         <is>
-          <t>City center</t>
+          <t>Brunch</t>
         </is>
       </c>
       <c r="E308" s="41" t="inlineStr">
         <is>
-          <t>Distancia al centro</t>
+          <t>Recomendación externa</t>
         </is>
       </c>
       <c r="F308" s="41" t="inlineStr">
         <is>
-          <t>26 m, 1 min caminando</t>
+          <t>No ofrecen brunch; recomiendan Restaurante Santé como alternativa externa</t>
         </is>
       </c>
       <c r="G308" s="41" t="inlineStr">
         <is>
-          <t>4 km</t>
+          <t>No ofrecemos brunch (se retira la recomendación externa)</t>
         </is>
       </c>
       <c r="H308" s="41" t="n"/>
@@ -17032,30 +17032,410 @@
       </c>
       <c r="C309" s="41" t="inlineStr">
         <is>
+          <t>18-26</t>
+        </is>
+      </c>
+      <c r="D309" s="41" t="inlineStr">
+        <is>
+          <t>Valentine's day</t>
+        </is>
+      </c>
+      <c r="E309" s="41" t="inlineStr">
+        <is>
+          <t>Forma de consulta</t>
+        </is>
+      </c>
+      <c r="F309" s="41" t="inlineStr">
+        <is>
+          <t>Ver oferta mediante enlace</t>
+        </is>
+      </c>
+      <c r="G309" s="41" t="inlineStr">
+        <is>
+          <t>Escribir a reservas.sonestaarequipa@ghlhoteles.com o contactar al +51 939753285</t>
+        </is>
+      </c>
+      <c r="H309" s="41" t="n"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B310" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C310" s="41" t="inlineStr">
+        <is>
+          <t>19-03</t>
+        </is>
+      </c>
+      <c r="D310" s="41" t="inlineStr">
+        <is>
+          <t>City center</t>
+        </is>
+      </c>
+      <c r="E310" s="41" t="inlineStr">
+        <is>
+          <t>Distancia al centro</t>
+        </is>
+      </c>
+      <c r="F310" s="41" t="inlineStr">
+        <is>
+          <t>26 m, 1 min caminando</t>
+        </is>
+      </c>
+      <c r="G310" s="41" t="inlineStr">
+        <is>
+          <t>4 km</t>
+        </is>
+      </c>
+      <c r="H310" s="41" t="n"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B311" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C311" s="41" t="inlineStr">
+        <is>
           <t>20-21</t>
         </is>
       </c>
-      <c r="D309" s="41" t="inlineStr">
+      <c r="D311" s="41" t="inlineStr">
         <is>
           <t>Celebration</t>
         </is>
       </c>
-      <c r="E309" s="41" t="inlineStr">
+      <c r="E311" s="41" t="inlineStr">
         <is>
           <t>Teléfono de eventos</t>
         </is>
       </c>
-      <c r="F309" s="41" t="inlineStr">
+      <c r="F311" s="41" t="inlineStr">
         <is>
           <t>+51 945 739 48</t>
         </is>
       </c>
-      <c r="G309" s="41" t="inlineStr">
+      <c r="G311" s="41" t="inlineStr">
         <is>
           <t>+51 945 739 484 (corrección de dígito faltante)</t>
         </is>
       </c>
-      <c r="H309" s="41" t="n"/>
+      <c r="H311" s="41" t="n"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B312" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C312" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D312" s="41" t="inlineStr">
+        <is>
+          <t>Check in time</t>
+        </is>
+      </c>
+      <c r="E312" s="41" t="inlineStr">
+        <is>
+          <t>Costo early check-in</t>
+        </is>
+      </c>
+      <c r="F312" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G312" s="41" t="inlineStr">
+        <is>
+          <t>$35.000, sujeto a disponibilidad</t>
+        </is>
+      </c>
+      <c r="H312" s="41" t="n"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B313" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C313" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D313" s="41" t="inlineStr">
+        <is>
+          <t>Check out time</t>
+        </is>
+      </c>
+      <c r="E313" s="41" t="inlineStr">
+        <is>
+          <t>Late check-out</t>
+        </is>
+      </c>
+      <c r="F313" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G313" s="41" t="inlineStr">
+        <is>
+          <t>$35.000 por hora; después de las 6:00 p.m. se cobra la tarifa completa</t>
+        </is>
+      </c>
+      <c r="H313" s="41" t="n"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B314" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C314" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D314" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E314" s="41" t="inlineStr">
+        <is>
+          <t>Horario sábados, domingos y festivos</t>
+        </is>
+      </c>
+      <c r="F314" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G314" s="41" t="inlineStr">
+        <is>
+          <t>6:30 a.m. a 10:30 a.m.</t>
+        </is>
+      </c>
+      <c r="H314" s="41" t="n"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B315" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C315" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D315" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E315" s="41" t="inlineStr">
+        <is>
+          <t>Precio por persona</t>
+        </is>
+      </c>
+      <c r="F315" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G315" s="41" t="inlineStr">
+        <is>
+          <t>$65.000 COP</t>
+        </is>
+      </c>
+      <c r="H315" s="41" t="n"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B316" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C316" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D316" s="41" t="inlineStr">
+        <is>
+          <t>Kids</t>
+        </is>
+      </c>
+      <c r="E316" s="41" t="inlineStr">
+        <is>
+          <t>Tarifa niños</t>
+        </is>
+      </c>
+      <c r="F316" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G316" s="41" t="inlineStr">
+        <is>
+          <t>Menores de 12 años gratis con sus padres; mayores de 12 años $80.000 por noche</t>
+        </is>
+      </c>
+      <c r="H316" s="41" t="n"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B317" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C317" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D317" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E317" s="41" t="inlineStr">
+        <is>
+          <t>Peso permitido</t>
+        </is>
+      </c>
+      <c r="F317" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G317" s="41" t="inlineStr">
+        <is>
+          <t>10 kg</t>
+        </is>
+      </c>
+      <c r="H317" s="41" t="n"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B318" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C318" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D318" s="41" t="inlineStr">
+        <is>
+          <t>Social &amp; photoshoot</t>
+        </is>
+      </c>
+      <c r="E318" s="41" t="inlineStr">
+        <is>
+          <t>Correo de contacto</t>
+        </is>
+      </c>
+      <c r="F318" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G318" s="41" t="inlineStr">
+        <is>
+          <t>cateryne.palacios@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="H318" s="41" t="n"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="40" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B319" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C319" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D319" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant Cook's Restaurante</t>
+        </is>
+      </c>
+      <c r="E319" s="41" t="inlineStr">
+        <is>
+          <t>Horario de apertura</t>
+        </is>
+      </c>
+      <c r="F319" s="41" t="inlineStr">
+        <is>
+          <t>Versión anterior</t>
+        </is>
+      </c>
+      <c r="G319" s="41" t="inlineStr">
+        <is>
+          <t>6:00 a.m. a 12:00 p.m.</t>
+        </is>
+      </c>
+      <c r="H319" s="41" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H227"/>
@@ -17387,6 +17767,8 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Abre el ciclo Ago-26 y registra 4 hoteles sin modificaciones
Duplica el bloque de 42 hoteles para el nuevo ciclo Ago-26 (envío
02/08/2026), con color ámbar en HTML y Excel. Registra que GHL Montería,
Sonesta Cusco, GHL Relax Hotel Costa Azul y Armeria Real confirmaron sin
modificaciones para agosto. Actualiza Dashboard cumplimiento y Resumen
por ciclo con la nueva fila de Ago-26 y los totales acumulados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -171,8 +171,23 @@
       <color rgb="00006100"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0092400E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="009C0006"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -260,8 +275,14 @@
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -341,11 +362,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00023859"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D1D1"/>
+      </right>
+      <top style="medium">
+        <color rgb="00023859"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00023859"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D1D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D1D1"/>
+      </right>
+      <top style="medium">
+        <color rgb="00023859"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D1D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -465,6 +530,9 @@
     <xf numFmtId="0" fontId="25" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -830,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4946,6 +5014,1600 @@
         </is>
       </c>
       <c r="L87" s="8" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Luis Saez</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>luis.saez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K88" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Biohotel</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Maria Del Pilar Narvaez</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>pilar.narvaez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K89" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Bioxury</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>calidad.bioxury@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K90" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Geotel Antofagasta</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Nelson Uriel Perez Ortiz</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>nelson.perez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K91" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Katherine Mora</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>katherine.mora@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K92" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>GHL Collection 93</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>James Mendoza</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>james.mendoza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K93" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Armeria Real</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Saray Estrada</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Saray.estrada@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para agosto</t>
+        </is>
+      </c>
+      <c r="K94" s="45" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>GHL Collection Hamilton</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Wilson Bohorquez</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>andres.bohorquez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K95" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>GHL Grand Villavicencio</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Ingrid Mendez</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>jimena.mendez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K96" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>GHL Hotel Capital</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Maira Piza</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>maira.piza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K97" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>GHL Lago Titicaca</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Milagros Velazco Reyes</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>milagros.velazco@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K98" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>GHL Montería</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Jose Medina</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>mauricio.medina@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para agosto</t>
+        </is>
+      </c>
+      <c r="K99" s="45" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>GHL Portón Medellín</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Jose Fernando Villareal</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>jose.villareal@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K100" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Maria Gomez</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>angelica.gomez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K101" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Corales de Indias</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Andres Narvaez</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>andres.narvaez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K102" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Costa Azul</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Marlis Marriaga</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>marlys.marriaga@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para agosto</t>
+        </is>
+      </c>
+      <c r="K103" s="45" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Juan Martinez</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>juan.martinez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K104" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>GHL Style Barrancabermeja</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Luis Martinez</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>luis.martinez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K105" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>GHL Style Bogotá Occidente</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Leidy Cely</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>jrecepcion.bogotaoccidente@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K106" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>GHL Style Neiva</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Carlos Robayo</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>yobani.robayo@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K107" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Mafy Daniela Rodriguez</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>daniela.rodriguez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K108" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Hotel Tequendama Bogotá</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Sara Judith Aguirre</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>sara.aguirre@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K109" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Katerine Ospina Gil</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>suprecepcion.abadiaplaza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K110" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Jose Carlos Ibañez</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>jose.ibanez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K111" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>LATAM XELA</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Gabriela Rodas</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>gabriela.rodas@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K112" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Jose Macea</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>jose.macea@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K113" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>reservas.parklake@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K114" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>San Lazaro Art</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Keilis Mercado</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>keilis.mercado@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K115" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Sonesta Bucaramanga</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Jeferson Reyes</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>jeferson.reyes@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K116" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Sonesta Cali</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Lorena Figueroa</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>lorena.figueroa@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K117" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Sonesta Cartagena</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Liliana Rodriguez</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>liliana.rodriguez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K118" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Sonesta Cusco</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Adolfo Alfaro</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>adolfo.alfaro@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para agosto</t>
+        </is>
+      </c>
+      <c r="K119" s="45" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Andrea Silvana Zevallos</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>andrea.zevallos@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K120" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Tania Catacora</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>jefederecepcion.sonestaarequipa@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K121" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Catalina Rojas</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>catalina.rojas@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K122" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Sonesta Ibagué</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Wilmer Rodriguez</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>wilmer.rodriguez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K123" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Sonesta Loja</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Miryam Ramirez</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>miryam.ramirez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K124" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Sonesta Osorno</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Cristina Sanzana</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>cristina.sanzana@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K125" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Edwar Pacanchique</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>edwar.pacanchique@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K126" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Sonesta Puno</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Delmy Nuñez</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>delmy.nunez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K127" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Sonesta Yucay</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Monica Chirinos</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>monica.chirinos@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K128" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Sonesta Valledupar</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Emerson David Cotes</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>emerson.cotes@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K129" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:M87"/>
@@ -4971,7 +6633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5111,6 +6773,40 @@
       </c>
       <c r="I5" s="17">
         <f>IF(B5&gt;0,C5/B5,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>38</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="I6" s="17">
+        <f>IF(B6&gt;0,C6/B6,0)</f>
         <v/>
       </c>
     </row>
@@ -5138,7 +6834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5222,106 +6918,140 @@
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
         <is>
-          <t>Jul-26</t>
+          <t>Ago-26</t>
         </is>
       </c>
       <c r="B4" s="19" t="n">
         <v>42</v>
       </c>
       <c r="C4" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>38</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="20" t="n">
+        <v>0.09523809523809523</v>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>███░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+      <c r="I4" s="22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>42</v>
+      </c>
+      <c r="C5" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="D4" s="19" t="n">
+      <c r="D5" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E5" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F5" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="G4" s="20" t="n">
+      <c r="G5" s="20" t="n">
         <v>0.3809523809523809</v>
       </c>
-      <c r="H4" s="21" t="inlineStr">
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>███████████░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
-      <c r="I4" s="22" t="inlineStr">
+      <c r="I5" s="22" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="23" t="inlineStr">
-        <is>
-          <t>Jun-26</t>
-        </is>
-      </c>
-      <c r="B5" s="24" t="n">
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n">
         <v>42</v>
       </c>
-      <c r="C5" s="24" t="n">
+      <c r="C6" s="24" t="n">
         <v>23</v>
       </c>
-      <c r="D5" s="24" t="n">
+      <c r="D6" s="24" t="n">
         <v>19</v>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="E6" s="24" t="n">
         <v>23</v>
       </c>
-      <c r="F5" s="24" t="n">
+      <c r="F6" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="20" t="n">
+      <c r="G6" s="20" t="n">
         <v>0.5476190476190477</v>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H6" s="25" t="inlineStr">
         <is>
           <t>████████████████░░░░░░░░░░░░░░</t>
         </is>
       </c>
-      <c r="I5" s="26" t="inlineStr">
+      <c r="I6" s="26" t="inlineStr">
         <is>
           <t>En progreso</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="28" t="n">
-        <v>84</v>
-      </c>
-      <c r="C6" s="28" t="n">
-        <v>39</v>
-      </c>
-      <c r="D6" s="28" t="n">
-        <v>45</v>
-      </c>
-      <c r="E6" s="28" t="n">
+      <c r="B7" t="n">
+        <v>126</v>
+      </c>
+      <c r="C7" t="n">
+        <v>43</v>
+      </c>
+      <c r="D7" t="n">
+        <v>83</v>
+      </c>
+      <c r="E7" t="n">
         <v>31</v>
       </c>
-      <c r="F6" s="28" t="n">
-        <v>8</v>
-      </c>
-      <c r="G6" s="29" t="n">
-        <v>0.4642857142857143</v>
-      </c>
-      <c r="H6" s="30" t="inlineStr">
-        <is>
-          <t>██████████████░░░░░░░░░░░░░░░░</t>
-        </is>
-      </c>
-      <c r="I6" s="28" t="inlineStr"/>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="36" t="inlineStr">
+      <c r="F7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.3412698412698413</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>██████████░░░░░░░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="inlineStr">
         <is>
           <t>Nota: La barra de progreso refleja % de hoteles que respondieron el correo (con o sin modificaciones). Completo = 100% · En progreso = 50-99% · Pendiente = &lt; 50%</t>
         </is>
@@ -5329,9 +7059,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A7:I7"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A6"/>
+    <mergeCell ref="A8:I8"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17767,8 +19497,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Registra respuestas de agosto de 12 hoteles con modificaciones
Extrae y registra 91 diálogos modificados de 12 hoteles a partir de los
correos de la carpeta Agosto (Sonesta Bogotá, Sonesta El Olivar, Sonesta
Osorno, GHL Style Yopal, Geotel Calama, GHL Style Bogotá Occidente, GHL
Hotel Grand Barranquilla, Sonesta Arequipa, Arsenal, Hotel Tequendama
Bogotá, GHL Relax Club Hotel el Puente, Sonesta Bucaramanga). Quedan en
estado "Pendiente actualización" hasta confirmar carga en el chatbot.

Se actualizan Dashboard cumplimiento y Resumen por ciclo con los nuevos
totales de Ago-26.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -184,6 +184,11 @@
     <font>
       <name val="Calibri"/>
       <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00856404"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -410,7 +415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -533,6 +538,7 @@
     <xf numFmtId="0" fontId="26" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5041,14 +5047,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K88" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>2 diálogos modificados: Breakfast time, Fitness gym</t>
+        </is>
+      </c>
+      <c r="K88" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -5189,14 +5205,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K92" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>14 diálogos modificados: Contact staff, Laundry/paraguas, Invoice, Currencies, Accommodation, Family accommodation, ...</t>
+        </is>
+      </c>
+      <c r="K92" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -5542,14 +5568,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K101" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>11 diálogos modificados: Opening, closing &amp; renovation, Day use reservation, Extra bed, View, TV, Pets, ...</t>
+        </is>
+      </c>
+      <c r="K101" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -5737,14 +5773,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K106" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>3 diálogos modificados: Business meetings, Breakfast rates, Private transfer</t>
+        </is>
+      </c>
+      <c r="K106" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -5811,14 +5857,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K108" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>7 diálogos modificados: Payment method, Check-in time, Check-out time, Breakfast time, Breakfast rates, Pets, ...</t>
+        </is>
+      </c>
+      <c r="K108" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -5848,14 +5904,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K109" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>2 diálogos modificados: Room service, Restaurant</t>
+        </is>
+      </c>
+      <c r="K109" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -5922,14 +5988,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K111" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>11 diálogos modificados: City tax, fees &amp; VAT, Payment method, Kids, Private transfer, Taxi, Smoking, ...</t>
+        </is>
+      </c>
+      <c r="K111" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -6107,14 +6183,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K116" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>4 diálogos modificados: Room service, Bar, Rooftop, Restaurant</t>
+        </is>
+      </c>
+      <c r="K116" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -6265,14 +6351,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K120" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>17 diálogos modificados: Contact staff, Check-in time, Check-out time, Breakfast rates, Parking, Connecting accommodation, ...</t>
+        </is>
+      </c>
+      <c r="K120" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -6302,14 +6398,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K121" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>14 diálogos modificados: Breakfast reservation, Medical services, Currencies, Private transfer reservation, Accommodation, Smoking, ...</t>
+        </is>
+      </c>
+      <c r="K121" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -6339,14 +6445,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K122" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>5 diálogos modificados: Breakfast time, Breakfast rates, Room service, Extra bed, Balcony &amp; windows</t>
+        </is>
+      </c>
+      <c r="K122" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -6450,14 +6566,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K125" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>1 diálogos modificados: Breakfast rates</t>
+        </is>
+      </c>
+      <c r="K125" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -6786,13 +6912,13 @@
         <v>42</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F6" s="12" t="n">
         <v>4</v>
@@ -6802,7 +6928,7 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="I6" s="17">
@@ -6925,23 +7051,23 @@
         <v>42</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F4" s="19" t="n">
         <v>4</v>
       </c>
       <c r="G4" s="20" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>███░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>███████████░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I4" s="22" t="inlineStr">
@@ -7030,23 +7156,23 @@
         <v>126</v>
       </c>
       <c r="C7" t="n">
+        <v>55</v>
+      </c>
+      <c r="D7" t="n">
+        <v>71</v>
+      </c>
+      <c r="E7" t="n">
         <v>43</v>
-      </c>
-      <c r="D7" t="n">
-        <v>83</v>
-      </c>
-      <c r="E7" t="n">
-        <v>31</v>
       </c>
       <c r="F7" t="n">
         <v>12</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3412698412698413</v>
+        <v>0.4365079365079365</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>██████████░░░░░░░░░░░░░░░░░░░░</t>
+          <t>█████████████░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -7074,7 +7200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H319"/>
+  <dimension ref="A1:H410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19166,6 +19292,3464 @@
         </is>
       </c>
       <c r="H319" s="41" t="n"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B320" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C320" s="41" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="D320" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E320" s="41" t="inlineStr">
+        <is>
+          <t>Servicio de desayuno en habitación</t>
+        </is>
+      </c>
+      <c r="F320" s="41" t="inlineStr">
+        <is>
+          <t>No se ofrecía desayuno en habitación</t>
+        </is>
+      </c>
+      <c r="G320" s="41" t="inlineStr">
+        <is>
+          <t>Se ofrece con costo adicional de $68.000 COP</t>
+        </is>
+      </c>
+      <c r="H320" s="41" t="n"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B321" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C321" s="41" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="D321" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E321" s="41" t="inlineStr">
+        <is>
+          <t>Precio por adulto</t>
+        </is>
+      </c>
+      <c r="F321" s="41" t="inlineStr">
+        <is>
+          <t>$65.000 COP</t>
+        </is>
+      </c>
+      <c r="G321" s="41" t="inlineStr">
+        <is>
+          <t>$68.000 COP</t>
+        </is>
+      </c>
+      <c r="H321" s="41" t="n"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B322" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C322" s="41" t="inlineStr">
+        <is>
+          <t>13-06</t>
+        </is>
+      </c>
+      <c r="D322" s="41" t="inlineStr">
+        <is>
+          <t>Room service</t>
+        </is>
+      </c>
+      <c r="E322" s="41" t="inlineStr">
+        <is>
+          <t>Horario y código de marcado</t>
+        </is>
+      </c>
+      <c r="F322" s="41" t="inlineStr">
+        <is>
+          <t>07:00 a 21:00, marcar 2</t>
+        </is>
+      </c>
+      <c r="G322" s="41" t="inlineStr">
+        <is>
+          <t>Disponible 24/7, marcar 1</t>
+        </is>
+      </c>
+      <c r="H322" s="41" t="n"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B323" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C323" s="41" t="inlineStr">
+        <is>
+          <t>15-23</t>
+        </is>
+      </c>
+      <c r="D323" s="41" t="inlineStr">
+        <is>
+          <t>Extra bed</t>
+        </is>
+      </c>
+      <c r="E323" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad y solicitud</t>
+        </is>
+      </c>
+      <c r="F323" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado previamente</t>
+        </is>
+      </c>
+      <c r="G323" s="41" t="inlineStr">
+        <is>
+          <t>Cama supletoria disponible; solicitar a reservas.sonestabogota@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="H323" s="41" t="n"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B324" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C324" s="41" t="inlineStr">
+        <is>
+          <t>15-61</t>
+        </is>
+      </c>
+      <c r="D324" s="41" t="inlineStr">
+        <is>
+          <t>Balcony &amp; windows</t>
+        </is>
+      </c>
+      <c r="E324" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad de balcón</t>
+        </is>
+      </c>
+      <c r="F324" s="41" t="inlineStr">
+        <is>
+          <t>Todas las habitaciones tienen balcón</t>
+        </is>
+      </c>
+      <c r="G324" s="41" t="inlineStr">
+        <is>
+          <t>Se elimina esa afirmación (ventanas no se abren por seguridad)</t>
+        </is>
+      </c>
+      <c r="H324" s="41" t="n"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B325" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C325" s="41" t="inlineStr">
+        <is>
+          <t>16-02</t>
+        </is>
+      </c>
+      <c r="D325" s="41" t="inlineStr">
+        <is>
+          <t>Contact staff</t>
+        </is>
+      </c>
+      <c r="E325" s="41" t="inlineStr">
+        <is>
+          <t>Teléfonos por departamento y correo reservas</t>
+        </is>
+      </c>
+      <c r="F325" s="41" t="inlineStr">
+        <is>
+          <t>Solo correos; reservas.sonestaolivar1@...</t>
+        </is>
+      </c>
+      <c r="G325" s="41" t="inlineStr">
+        <is>
+          <t>Se agregan celulares por área; correo reservas pasa a reservas.sonestaolivar@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="H325" s="41" t="n"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B326" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C326" s="41" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="D326" s="41" t="inlineStr">
+        <is>
+          <t>Check-in time</t>
+        </is>
+      </c>
+      <c r="E326" s="41" t="inlineStr">
+        <is>
+          <t>Costo early check-in</t>
+        </is>
+      </c>
+      <c r="F326" s="41" t="inlineStr">
+        <is>
+          <t>Desde 07:00 por 83.300 USD/habitación</t>
+        </is>
+      </c>
+      <c r="G326" s="41" t="inlineStr">
+        <is>
+          <t>Desde 10:00 por media tarifa/habitación</t>
+        </is>
+      </c>
+      <c r="H326" s="41" t="n"/>
+    </row>
+    <row r="327">
+      <c r="A327" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B327" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C327" s="41" t="inlineStr">
+        <is>
+          <t>11-11</t>
+        </is>
+      </c>
+      <c r="D327" s="41" t="inlineStr">
+        <is>
+          <t>Check-out time</t>
+        </is>
+      </c>
+      <c r="E327" s="41" t="inlineStr">
+        <is>
+          <t>Check-out normal y tardío</t>
+        </is>
+      </c>
+      <c r="F327" s="41" t="inlineStr">
+        <is>
+          <t>Antes de 13:00; tardío 83.300 USD</t>
+        </is>
+      </c>
+      <c r="G327" s="41" t="inlineStr">
+        <is>
+          <t>Antes del mediodía; tardío por media tarifa</t>
+        </is>
+      </c>
+      <c r="H327" s="41" t="n"/>
+    </row>
+    <row r="328">
+      <c r="A328" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B328" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C328" s="41" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="D328" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E328" s="41" t="inlineStr">
+        <is>
+          <t>Precio adulto/niño</t>
+        </is>
+      </c>
+      <c r="F328" s="41" t="inlineStr">
+        <is>
+          <t>26 USD adulto / 14 USD niño</t>
+        </is>
+      </c>
+      <c r="G328" s="41" t="inlineStr">
+        <is>
+          <t>S/79 (Lun-Sáb) / S/89 (Dom) adulto; S/45 niño</t>
+        </is>
+      </c>
+      <c r="H328" s="41" t="n"/>
+    </row>
+    <row r="329">
+      <c r="A329" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B329" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C329" s="41" t="inlineStr">
+        <is>
+          <t>13-01</t>
+        </is>
+      </c>
+      <c r="D329" s="41" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="E329" s="41" t="inlineStr">
+        <is>
+          <t>Servicio de aparcacoches</t>
+        </is>
+      </c>
+      <c r="F329" s="41" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="G329" s="41" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="H329" s="41" t="n"/>
+    </row>
+    <row r="330">
+      <c r="A330" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B330" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C330" s="41" t="inlineStr">
+        <is>
+          <t>14-02</t>
+        </is>
+      </c>
+      <c r="D330" s="41" t="inlineStr">
+        <is>
+          <t>Connecting accommodation</t>
+        </is>
+      </c>
+      <c r="E330" s="41" t="inlineStr">
+        <is>
+          <t>Tipos de habitación conectados</t>
+        </is>
+      </c>
+      <c r="F330" s="41" t="inlineStr">
+        <is>
+          <t>6 tipos disponibles</t>
+        </is>
+      </c>
+      <c r="G330" s="41" t="inlineStr">
+        <is>
+          <t>Solo Executive Double</t>
+        </is>
+      </c>
+      <c r="H330" s="41" t="n"/>
+    </row>
+    <row r="331">
+      <c r="A331" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B331" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C331" s="41" t="inlineStr">
+        <is>
+          <t>14-04</t>
+        </is>
+      </c>
+      <c r="D331" s="41" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="E331" s="41" t="inlineStr">
+        <is>
+          <t>Detectores de humo y tarifa</t>
+        </is>
+      </c>
+      <c r="F331" s="41" t="inlineStr">
+        <is>
+          <t>Sin detectores; tarifa 0 USD</t>
+        </is>
+      </c>
+      <c r="G331" s="41" t="inlineStr">
+        <is>
+          <t>Con detectores; tarifa 200 USD + impuestos</t>
+        </is>
+      </c>
+      <c r="H331" s="41" t="n"/>
+    </row>
+    <row r="332">
+      <c r="A332" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B332" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C332" s="41" t="inlineStr">
+        <is>
+          <t>15-06</t>
+        </is>
+      </c>
+      <c r="D332" s="41" t="inlineStr">
+        <is>
+          <t>Bathroom equipment</t>
+        </is>
+      </c>
+      <c r="E332" s="41" t="inlineStr">
+        <is>
+          <t>Amenidades gratuitas a petición</t>
+        </is>
+      </c>
+      <c r="F332" s="41" t="inlineStr">
+        <is>
+          <t>Pantuflas, pasta dientes, kit afeitar</t>
+        </is>
+      </c>
+      <c r="G332" s="41" t="inlineStr">
+        <is>
+          <t>Pantuflas, vanity kit, kit dental, kit afeitar, peine</t>
+        </is>
+      </c>
+      <c r="H332" s="41" t="n"/>
+    </row>
+    <row r="333">
+      <c r="A333" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B333" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C333" s="41" t="inlineStr">
+        <is>
+          <t>15-09</t>
+        </is>
+      </c>
+      <c r="D333" s="41" t="inlineStr">
+        <is>
+          <t>Shower/bathtub/jacuzzi</t>
+        </is>
+      </c>
+      <c r="E333" s="41" t="inlineStr">
+        <is>
+          <t>Habitaciones con ducha/bañera</t>
+        </is>
+      </c>
+      <c r="F333" s="41" t="inlineStr">
+        <is>
+          <t>Incluye Ejecutiva Simple y Junior Suite con bañera</t>
+        </is>
+      </c>
+      <c r="G333" s="41" t="inlineStr">
+        <is>
+          <t>Se renombran categorías; Suite solo con ducha</t>
+        </is>
+      </c>
+      <c r="H333" s="41" t="n"/>
+    </row>
+    <row r="334">
+      <c r="A334" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B334" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C334" s="41" t="inlineStr">
+        <is>
+          <t>15-61</t>
+        </is>
+      </c>
+      <c r="D334" s="41" t="inlineStr">
+        <is>
+          <t>Balcony &amp; windows</t>
+        </is>
+      </c>
+      <c r="E334" s="41" t="inlineStr">
+        <is>
+          <t>Ventanas y balcón</t>
+        </is>
+      </c>
+      <c r="F334" s="41" t="inlineStr">
+        <is>
+          <t>No se abren; todas con balcón</t>
+        </is>
+      </c>
+      <c r="G334" s="41" t="inlineStr">
+        <is>
+          <t>Sí se abren; no todas tienen balcón</t>
+        </is>
+      </c>
+      <c r="H334" s="41" t="n"/>
+    </row>
+    <row r="335">
+      <c r="A335" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B335" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C335" s="41" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D335" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E335" s="41" t="inlineStr">
+        <is>
+          <t>Restricciones</t>
+        </is>
+      </c>
+      <c r="F335" s="41" t="inlineStr">
+        <is>
+          <t>Máx. 2 mascotas; peso 20kg</t>
+        </is>
+      </c>
+      <c r="G335" s="41" t="inlineStr">
+        <is>
+          <t>Solo 2 habitaciones pet-friendly; máx. 1 mascota</t>
+        </is>
+      </c>
+      <c r="H335" s="41" t="n"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B336" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C336" s="41" t="inlineStr">
+        <is>
+          <t>17-01</t>
+        </is>
+      </c>
+      <c r="D336" s="41" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="E336" s="41" t="inlineStr">
+        <is>
+          <t>Horario y servicio de comida</t>
+        </is>
+      </c>
+      <c r="F336" s="41" t="inlineStr">
+        <is>
+          <t>12:00-21:00, se sirve comida</t>
+        </is>
+      </c>
+      <c r="G336" s="41" t="inlineStr">
+        <is>
+          <t>12:00-23:00, ya no se sirve comida</t>
+        </is>
+      </c>
+      <c r="H336" s="41" t="n"/>
+    </row>
+    <row r="337">
+      <c r="A337" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B337" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C337" s="41" t="inlineStr">
+        <is>
+          <t>17-31</t>
+        </is>
+      </c>
+      <c r="D337" s="41" t="inlineStr">
+        <is>
+          <t>Fitness gym</t>
+        </is>
+      </c>
+      <c r="E337" s="41" t="inlineStr">
+        <is>
+          <t>Equipamiento</t>
+        </is>
+      </c>
+      <c r="F337" s="41" t="inlineStr">
+        <is>
+          <t>Solo cinta de correr</t>
+        </is>
+      </c>
+      <c r="G337" s="41" t="inlineStr">
+        <is>
+          <t>Se agregan máquinas, pesas y mat de yoga</t>
+        </is>
+      </c>
+      <c r="H337" s="41" t="n"/>
+    </row>
+    <row r="338">
+      <c r="A338" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B338" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C338" s="41" t="inlineStr">
+        <is>
+          <t>17-34</t>
+        </is>
+      </c>
+      <c r="D338" s="41" t="inlineStr">
+        <is>
+          <t>Rooftop</t>
+        </is>
+      </c>
+      <c r="E338" s="41" t="inlineStr">
+        <is>
+          <t>Acceso</t>
+        </is>
+      </c>
+      <c r="F338" s="41" t="inlineStr">
+        <is>
+          <t>Clientes y visitantes</t>
+        </is>
+      </c>
+      <c r="G338" s="41" t="inlineStr">
+        <is>
+          <t>Solo clientes del hotel</t>
+        </is>
+      </c>
+      <c r="H338" s="41" t="n"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B339" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C339" s="41" t="inlineStr">
+        <is>
+          <t>17-43</t>
+        </is>
+      </c>
+      <c r="D339" s="41" t="inlineStr">
+        <is>
+          <t>Floor arrangement</t>
+        </is>
+      </c>
+      <c r="E339" s="41" t="inlineStr">
+        <is>
+          <t>Piso Senior/Presidential Suite</t>
+        </is>
+      </c>
+      <c r="F339" s="41" t="inlineStr">
+        <is>
+          <t>Cualquier piso</t>
+        </is>
+      </c>
+      <c r="G339" s="41" t="inlineStr">
+        <is>
+          <t>Senior Suite pisos 2-3-4; Presidential piso 5</t>
+        </is>
+      </c>
+      <c r="H339" s="41" t="n"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B340" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C340" s="41" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D340" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E340" s="41" t="inlineStr">
+        <is>
+          <t>Horario Sushi Bar</t>
+        </is>
+      </c>
+      <c r="F340" s="41" t="inlineStr">
+        <is>
+          <t>Lunes a viernes</t>
+        </is>
+      </c>
+      <c r="G340" s="41" t="inlineStr">
+        <is>
+          <t>Lunes a sábado (agrega sábado 13:00-20:00)</t>
+        </is>
+      </c>
+      <c r="H340" s="41" t="n"/>
+    </row>
+    <row r="341">
+      <c r="A341" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B341" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C341" s="41" t="inlineStr">
+        <is>
+          <t>18-08</t>
+        </is>
+      </c>
+      <c r="D341" s="41" t="inlineStr">
+        <is>
+          <t>Takeaway &amp; delivery</t>
+        </is>
+      </c>
+      <c r="E341" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad</t>
+        </is>
+      </c>
+      <c r="F341" s="41" t="inlineStr">
+        <is>
+          <t>Sí, con plataformas</t>
+        </is>
+      </c>
+      <c r="G341" s="41" t="inlineStr">
+        <is>
+          <t>No se realiza delivery</t>
+        </is>
+      </c>
+      <c r="H341" s="41" t="n"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B342" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Osorno</t>
+        </is>
+      </c>
+      <c r="C342" s="41" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="D342" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E342" s="41" t="inlineStr">
+        <is>
+          <t>Precio por adulto</t>
+        </is>
+      </c>
+      <c r="F342" s="41" t="inlineStr">
+        <is>
+          <t>15 USD</t>
+        </is>
+      </c>
+      <c r="G342" s="41" t="inlineStr">
+        <is>
+          <t>25 USD</t>
+        </is>
+      </c>
+      <c r="H342" s="41" t="n"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B343" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C343" s="41" t="inlineStr">
+        <is>
+          <t>10-71</t>
+        </is>
+      </c>
+      <c r="D343" s="41" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="E343" s="41" t="inlineStr">
+        <is>
+          <t>Efectivo y tarjetas aceptadas</t>
+        </is>
+      </c>
+      <c r="F343" s="41" t="inlineStr">
+        <is>
+          <t>No se aceptaba efectivo; sin Visa</t>
+        </is>
+      </c>
+      <c r="G343" s="41" t="inlineStr">
+        <is>
+          <t>Se acepta efectivo; se agrega Visa</t>
+        </is>
+      </c>
+      <c r="H343" s="41" t="n"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B344" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C344" s="41" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="D344" s="41" t="inlineStr">
+        <is>
+          <t>Check-in time</t>
+        </is>
+      </c>
+      <c r="E344" s="41" t="inlineStr">
+        <is>
+          <t>Costo early check-in</t>
+        </is>
+      </c>
+      <c r="F344" s="41" t="inlineStr">
+        <is>
+          <t>70.000 COP</t>
+        </is>
+      </c>
+      <c r="G344" s="41" t="inlineStr">
+        <is>
+          <t>70.000 COP + IVA</t>
+        </is>
+      </c>
+      <c r="H344" s="41" t="n"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B345" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C345" s="41" t="inlineStr">
+        <is>
+          <t>11-11</t>
+        </is>
+      </c>
+      <c r="D345" s="41" t="inlineStr">
+        <is>
+          <t>Check-out time</t>
+        </is>
+      </c>
+      <c r="E345" s="41" t="inlineStr">
+        <is>
+          <t>Costo late check-out</t>
+        </is>
+      </c>
+      <c r="F345" s="41" t="inlineStr">
+        <is>
+          <t>70.000 COP</t>
+        </is>
+      </c>
+      <c r="G345" s="41" t="inlineStr">
+        <is>
+          <t>70.000 COP + IVA</t>
+        </is>
+      </c>
+      <c r="H345" s="41" t="n"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B346" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C346" s="41" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="D346" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E346" s="41" t="inlineStr">
+        <is>
+          <t>Horario y servicio en habitación</t>
+        </is>
+      </c>
+      <c r="F346" s="41" t="inlineStr">
+        <is>
+          <t>06:00-10:00 todos los días; sin servicio en habitación</t>
+        </is>
+      </c>
+      <c r="G346" s="41" t="inlineStr">
+        <is>
+          <t>Lun-Sáb 06:00-10:00, Dom/festivos 06:00-10:30; ahora con servicio en habitación (costo adicional)</t>
+        </is>
+      </c>
+      <c r="H346" s="41" t="n"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B347" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C347" s="41" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="D347" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E347" s="41" t="inlineStr">
+        <is>
+          <t>Precio por adulto</t>
+        </is>
+      </c>
+      <c r="F347" s="41" t="inlineStr">
+        <is>
+          <t>48.000 COP</t>
+        </is>
+      </c>
+      <c r="G347" s="41" t="inlineStr">
+        <is>
+          <t>40.000 COP</t>
+        </is>
+      </c>
+      <c r="H347" s="41" t="n"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B348" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C348" s="41" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D348" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E348" s="41" t="inlineStr">
+        <is>
+          <t>Tasa por mascota</t>
+        </is>
+      </c>
+      <c r="F348" s="41" t="inlineStr">
+        <is>
+          <t>70.000 COP/mascota</t>
+        </is>
+      </c>
+      <c r="G348" s="41" t="inlineStr">
+        <is>
+          <t>70.000 COP + IVA/mascota</t>
+        </is>
+      </c>
+      <c r="H348" s="41" t="n"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B349" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C349" s="41" t="inlineStr">
+        <is>
+          <t>17-15</t>
+        </is>
+      </c>
+      <c r="D349" s="41" t="inlineStr">
+        <is>
+          <t>Spa hours</t>
+        </is>
+      </c>
+      <c r="E349" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad de spa</t>
+        </is>
+      </c>
+      <c r="F349" s="41" t="inlineStr">
+        <is>
+          <t>Horario sin límite, todo el año</t>
+        </is>
+      </c>
+      <c r="G349" s="41" t="inlineStr">
+        <is>
+          <t>Ya no se cuenta con spa</t>
+        </is>
+      </c>
+      <c r="H349" s="41" t="n"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B350" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C350" s="41" t="inlineStr">
+        <is>
+          <t>16-02</t>
+        </is>
+      </c>
+      <c r="D350" s="41" t="inlineStr">
+        <is>
+          <t>Contact staff</t>
+        </is>
+      </c>
+      <c r="E350" s="41" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="F350" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G350" s="41" t="inlineStr">
+        <is>
+          <t>+56 931909316 / +56 996795687</t>
+        </is>
+      </c>
+      <c r="H350" s="41" t="n"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B351" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C351" s="41" t="inlineStr">
+        <is>
+          <t>13-15</t>
+        </is>
+      </c>
+      <c r="D351" s="41" t="inlineStr">
+        <is>
+          <t>Laundry/paraguas</t>
+        </is>
+      </c>
+      <c r="E351" s="41" t="inlineStr">
+        <is>
+          <t>Servicio de paraguas y lavandería</t>
+        </is>
+      </c>
+      <c r="F351" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G351" s="41" t="inlineStr">
+        <is>
+          <t>No disponen de paraguas; ofrecen lavandería regular y express (+50% recargo)</t>
+        </is>
+      </c>
+      <c r="H351" s="41" t="n"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B352" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C352" s="41" t="inlineStr">
+        <is>
+          <t>13-47</t>
+        </is>
+      </c>
+      <c r="D352" s="41" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="E352" s="41" t="inlineStr">
+        <is>
+          <t>Datos requeridos</t>
+        </is>
+      </c>
+      <c r="F352" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G352" s="41" t="inlineStr">
+        <is>
+          <t>Enviar Rol Único Tributario por correo o presentarlo en recepción</t>
+        </is>
+      </c>
+      <c r="H352" s="41" t="n"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B353" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C353" s="41" t="inlineStr">
+        <is>
+          <t>13-48</t>
+        </is>
+      </c>
+      <c r="D353" s="41" t="inlineStr">
+        <is>
+          <t>Currencies</t>
+        </is>
+      </c>
+      <c r="E353" s="41" t="inlineStr">
+        <is>
+          <t>Monedas aceptadas</t>
+        </is>
+      </c>
+      <c r="F353" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G353" s="41" t="inlineStr">
+        <is>
+          <t>Aceptan pagos en CLP y USD; facturas en CLP y USD</t>
+        </is>
+      </c>
+      <c r="H353" s="41" t="n"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B354" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C354" s="41" t="inlineStr">
+        <is>
+          <t>14-01</t>
+        </is>
+      </c>
+      <c r="D354" s="41" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="E354" s="41" t="inlineStr">
+        <is>
+          <t>Ocupación y composición por tipo</t>
+        </is>
+      </c>
+      <c r="F354" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G354" s="41" t="inlineStr">
+        <is>
+          <t>Queen/Junior Suite: máx. 2 adultos+1 niño; Suite especial: máx. 4 adultos+2 niños; no fumar ni mascotas</t>
+        </is>
+      </c>
+      <c r="H354" s="41" t="n"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B355" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C355" s="41" t="inlineStr">
+        <is>
+          <t>14-03</t>
+        </is>
+      </c>
+      <c r="D355" s="41" t="inlineStr">
+        <is>
+          <t>Family accommodation</t>
+        </is>
+      </c>
+      <c r="E355" s="41" t="inlineStr">
+        <is>
+          <t>Ocupación máxima por tipo</t>
+        </is>
+      </c>
+      <c r="F355" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G355" s="41" t="inlineStr">
+        <is>
+          <t>Queen y Junior Suite máx. 2 adultos+1 niño; Suite Doble máx. 4 adultos+2 niños</t>
+        </is>
+      </c>
+      <c r="H355" s="41" t="n"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B356" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C356" s="41" t="inlineStr">
+        <is>
+          <t>14-04</t>
+        </is>
+      </c>
+      <c r="D356" s="41" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="E356" s="41" t="inlineStr">
+        <is>
+          <t>Tarifa limpieza por humo</t>
+        </is>
+      </c>
+      <c r="F356" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G356" s="41" t="inlineStr">
+        <is>
+          <t>200 USD</t>
+        </is>
+      </c>
+      <c r="H356" s="41" t="n"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B357" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C357" s="41" t="inlineStr">
+        <is>
+          <t>15-26</t>
+        </is>
+      </c>
+      <c r="D357" s="41" t="inlineStr">
+        <is>
+          <t>Twin beds</t>
+        </is>
+      </c>
+      <c r="E357" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad</t>
+        </is>
+      </c>
+      <c r="F357" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G357" s="41" t="inlineStr">
+        <is>
+          <t>No ofrecen camas individuales, adicionales ni sofacamas</t>
+        </is>
+      </c>
+      <c r="H357" s="41" t="n"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B358" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C358" s="41" t="inlineStr">
+        <is>
+          <t>15-48</t>
+        </is>
+      </c>
+      <c r="D358" s="41" t="inlineStr">
+        <is>
+          <t>Electrical facilities</t>
+        </is>
+      </c>
+      <c r="E358" s="41" t="inlineStr">
+        <is>
+          <t>Adaptadores y cargador</t>
+        </is>
+      </c>
+      <c r="F358" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G358" s="41" t="inlineStr">
+        <is>
+          <t>Consultar disponibilidad y precio en recepción</t>
+        </is>
+      </c>
+      <c r="H358" s="41" t="n"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B359" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C359" s="41" t="inlineStr">
+        <is>
+          <t>15-61</t>
+        </is>
+      </c>
+      <c r="D359" s="41" t="inlineStr">
+        <is>
+          <t>Balcony &amp; windows</t>
+        </is>
+      </c>
+      <c r="E359" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad de balcón</t>
+        </is>
+      </c>
+      <c r="F359" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G359" s="41" t="inlineStr">
+        <is>
+          <t>Junior Suite y Suite Doble cuentan con balcones pequeños</t>
+        </is>
+      </c>
+      <c r="H359" s="41" t="n"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B360" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C360" s="41" t="inlineStr">
+        <is>
+          <t>17-15</t>
+        </is>
+      </c>
+      <c r="D360" s="41" t="inlineStr">
+        <is>
+          <t>Spa hours</t>
+        </is>
+      </c>
+      <c r="E360" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad de spa</t>
+        </is>
+      </c>
+      <c r="F360" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G360" s="41" t="inlineStr">
+        <is>
+          <t>No cuentan con spa</t>
+        </is>
+      </c>
+      <c r="H360" s="41" t="n"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B361" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C361" s="41" t="inlineStr">
+        <is>
+          <t>17-31</t>
+        </is>
+      </c>
+      <c r="D361" s="41" t="inlineStr">
+        <is>
+          <t>Fitness gym</t>
+        </is>
+      </c>
+      <c r="E361" s="41" t="inlineStr">
+        <is>
+          <t>Horario y acceso</t>
+        </is>
+      </c>
+      <c r="F361" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G361" s="41" t="inlineStr">
+        <is>
+          <t>Lun-Dom 05:00-23:00, código de acceso en recepción</t>
+        </is>
+      </c>
+      <c r="H361" s="41" t="n"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B362" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C362" s="41" t="inlineStr">
+        <is>
+          <t>17-44</t>
+        </is>
+      </c>
+      <c r="D362" s="41" t="inlineStr">
+        <is>
+          <t>Disabled guest</t>
+        </is>
+      </c>
+      <c r="E362" s="41" t="inlineStr">
+        <is>
+          <t>Habitación adaptada</t>
+        </is>
+      </c>
+      <c r="F362" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G362" s="41" t="inlineStr">
+        <is>
+          <t>Habitación con 2 camas individuales y baño adaptado</t>
+        </is>
+      </c>
+      <c r="H362" s="41" t="n"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B363" s="41" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C363" s="41" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D363" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E363" s="41" t="inlineStr">
+        <is>
+          <t>Nombre y capacidad</t>
+        </is>
+      </c>
+      <c r="F363" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G363" s="41" t="inlineStr">
+        <is>
+          <t>Restaurante "Entre piedras"; ofrece tronas/sillas para niños</t>
+        </is>
+      </c>
+      <c r="H363" s="41" t="n"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B364" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Bogotá Occidente</t>
+        </is>
+      </c>
+      <c r="C364" s="41" t="inlineStr">
+        <is>
+          <t>20-01</t>
+        </is>
+      </c>
+      <c r="D364" s="41" t="inlineStr">
+        <is>
+          <t>Business meetings</t>
+        </is>
+      </c>
+      <c r="E364" s="41" t="inlineStr">
+        <is>
+          <t>Correo de contacto eventos</t>
+        </is>
+      </c>
+      <c r="F364" s="41" t="inlineStr">
+        <is>
+          <t>sandra.castillo@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="G364" s="41" t="inlineStr">
+        <is>
+          <t>eventos.bogotaoccidente@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="H364" s="41" t="n"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B365" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Bogotá Occidente</t>
+        </is>
+      </c>
+      <c r="C365" s="41" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="D365" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E365" s="41" t="inlineStr">
+        <is>
+          <t>Redacción del beneficio</t>
+        </is>
+      </c>
+      <c r="F365" s="41" t="inlineStr">
+        <is>
+          <t>"Incluido en la tarifa"</t>
+        </is>
+      </c>
+      <c r="G365" s="41" t="inlineStr">
+        <is>
+          <t>"Cortesía para huéspedes" (no reembolsable)</t>
+        </is>
+      </c>
+      <c r="H365" s="41" t="n"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B366" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Bogotá Occidente</t>
+        </is>
+      </c>
+      <c r="C366" s="41" t="inlineStr">
+        <is>
+          <t>13-51</t>
+        </is>
+      </c>
+      <c r="D366" s="41" t="inlineStr">
+        <is>
+          <t>Private transfer</t>
+        </is>
+      </c>
+      <c r="E366" s="41" t="inlineStr">
+        <is>
+          <t>Tarifas aeropuerto y espera</t>
+        </is>
+      </c>
+      <c r="F366" s="41" t="inlineStr">
+        <is>
+          <t>$95.000/$100.000; espera $30.000</t>
+        </is>
+      </c>
+      <c r="G366" s="41" t="inlineStr">
+        <is>
+          <t>$102.000/$107.000; espera $33.000</t>
+        </is>
+      </c>
+      <c r="H366" s="41" t="n"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B367" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C367" s="41" t="inlineStr">
+        <is>
+          <t>10-51</t>
+        </is>
+      </c>
+      <c r="D367" s="41" t="inlineStr">
+        <is>
+          <t>City tax, fees &amp; VAT</t>
+        </is>
+      </c>
+      <c r="E367" s="41" t="inlineStr">
+        <is>
+          <t>Impuestos aplicables</t>
+        </is>
+      </c>
+      <c r="F367" s="41" t="inlineStr">
+        <is>
+          <t>No hay impuesto municipal</t>
+        </is>
+      </c>
+      <c r="G367" s="41" t="inlineStr">
+        <is>
+          <t>Se cobran IVA e IPC (exento para extranjeros que califiquen)</t>
+        </is>
+      </c>
+      <c r="H367" s="41" t="n"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B368" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C368" s="41" t="inlineStr">
+        <is>
+          <t>10-71</t>
+        </is>
+      </c>
+      <c r="D368" s="41" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="E368" s="41" t="inlineStr">
+        <is>
+          <t>Métodos de pago aceptados</t>
+        </is>
+      </c>
+      <c r="F368" s="41" t="inlineStr">
+        <is>
+          <t>Incluía Paypal</t>
+        </is>
+      </c>
+      <c r="G368" s="41" t="inlineStr">
+        <is>
+          <t>Se retira Paypal de la lista</t>
+        </is>
+      </c>
+      <c r="H368" s="41" t="n"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B369" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C369" s="41" t="inlineStr">
+        <is>
+          <t>13-21</t>
+        </is>
+      </c>
+      <c r="D369" s="41" t="inlineStr">
+        <is>
+          <t>Kids</t>
+        </is>
+      </c>
+      <c r="E369" s="41" t="inlineStr">
+        <is>
+          <t>Rango de edad tarifa infantil</t>
+        </is>
+      </c>
+      <c r="F369" s="41" t="inlineStr">
+        <is>
+          <t>12 a 18 años</t>
+        </is>
+      </c>
+      <c r="G369" s="41" t="inlineStr">
+        <is>
+          <t>12 a 17 años</t>
+        </is>
+      </c>
+      <c r="H369" s="41" t="n"/>
+    </row>
+    <row r="370">
+      <c r="A370" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B370" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C370" s="41" t="inlineStr">
+        <is>
+          <t>13-51</t>
+        </is>
+      </c>
+      <c r="D370" s="41" t="inlineStr">
+        <is>
+          <t>Private transfer</t>
+        </is>
+      </c>
+      <c r="E370" s="41" t="inlineStr">
+        <is>
+          <t>Tarifa en USD</t>
+        </is>
+      </c>
+      <c r="F370" s="41" t="inlineStr">
+        <is>
+          <t>15 USD (ida y vuelta)</t>
+        </is>
+      </c>
+      <c r="G370" s="41" t="inlineStr">
+        <is>
+          <t>25 USD (ida y vuelta)</t>
+        </is>
+      </c>
+      <c r="H370" s="41" t="n"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B371" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C371" s="41" t="inlineStr">
+        <is>
+          <t>13-53</t>
+        </is>
+      </c>
+      <c r="D371" s="41" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="E371" s="41" t="inlineStr">
+        <is>
+          <t>Precios de referencia</t>
+        </is>
+      </c>
+      <c r="F371" s="41" t="inlineStr">
+        <is>
+          <t>Estadio 30.000, Malecón 20.000, Ventana 1.000 COP</t>
+        </is>
+      </c>
+      <c r="G371" s="41" t="inlineStr">
+        <is>
+          <t>Estadio 35.000, Malecón 25.000, Ventana 15.000 COP</t>
+        </is>
+      </c>
+      <c r="H371" s="41" t="n"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B372" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C372" s="41" t="inlineStr">
+        <is>
+          <t>14-04</t>
+        </is>
+      </c>
+      <c r="D372" s="41" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="E372" s="41" t="inlineStr">
+        <is>
+          <t>Tarifa limpieza por humo</t>
+        </is>
+      </c>
+      <c r="F372" s="41" t="inlineStr">
+        <is>
+          <t>35.000 COP</t>
+        </is>
+      </c>
+      <c r="G372" s="41" t="inlineStr">
+        <is>
+          <t>100 USD</t>
+        </is>
+      </c>
+      <c r="H372" s="41" t="n"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B373" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C373" s="41" t="inlineStr">
+        <is>
+          <t>17-01</t>
+        </is>
+      </c>
+      <c r="D373" s="41" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="E373" s="41" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="F373" s="41" t="inlineStr">
+        <is>
+          <t>Texto genérico sin información</t>
+        </is>
+      </c>
+      <c r="G373" s="41" t="inlineStr">
+        <is>
+          <t>Lobby Bar en el primer piso con bebidas y alimentos</t>
+        </is>
+      </c>
+      <c r="H373" s="41" t="n"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B374" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C374" s="41" t="inlineStr">
+        <is>
+          <t>17-15</t>
+        </is>
+      </c>
+      <c r="D374" s="41" t="inlineStr">
+        <is>
+          <t>Spa hours</t>
+        </is>
+      </c>
+      <c r="E374" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad de spa</t>
+        </is>
+      </c>
+      <c r="F374" s="41" t="inlineStr">
+        <is>
+          <t>Listaba horario de spa</t>
+        </is>
+      </c>
+      <c r="G374" s="41" t="inlineStr">
+        <is>
+          <t>No cuentan con spa</t>
+        </is>
+      </c>
+      <c r="H374" s="41" t="n"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B375" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C375" s="41" t="inlineStr">
+        <is>
+          <t>17-31</t>
+        </is>
+      </c>
+      <c r="D375" s="41" t="inlineStr">
+        <is>
+          <t>Fitness gym</t>
+        </is>
+      </c>
+      <c r="E375" s="41" t="inlineStr">
+        <is>
+          <t>Ubicación</t>
+        </is>
+      </c>
+      <c r="F375" s="41" t="inlineStr">
+        <is>
+          <t>Piso 123 (error tipográfico)</t>
+        </is>
+      </c>
+      <c r="G375" s="41" t="inlineStr">
+        <is>
+          <t>Piso 13</t>
+        </is>
+      </c>
+      <c r="H375" s="41" t="n"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B376" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C376" s="41" t="inlineStr">
+        <is>
+          <t>17-34</t>
+        </is>
+      </c>
+      <c r="D376" s="41" t="inlineStr">
+        <is>
+          <t>Rooftop</t>
+        </is>
+      </c>
+      <c r="E376" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad</t>
+        </is>
+      </c>
+      <c r="F376" s="41" t="inlineStr">
+        <is>
+          <t>"No tenemos terraza"</t>
+        </is>
+      </c>
+      <c r="G376" s="41" t="inlineStr">
+        <is>
+          <t>Bar Terraza en el piso 13 con bebidas y alimentos</t>
+        </is>
+      </c>
+      <c r="H376" s="41" t="n"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B377" s="41" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C377" s="41" t="inlineStr">
+        <is>
+          <t>17-61</t>
+        </is>
+      </c>
+      <c r="D377" s="41" t="inlineStr">
+        <is>
+          <t>Swimming pool</t>
+        </is>
+      </c>
+      <c r="E377" s="41" t="inlineStr">
+        <is>
+          <t>Precio público por día</t>
+        </is>
+      </c>
+      <c r="F377" s="41" t="inlineStr">
+        <is>
+          <t>80.000 COP/día</t>
+        </is>
+      </c>
+      <c r="G377" s="41" t="inlineStr">
+        <is>
+          <t>150.000 COP/día</t>
+        </is>
+      </c>
+      <c r="H377" s="41" t="n"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B378" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C378" s="41" t="inlineStr">
+        <is>
+          <t>12-04</t>
+        </is>
+      </c>
+      <c r="D378" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast reservation</t>
+        </is>
+      </c>
+      <c r="E378" s="41" t="inlineStr">
+        <is>
+          <t>Correo para reservar desayuno</t>
+        </is>
+      </c>
+      <c r="F378" s="41" t="inlineStr">
+        <is>
+          <t>reservas.sonestaarequipa@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="G378" s="41" t="inlineStr">
+        <is>
+          <t>restaurante.sonestaarequipa@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="H378" s="41" t="n"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B379" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C379" s="41" t="inlineStr">
+        <is>
+          <t>13-32</t>
+        </is>
+      </c>
+      <c r="D379" s="41" t="inlineStr">
+        <is>
+          <t>Medical services</t>
+        </is>
+      </c>
+      <c r="E379" s="41" t="inlineStr">
+        <is>
+          <t>Números de emergencia</t>
+        </is>
+      </c>
+      <c r="F379" s="41" t="inlineStr">
+        <is>
+          <t>Policía 911, Fuego 911, Ambulancia 911</t>
+        </is>
+      </c>
+      <c r="G379" s="41" t="inlineStr">
+        <is>
+          <t>Policía 105, Fuego 116, Ambulancia 106</t>
+        </is>
+      </c>
+      <c r="H379" s="41" t="n"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B380" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C380" s="41" t="inlineStr">
+        <is>
+          <t>13-48</t>
+        </is>
+      </c>
+      <c r="D380" s="41" t="inlineStr">
+        <is>
+          <t>Currencies</t>
+        </is>
+      </c>
+      <c r="E380" s="41" t="inlineStr">
+        <is>
+          <t>Pagos en propiedad</t>
+        </is>
+      </c>
+      <c r="F380" s="41" t="inlineStr">
+        <is>
+          <t>Solo PEN</t>
+        </is>
+      </c>
+      <c r="G380" s="41" t="inlineStr">
+        <is>
+          <t>PEN y USD</t>
+        </is>
+      </c>
+      <c r="H380" s="41" t="n"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B381" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C381" s="41" t="inlineStr">
+        <is>
+          <t>13-52</t>
+        </is>
+      </c>
+      <c r="D381" s="41" t="inlineStr">
+        <is>
+          <t>Private transfer reservation</t>
+        </is>
+      </c>
+      <c r="E381" s="41" t="inlineStr">
+        <is>
+          <t>Información requerida</t>
+        </is>
+      </c>
+      <c r="F381" s="41" t="inlineStr">
+        <is>
+          <t>Incluía número de vuelo/tren y estación</t>
+        </is>
+      </c>
+      <c r="G381" s="41" t="inlineStr">
+        <is>
+          <t>Se retira estación de tren/aeropuerto</t>
+        </is>
+      </c>
+      <c r="H381" s="41" t="n"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B382" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C382" s="41" t="inlineStr">
+        <is>
+          <t>14-01</t>
+        </is>
+      </c>
+      <c r="D382" s="41" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="E382" s="41" t="inlineStr">
+        <is>
+          <t>Superficie de habitaciones (m²)</t>
+        </is>
+      </c>
+      <c r="F382" s="41" t="inlineStr">
+        <is>
+          <t>28 m² (King/Twin/Ejecutiva)</t>
+        </is>
+      </c>
+      <c r="G382" s="41" t="inlineStr">
+        <is>
+          <t>34 m²; Ejecutiva King pasa a llamarse Superior King</t>
+        </is>
+      </c>
+      <c r="H382" s="41" t="n"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B383" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C383" s="41" t="inlineStr">
+        <is>
+          <t>14-04</t>
+        </is>
+      </c>
+      <c r="D383" s="41" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="E383" s="41" t="inlineStr">
+        <is>
+          <t>Detectores y tarifa limpieza</t>
+        </is>
+      </c>
+      <c r="F383" s="41" t="inlineStr">
+        <is>
+          <t>Sin detectores; tarifa 0 PEN</t>
+        </is>
+      </c>
+      <c r="G383" s="41" t="inlineStr">
+        <is>
+          <t>Con detectores; tarifa USD 200</t>
+        </is>
+      </c>
+      <c r="H383" s="41" t="n"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B384" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C384" s="41" t="inlineStr">
+        <is>
+          <t>15-06</t>
+        </is>
+      </c>
+      <c r="D384" s="41" t="inlineStr">
+        <is>
+          <t>Bathroom equipment</t>
+        </is>
+      </c>
+      <c r="E384" s="41" t="inlineStr">
+        <is>
+          <t>Amenidades gratuitas a petición</t>
+        </is>
+      </c>
+      <c r="F384" s="41" t="inlineStr">
+        <is>
+          <t>Pantuflas, pasta dientes, kit afeitar</t>
+        </is>
+      </c>
+      <c r="G384" s="41" t="inlineStr">
+        <is>
+          <t>Pantuflas, vanity kit, kit dental, kit afeitar, peine</t>
+        </is>
+      </c>
+      <c r="H384" s="41" t="n"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B385" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C385" s="41" t="inlineStr">
+        <is>
+          <t>15-09</t>
+        </is>
+      </c>
+      <c r="D385" s="41" t="inlineStr">
+        <is>
+          <t>Shower/bathtub</t>
+        </is>
+      </c>
+      <c r="E385" s="41" t="inlineStr">
+        <is>
+          <t>Nombres de categorías</t>
+        </is>
+      </c>
+      <c r="F385" s="41" t="inlineStr">
+        <is>
+          <t>Ejecutiva King</t>
+        </is>
+      </c>
+      <c r="G385" s="41" t="inlineStr">
+        <is>
+          <t>Superior King</t>
+        </is>
+      </c>
+      <c r="H385" s="41" t="n"/>
+    </row>
+    <row r="386">
+      <c r="A386" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B386" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C386" s="41" t="inlineStr">
+        <is>
+          <t>15-21</t>
+        </is>
+      </c>
+      <c r="D386" s="41" t="inlineStr">
+        <is>
+          <t>Bedding</t>
+        </is>
+      </c>
+      <c r="E386" s="41" t="inlineStr">
+        <is>
+          <t>Nombres de categorías</t>
+        </is>
+      </c>
+      <c r="F386" s="41" t="inlineStr">
+        <is>
+          <t>Ejecutiva King</t>
+        </is>
+      </c>
+      <c r="G386" s="41" t="inlineStr">
+        <is>
+          <t>Superior King</t>
+        </is>
+      </c>
+      <c r="H386" s="41" t="n"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B387" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C387" s="41" t="inlineStr">
+        <is>
+          <t>16-06</t>
+        </is>
+      </c>
+      <c r="D387" s="41" t="inlineStr">
+        <is>
+          <t>Jobs &amp; internships</t>
+        </is>
+      </c>
+      <c r="E387" s="41" t="inlineStr">
+        <is>
+          <t>Correo y teléfono RR.HH.</t>
+        </is>
+      </c>
+      <c r="F387" s="41" t="inlineStr">
+        <is>
+          <t>contactenos@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="G387" s="41" t="inlineStr">
+        <is>
+          <t>laydy.pauca@ghlhoteles.com / +054 308 777</t>
+        </is>
+      </c>
+      <c r="H387" s="41" t="n"/>
+    </row>
+    <row r="388">
+      <c r="A388" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B388" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C388" s="41" t="inlineStr">
+        <is>
+          <t>16-25</t>
+        </is>
+      </c>
+      <c r="D388" s="41" t="inlineStr">
+        <is>
+          <t>Tips policy</t>
+        </is>
+      </c>
+      <c r="E388" s="41" t="inlineStr">
+        <is>
+          <t>Redacción de la política</t>
+        </is>
+      </c>
+      <c r="F388" s="41" t="inlineStr">
+        <is>
+          <t>Incluía "es costumbre dejar propina"</t>
+        </is>
+      </c>
+      <c r="G388" s="41" t="inlineStr">
+        <is>
+          <t>Se retira esa línea</t>
+        </is>
+      </c>
+      <c r="H388" s="41" t="n"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B389" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C389" s="41" t="inlineStr">
+        <is>
+          <t>17-31</t>
+        </is>
+      </c>
+      <c r="D389" s="41" t="inlineStr">
+        <is>
+          <t>Fitness gym</t>
+        </is>
+      </c>
+      <c r="E389" s="41" t="inlineStr">
+        <is>
+          <t>Equipamiento</t>
+        </is>
+      </c>
+      <c r="F389" s="41" t="inlineStr">
+        <is>
+          <t>Incluía bicicleta estática</t>
+        </is>
+      </c>
+      <c r="G389" s="41" t="inlineStr">
+        <is>
+          <t>Se retira bicicleta estática</t>
+        </is>
+      </c>
+      <c r="H389" s="41" t="n"/>
+    </row>
+    <row r="390">
+      <c r="A390" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B390" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C390" s="41" t="inlineStr">
+        <is>
+          <t>17-41</t>
+        </is>
+      </c>
+      <c r="D390" s="41" t="inlineStr">
+        <is>
+          <t>Heating &amp; cooling</t>
+        </is>
+      </c>
+      <c r="E390" s="41" t="inlineStr">
+        <is>
+          <t>Nombre de equipo y tipo A/A</t>
+        </is>
+      </c>
+      <c r="F390" s="41" t="inlineStr">
+        <is>
+          <t>"Radiador"; tipo Reversible (Caliente/Frío)</t>
+        </is>
+      </c>
+      <c r="G390" s="41" t="inlineStr">
+        <is>
+          <t>"Calefactor"; tipo Frío únicamente</t>
+        </is>
+      </c>
+      <c r="H390" s="41" t="n"/>
+    </row>
+    <row r="391">
+      <c r="A391" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B391" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C391" s="41" t="inlineStr">
+        <is>
+          <t>19-03</t>
+        </is>
+      </c>
+      <c r="D391" s="41" t="inlineStr">
+        <is>
+          <t>City center</t>
+        </is>
+      </c>
+      <c r="E391" s="41" t="inlineStr">
+        <is>
+          <t>Redacción de indicaciones</t>
+        </is>
+      </c>
+      <c r="F391" s="41" t="inlineStr">
+        <is>
+          <t>Incluía tiempo a pie</t>
+        </is>
+      </c>
+      <c r="G391" s="41" t="inlineStr">
+        <is>
+          <t>Se simplifica, solo enlace de indicaciones</t>
+        </is>
+      </c>
+      <c r="H391" s="41" t="n"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B392" s="41" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C392" s="41" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="D392" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E392" s="41" t="inlineStr">
+        <is>
+          <t>Nombre del restaurante</t>
+        </is>
+      </c>
+      <c r="F392" s="41" t="inlineStr">
+        <is>
+          <t>Restaurante Corozo &amp; Timbal</t>
+        </is>
+      </c>
+      <c r="G392" s="41" t="inlineStr">
+        <is>
+          <t>Restaurante Úrsula</t>
+        </is>
+      </c>
+      <c r="H392" s="41" t="n"/>
+    </row>
+    <row r="393">
+      <c r="A393" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B393" s="41" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C393" s="41" t="inlineStr">
+        <is>
+          <t>17-31</t>
+        </is>
+      </c>
+      <c r="D393" s="41" t="inlineStr">
+        <is>
+          <t>Fitness gym</t>
+        </is>
+      </c>
+      <c r="E393" s="41" t="inlineStr">
+        <is>
+          <t>Equipamiento</t>
+        </is>
+      </c>
+      <c r="F393" s="41" t="inlineStr">
+        <is>
+          <t>Incluía máquina de remo</t>
+        </is>
+      </c>
+      <c r="G393" s="41" t="inlineStr">
+        <is>
+          <t>Se retira máquina de remo</t>
+        </is>
+      </c>
+      <c r="H393" s="41" t="n"/>
+    </row>
+    <row r="394">
+      <c r="A394" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B394" s="41" t="inlineStr">
+        <is>
+          <t>Hotel Tequendama Bogotá</t>
+        </is>
+      </c>
+      <c r="C394" s="41" t="inlineStr">
+        <is>
+          <t>13-06</t>
+        </is>
+      </c>
+      <c r="D394" s="41" t="inlineStr">
+        <is>
+          <t>Room service</t>
+        </is>
+      </c>
+      <c r="E394" s="41" t="inlineStr">
+        <is>
+          <t>Código de marcado</t>
+        </is>
+      </c>
+      <c r="F394" s="41" t="inlineStr">
+        <is>
+          <t>Marcar 2</t>
+        </is>
+      </c>
+      <c r="G394" s="41" t="inlineStr">
+        <is>
+          <t>Marcar *2</t>
+        </is>
+      </c>
+      <c r="H394" s="41" t="n"/>
+    </row>
+    <row r="395">
+      <c r="A395" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B395" s="41" t="inlineStr">
+        <is>
+          <t>Hotel Tequendama Bogotá</t>
+        </is>
+      </c>
+      <c r="C395" s="41" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D395" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E395" s="41" t="inlineStr">
+        <is>
+          <t>Días de apertura Café Vienes</t>
+        </is>
+      </c>
+      <c r="F395" s="41" t="inlineStr">
+        <is>
+          <t>Abierto 7/7</t>
+        </is>
+      </c>
+      <c r="G395" s="41" t="inlineStr">
+        <is>
+          <t>Abierto de lunes a viernes</t>
+        </is>
+      </c>
+      <c r="H395" s="41" t="n"/>
+    </row>
+    <row r="396">
+      <c r="A396" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B396" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C396" s="41" t="inlineStr">
+        <is>
+          <t>10-13</t>
+        </is>
+      </c>
+      <c r="D396" s="41" t="inlineStr">
+        <is>
+          <t>Opening, closing &amp; renovation</t>
+        </is>
+      </c>
+      <c r="E396" s="41" t="inlineStr">
+        <is>
+          <t>Fecha fin remodelación</t>
+        </is>
+      </c>
+      <c r="F396" s="41" t="inlineStr">
+        <is>
+          <t>30 de agosto de 2026</t>
+        </is>
+      </c>
+      <c r="G396" s="41" t="inlineStr">
+        <is>
+          <t>30 de septiembre de 2026</t>
+        </is>
+      </c>
+      <c r="H396" s="41" t="n"/>
+    </row>
+    <row r="397">
+      <c r="A397" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B397" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C397" s="41" t="inlineStr">
+        <is>
+          <t>10-42</t>
+        </is>
+      </c>
+      <c r="D397" s="41" t="inlineStr">
+        <is>
+          <t>Day use reservation</t>
+        </is>
+      </c>
+      <c r="E397" s="41" t="inlineStr">
+        <is>
+          <t>Fecha fin remodelación</t>
+        </is>
+      </c>
+      <c r="F397" s="41" t="inlineStr">
+        <is>
+          <t>31 de agosto</t>
+        </is>
+      </c>
+      <c r="G397" s="41" t="inlineStr">
+        <is>
+          <t>30 de septiembre</t>
+        </is>
+      </c>
+      <c r="H397" s="41" t="n"/>
+    </row>
+    <row r="398">
+      <c r="A398" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B398" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C398" s="41" t="inlineStr">
+        <is>
+          <t>15-23</t>
+        </is>
+      </c>
+      <c r="D398" s="41" t="inlineStr">
+        <is>
+          <t>Extra bed</t>
+        </is>
+      </c>
+      <c r="E398" s="41" t="inlineStr">
+        <is>
+          <t>Precio por noche</t>
+        </is>
+      </c>
+      <c r="F398" s="41" t="inlineStr">
+        <is>
+          <t>80.000 COP</t>
+        </is>
+      </c>
+      <c r="G398" s="41" t="inlineStr">
+        <is>
+          <t>90.000 COP</t>
+        </is>
+      </c>
+      <c r="H398" s="41" t="n"/>
+    </row>
+    <row r="399">
+      <c r="A399" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B399" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C399" s="41" t="inlineStr">
+        <is>
+          <t>15-62</t>
+        </is>
+      </c>
+      <c r="D399" s="41" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="E399" s="41" t="inlineStr">
+        <is>
+          <t>Redacción de la vista</t>
+        </is>
+      </c>
+      <c r="F399" s="41" t="inlineStr">
+        <is>
+          <t>Depende de la ubicación asignada</t>
+        </is>
+      </c>
+      <c r="G399" s="41" t="inlineStr">
+        <is>
+          <t>Vista interna, depende de la ubicación asignada</t>
+        </is>
+      </c>
+      <c r="H399" s="41" t="n"/>
+    </row>
+    <row r="400">
+      <c r="A400" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B400" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C400" s="41" t="inlineStr">
+        <is>
+          <t>15-81</t>
+        </is>
+      </c>
+      <c r="D400" s="41" t="inlineStr">
+        <is>
+          <t>TV</t>
+        </is>
+      </c>
+      <c r="E400" s="41" t="inlineStr">
+        <is>
+          <t>Guía de canales</t>
+        </is>
+      </c>
+      <c r="F400" s="41" t="inlineStr">
+        <is>
+          <t>Disponible en app GHL Plus</t>
+        </is>
+      </c>
+      <c r="G400" s="41" t="inlineStr">
+        <is>
+          <t>Se retira mención de la app</t>
+        </is>
+      </c>
+      <c r="H400" s="41" t="n"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B401" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C401" s="41" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D401" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E401" s="41" t="inlineStr">
+        <is>
+          <t>Máximo de mascotas y correa</t>
+        </is>
+      </c>
+      <c r="F401" s="41" t="inlineStr">
+        <is>
+          <t>Máx. 2 mascotas por habitación</t>
+        </is>
+      </c>
+      <c r="G401" s="41" t="inlineStr">
+        <is>
+          <t>Máx. 1 mascota; se exige correa</t>
+        </is>
+      </c>
+      <c r="H401" s="41" t="n"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B402" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C402" s="41" t="inlineStr">
+        <is>
+          <t>17-11</t>
+        </is>
+      </c>
+      <c r="D402" s="41" t="inlineStr">
+        <is>
+          <t>Spa reservation</t>
+        </is>
+      </c>
+      <c r="E402" s="41" t="inlineStr">
+        <is>
+          <t>Método de contacto</t>
+        </is>
+      </c>
+      <c r="F402" s="41" t="inlineStr">
+        <is>
+          <t>Reservar por correo</t>
+        </is>
+      </c>
+      <c r="G402" s="41" t="inlineStr">
+        <is>
+          <t>Teléfono/WhatsApp +57 3138725411</t>
+        </is>
+      </c>
+      <c r="H402" s="41" t="n"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B403" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C403" s="41" t="inlineStr">
+        <is>
+          <t>17-41</t>
+        </is>
+      </c>
+      <c r="D403" s="41" t="inlineStr">
+        <is>
+          <t>Heating &amp; cooling</t>
+        </is>
+      </c>
+      <c r="E403" s="41" t="inlineStr">
+        <is>
+          <t>Sistema de climatización</t>
+        </is>
+      </c>
+      <c r="F403" s="41" t="inlineStr">
+        <is>
+          <t>Sistemas de regulación de temperatura</t>
+        </is>
+      </c>
+      <c r="G403" s="41" t="inlineStr">
+        <is>
+          <t>Ambiente con temperatura natural de la región (sin A/A)</t>
+        </is>
+      </c>
+      <c r="H403" s="41" t="n"/>
+    </row>
+    <row r="404">
+      <c r="A404" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B404" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C404" s="41" t="inlineStr">
+        <is>
+          <t>17-43</t>
+        </is>
+      </c>
+      <c r="D404" s="41" t="inlineStr">
+        <is>
+          <t>Floor arrangement</t>
+        </is>
+      </c>
+      <c r="E404" s="41" t="inlineStr">
+        <is>
+          <t>Ubicación Superior Twin</t>
+        </is>
+      </c>
+      <c r="F404" s="41" t="inlineStr">
+        <is>
+          <t>Solo planta baja</t>
+        </is>
+      </c>
+      <c r="G404" s="41" t="inlineStr">
+        <is>
+          <t>Planta baja y planta alta</t>
+        </is>
+      </c>
+      <c r="H404" s="41" t="n"/>
+    </row>
+    <row r="405">
+      <c r="A405" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B405" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C405" s="41" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D405" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E405" s="41" t="inlineStr">
+        <is>
+          <t>Código de vestimenta</t>
+        </is>
+      </c>
+      <c r="F405" s="41" t="inlineStr">
+        <is>
+          <t>Casual con detalle de outfits</t>
+        </is>
+      </c>
+      <c r="G405" s="41" t="inlineStr">
+        <is>
+          <t>Casual; no se permite traje de baño ni ropa húmeda</t>
+        </is>
+      </c>
+      <c r="H405" s="41" t="n"/>
+    </row>
+    <row r="406">
+      <c r="A406" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B406" s="41" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C406" s="41" t="inlineStr">
+        <is>
+          <t>20-21</t>
+        </is>
+      </c>
+      <c r="D406" s="41" t="inlineStr">
+        <is>
+          <t>Celebration</t>
+        </is>
+      </c>
+      <c r="E406" s="41" t="inlineStr">
+        <is>
+          <t>Teléfono de eventos</t>
+        </is>
+      </c>
+      <c r="F406" s="41" t="inlineStr">
+        <is>
+          <t>+57 601 8366824</t>
+        </is>
+      </c>
+      <c r="G406" s="41" t="inlineStr">
+        <is>
+          <t>+57 321 469 3086</t>
+        </is>
+      </c>
+      <c r="H406" s="41" t="n"/>
+    </row>
+    <row r="407">
+      <c r="A407" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B407" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bucaramanga</t>
+        </is>
+      </c>
+      <c r="C407" s="41" t="inlineStr">
+        <is>
+          <t>13-06</t>
+        </is>
+      </c>
+      <c r="D407" s="41" t="inlineStr">
+        <is>
+          <t>Room service</t>
+        </is>
+      </c>
+      <c r="E407" s="41" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="F407" s="41" t="inlineStr">
+        <is>
+          <t>Disponible 24/7</t>
+        </is>
+      </c>
+      <c r="G407" s="41" t="inlineStr">
+        <is>
+          <t>06:00 a 22:00, jornada continua</t>
+        </is>
+      </c>
+      <c r="H407" s="41" t="n"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B408" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bucaramanga</t>
+        </is>
+      </c>
+      <c r="C408" s="41" t="inlineStr">
+        <is>
+          <t>17-01</t>
+        </is>
+      </c>
+      <c r="D408" s="41" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="E408" s="41" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="F408" s="41" t="inlineStr">
+        <is>
+          <t>Lun-Jue 12:00-23:00; Vie-Sáb 12:00-23:59</t>
+        </is>
+      </c>
+      <c r="G408" s="41" t="inlineStr">
+        <is>
+          <t>Dom-Lun 12:00-22:00; Vie-Sáb 12:00-23:00</t>
+        </is>
+      </c>
+      <c r="H408" s="41" t="n"/>
+    </row>
+    <row r="409">
+      <c r="A409" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B409" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bucaramanga</t>
+        </is>
+      </c>
+      <c r="C409" s="41" t="inlineStr">
+        <is>
+          <t>17-34</t>
+        </is>
+      </c>
+      <c r="D409" s="41" t="inlineStr">
+        <is>
+          <t>Rooftop</t>
+        </is>
+      </c>
+      <c r="E409" s="41" t="inlineStr">
+        <is>
+          <t>Días y horario</t>
+        </is>
+      </c>
+      <c r="F409" s="41" t="inlineStr">
+        <is>
+          <t>Cerrado domingos; horarios variables</t>
+        </is>
+      </c>
+      <c r="G409" s="41" t="inlineStr">
+        <is>
+          <t>Abierto todos los días; horario unificado (Vie-Sáb hasta 23:00, resto hasta 22:00)</t>
+        </is>
+      </c>
+      <c r="H409" s="41" t="n"/>
+    </row>
+    <row r="410">
+      <c r="A410" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B410" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Bucaramanga</t>
+        </is>
+      </c>
+      <c r="C410" s="41" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D410" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E410" s="41" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="F410" s="41" t="inlineStr">
+        <is>
+          <t>Variable por día hasta 00:00 Vie-Sáb</t>
+        </is>
+      </c>
+      <c r="G410" s="41" t="inlineStr">
+        <is>
+          <t>Horario unificado, Vie-Sáb hasta 23:00, resto hasta 22:00</t>
+        </is>
+      </c>
+      <c r="H410" s="41" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H227"/>

</xml_diff>

<commit_message>
Registra 7 diálogos de Sonesta Puno para agosto
Delmy Nuñez envió el formato de manera informal (Antes/Ahora en vez de
Antes/Después); se interpreta "Ahora" como el valor "después" según
indicación de Santiago, y se marca "⚠ No especificado" donde no dio un
valor "antes". Estado: Pendiente actualización.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -6650,14 +6650,29 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K127" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>7 diálogos modificados: desayuno, taxi, habitaciones conectadas, ducha/tina, mascotas, restaurante, celebraciones</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>El hotel envió el formato de manera informal (Antes/Ahora); se interpretó "Ahora" como el valor "después"</t>
+        </is>
+      </c>
+      <c r="K127" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -6912,13 +6927,13 @@
         <v>42</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F6" s="12" t="n">
         <v>4</v>
@@ -6928,7 +6943,7 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="I6" s="17">
@@ -7051,23 +7066,23 @@
         <v>42</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F4" s="19" t="n">
         <v>4</v>
       </c>
       <c r="G4" s="20" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.4047619047619048</v>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>███████████░░░░░░░░░░░░░░░░░░░</t>
+          <t>████████████░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I4" s="22" t="inlineStr">
@@ -7156,19 +7171,19 @@
         <v>126</v>
       </c>
       <c r="C7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D7" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E7" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F7" t="n">
         <v>12</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4365079365079365</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -7200,7 +7215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H410"/>
+  <dimension ref="A1:H417"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22750,6 +22765,272 @@
         </is>
       </c>
       <c r="H410" s="41" t="n"/>
+    </row>
+    <row r="411">
+      <c r="A411" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B411" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Puno</t>
+        </is>
+      </c>
+      <c r="C411" s="41" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="D411" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E411" s="41" t="inlineStr">
+        <is>
+          <t>Horario y precio</t>
+        </is>
+      </c>
+      <c r="F411" s="41" t="inlineStr">
+        <is>
+          <t>10:30am; precio sin especificar</t>
+        </is>
+      </c>
+      <c r="G411" s="41" t="inlineStr">
+        <is>
+          <t>09:30am; USD 18.00</t>
+        </is>
+      </c>
+      <c r="H411" s="41" t="n"/>
+    </row>
+    <row r="412">
+      <c r="A412" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B412" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Puno</t>
+        </is>
+      </c>
+      <c r="C412" s="41" t="inlineStr">
+        <is>
+          <t>13-53</t>
+        </is>
+      </c>
+      <c r="D412" s="41" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="E412" s="41" t="inlineStr">
+        <is>
+          <t>Precios</t>
+        </is>
+      </c>
+      <c r="F412" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G412" s="41" t="inlineStr">
+        <is>
+          <t>Downtown $6.00; Aeropuerto Juliaca $80.00</t>
+        </is>
+      </c>
+      <c r="H412" s="41" t="n"/>
+    </row>
+    <row r="413">
+      <c r="A413" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B413" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Puno</t>
+        </is>
+      </c>
+      <c r="C413" s="41" t="inlineStr">
+        <is>
+          <t>14-03</t>
+        </is>
+      </c>
+      <c r="D413" s="41" t="inlineStr">
+        <is>
+          <t>Family accommodation</t>
+        </is>
+      </c>
+      <c r="E413" s="41" t="inlineStr">
+        <is>
+          <t>Habitaciones conectadas</t>
+        </is>
+      </c>
+      <c r="F413" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G413" s="41" t="inlineStr">
+        <is>
+          <t>Se elimina la mención de habitaciones conectadas</t>
+        </is>
+      </c>
+      <c r="H413" s="41" t="n"/>
+    </row>
+    <row r="414">
+      <c r="A414" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B414" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Puno</t>
+        </is>
+      </c>
+      <c r="C414" s="41" t="inlineStr">
+        <is>
+          <t>15-09</t>
+        </is>
+      </c>
+      <c r="D414" s="41" t="inlineStr">
+        <is>
+          <t>Shower, bathtub, jacuzzi, pool</t>
+        </is>
+      </c>
+      <c r="E414" s="41" t="inlineStr">
+        <is>
+          <t>Ducha y tina</t>
+        </is>
+      </c>
+      <c r="F414" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G414" s="41" t="inlineStr">
+        <is>
+          <t>Disponibles con garantía desde reservas</t>
+        </is>
+      </c>
+      <c r="H414" s="41" t="n"/>
+    </row>
+    <row r="415">
+      <c r="A415" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B415" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Puno</t>
+        </is>
+      </c>
+      <c r="C415" s="41" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D415" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E415" s="41" t="inlineStr">
+        <is>
+          <t>Restricciones y tasas por daños</t>
+        </is>
+      </c>
+      <c r="F415" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G415" s="41" t="inlineStr">
+        <is>
+          <t>Máximo 1 mascota hasta 15kg; tasas por daños: USD 80 muebles, USD 50 lencería, USD 400 colchón</t>
+        </is>
+      </c>
+      <c r="H415" s="41" t="n"/>
+    </row>
+    <row r="416">
+      <c r="A416" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B416" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Puno</t>
+        </is>
+      </c>
+      <c r="C416" s="41" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D416" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E416" s="41" t="inlineStr">
+        <is>
+          <t>Picnic y capacidad Inkafe</t>
+        </is>
+      </c>
+      <c r="F416" s="41" t="inlineStr">
+        <is>
+          <t>⚠ No especificado</t>
+        </is>
+      </c>
+      <c r="G416" s="41" t="inlineStr">
+        <is>
+          <t>Picnic con reserva mínimo 24h antes; capacidad máxima Inkafe 90 personas</t>
+        </is>
+      </c>
+      <c r="H416" s="41" t="n"/>
+    </row>
+    <row r="417">
+      <c r="A417" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B417" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Puno</t>
+        </is>
+      </c>
+      <c r="C417" s="41" t="inlineStr">
+        <is>
+          <t>20-21</t>
+        </is>
+      </c>
+      <c r="D417" s="41" t="inlineStr">
+        <is>
+          <t>Celebration</t>
+        </is>
+      </c>
+      <c r="E417" s="41" t="inlineStr">
+        <is>
+          <t>Correo de contacto</t>
+        </is>
+      </c>
+      <c r="F417" s="41" t="inlineStr">
+        <is>
+          <t>ubaldo.laquise@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="G417" s="41" t="inlineStr">
+        <is>
+          <t>restaurante.spipuno@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="H417" s="41" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H227"/>

</xml_diff>

<commit_message>
Registra 4 diálogos de GHL Style Barrancabermeja para agosto
Contenido del Word adjunto (INFORMACIÓN A ACTUALIZAR HOTEL.docx) provisto
directamente por Santiago: contacto eventos, tarifa desayuno, horario y
acceso del bar, horario de la terraza. Estado: Pendiente actualización.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -5736,14 +5736,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K105" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>4 diálogos modificados: contacto eventos, desayuno, bar, terraza</t>
+        </is>
+      </c>
+      <c r="K105" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -6927,13 +6937,13 @@
         <v>42</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F6" s="12" t="n">
         <v>4</v>
@@ -6943,7 +6953,7 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="I6" s="17">
@@ -7066,23 +7076,23 @@
         <v>42</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F4" s="19" t="n">
         <v>4</v>
       </c>
       <c r="G4" s="20" t="n">
-        <v>0.4047619047619048</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>████████████░░░░░░░░░░░░░░░░░░</t>
+          <t>█████████████░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I4" s="22" t="inlineStr">
@@ -7171,23 +7181,23 @@
         <v>126</v>
       </c>
       <c r="C7" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D7" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E7" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F7" t="n">
         <v>12</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.4523809523809524</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>█████████████░░░░░░░░░░░░░░░░░</t>
+          <t>██████████████░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -7215,7 +7225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H417"/>
+  <dimension ref="A1:H421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23031,6 +23041,158 @@
         </is>
       </c>
       <c r="H417" s="41" t="n"/>
+    </row>
+    <row r="418">
+      <c r="A418" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B418" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Barrancabermeja</t>
+        </is>
+      </c>
+      <c r="C418" s="41" t="inlineStr">
+        <is>
+          <t>16-02</t>
+        </is>
+      </c>
+      <c r="D418" s="41" t="inlineStr">
+        <is>
+          <t>Contact staff</t>
+        </is>
+      </c>
+      <c r="E418" s="41" t="inlineStr">
+        <is>
+          <t>Teléfono Eventos</t>
+        </is>
+      </c>
+      <c r="F418" s="41" t="inlineStr">
+        <is>
+          <t>+57 319 7530014</t>
+        </is>
+      </c>
+      <c r="G418" s="41" t="inlineStr">
+        <is>
+          <t>+57 311 2845935</t>
+        </is>
+      </c>
+      <c r="H418" s="41" t="n"/>
+    </row>
+    <row r="419">
+      <c r="A419" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B419" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Barrancabermeja</t>
+        </is>
+      </c>
+      <c r="C419" s="41" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="D419" s="41" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E419" s="41" t="inlineStr">
+        <is>
+          <t>Precio por adulto</t>
+        </is>
+      </c>
+      <c r="F419" s="41" t="inlineStr">
+        <is>
+          <t>36.000 COP</t>
+        </is>
+      </c>
+      <c r="G419" s="41" t="inlineStr">
+        <is>
+          <t>59.000 COP</t>
+        </is>
+      </c>
+      <c r="H419" s="41" t="n"/>
+    </row>
+    <row r="420">
+      <c r="A420" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B420" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Barrancabermeja</t>
+        </is>
+      </c>
+      <c r="C420" s="41" t="inlineStr">
+        <is>
+          <t>17-01</t>
+        </is>
+      </c>
+      <c r="D420" s="41" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="E420" s="41" t="inlineStr">
+        <is>
+          <t>Horario y acceso</t>
+        </is>
+      </c>
+      <c r="F420" s="41" t="inlineStr">
+        <is>
+          <t>17:00 a 22:00; solo clientes del hotel</t>
+        </is>
+      </c>
+      <c r="G420" s="41" t="inlineStr">
+        <is>
+          <t>11:00 a 22:00; abierto para visitantes y huéspedes</t>
+        </is>
+      </c>
+      <c r="H420" s="41" t="n"/>
+    </row>
+    <row r="421">
+      <c r="A421" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B421" s="41" t="inlineStr">
+        <is>
+          <t>GHL Style Barrancabermeja</t>
+        </is>
+      </c>
+      <c r="C421" s="41" t="inlineStr">
+        <is>
+          <t>17-34</t>
+        </is>
+      </c>
+      <c r="D421" s="41" t="inlineStr">
+        <is>
+          <t>Rooftop</t>
+        </is>
+      </c>
+      <c r="E421" s="41" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="F421" s="41" t="inlineStr">
+        <is>
+          <t>17:00 a 22:00 todos los días</t>
+        </is>
+      </c>
+      <c r="G421" s="41" t="inlineStr">
+        <is>
+          <t>11:00 a 22:00 todos los días</t>
+        </is>
+      </c>
+      <c r="H421" s="41" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H227"/>

</xml_diff>

<commit_message>
Registra nuevo contacto de Park Lake Luxury y corrige detección de cambios
- Park Lake Luxury (Ago-26): nuevo contacto Sergio Víctor Alejandro Yevenes
  Escobar (Jefe de Recepción), sergio.yevenes@ghlhoteles.com — antes solo se
  tenía el correo genérico de reservas sin nombre de contacto.
- Corrige listCambiosContacto(): la función descartaba cualquier transición
  donde uno de los ciclos tuviera "—" (sin contacto), justo el caso más
  importante de detectar (pasar de sin contacto a un contacto real).
- Bioxury y Sonesta Bogotá: se verificó que el contacto actual ya coincide
  con la información más reciente proporcionada; no requirieron cambios en
  los ciclos ya registrados (Jun/Jul/Ago-26).
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -6106,22 +6106,27 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
+          <t>Sergio Víctor Alejandro Yevenes Escobar</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>sergio.yevenes@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>reservas.parklake@ghlhoteles.com</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Nuevo contacto: Jefe de Recepción. Antes solo se tenía el correo genérico reservas.parklake@ghlhoteles.com, sin nombre de contacto.</t>
         </is>
       </c>
       <c r="K114" s="44" t="inlineStr">

</xml_diff>

<commit_message>
Registra respuesta de Bioxury para Ago-26: mascotas y restaurante
Bioxury respondió el 06/08/2026. Comparando el PDF nuevo contra el anterior
(el anterior solo tenía texto extraíble en las secciones editadas en rojo),
se confirmaron 7 cambios reales en 2 diálogos:
- 16-10 Pets: máximo de mascotas (2→1), peso máximo (5→10kg), altura máxima
  (20→30cm), tasa (90.000→119.000 COP/día), zonas excluidas (+Playas,
  +Gitane), cama para mascotas (no disponible→disponible gratis).
- 18-01 Restaurant: horario Restaurante Salvaje (12:00–20:00→12:00–21:00).

Dos hallazgos ambiguos (10-71 Payment method: solo cambio de idioma en
rótulos; 17-43 Floor arrangement: teléfono adicional anotado que no aparece
en el archivo final) se dejaron fuera del registro y se anotaron en
comentarios para verificar con el hotel.
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -5131,14 +5131,29 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K90" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>7 diálogos modificados: mascotas, restaurante</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>⚠ Verificar con el hotel: 10-71 (Payment method) solo cambió el idioma de los rótulos y una nota de 'Moneda Local' que desapareció — no se registró como cambio real. 17-43 (Floor arrangement) tenía anotado un posible teléfono adicional 314 8839675 que no aparece en el archivo final — no se registró.</t>
+        </is>
+      </c>
+      <c r="K90" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -6942,13 +6957,13 @@
         <v>42</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" s="12" t="n">
         <v>4</v>
@@ -6958,7 +6973,7 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="I6" s="17">
@@ -7081,23 +7096,23 @@
         <v>42</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" s="19" t="n">
         <v>4</v>
       </c>
       <c r="G4" s="20" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.4523809523809524</v>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>█████████████░░░░░░░░░░░░░░░░░</t>
+          <t>██████████████░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I4" s="22" t="inlineStr">
@@ -7186,19 +7201,19 @@
         <v>126</v>
       </c>
       <c r="C7" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D7" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E7" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F7" t="n">
         <v>12</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.4603174603174603</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -7230,7 +7245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H421"/>
+  <dimension ref="A1:H428"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23198,6 +23213,272 @@
         </is>
       </c>
       <c r="H421" s="41" t="n"/>
+    </row>
+    <row r="422">
+      <c r="A422" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B422" s="41" t="inlineStr">
+        <is>
+          <t>Bioxury</t>
+        </is>
+      </c>
+      <c r="C422" s="41" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D422" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E422" s="41" t="inlineStr">
+        <is>
+          <t>Máximo mascotas por habitación</t>
+        </is>
+      </c>
+      <c r="F422" s="41" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G422" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H422" s="41" t="n"/>
+    </row>
+    <row r="423">
+      <c r="A423" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B423" s="41" t="inlineStr">
+        <is>
+          <t>Bioxury</t>
+        </is>
+      </c>
+      <c r="C423" s="41" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D423" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E423" s="41" t="inlineStr">
+        <is>
+          <t>Peso máximo</t>
+        </is>
+      </c>
+      <c r="F423" s="41" t="inlineStr">
+        <is>
+          <t>5 kg</t>
+        </is>
+      </c>
+      <c r="G423" s="41" t="inlineStr">
+        <is>
+          <t>10 kg</t>
+        </is>
+      </c>
+      <c r="H423" s="41" t="n"/>
+    </row>
+    <row r="424">
+      <c r="A424" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B424" s="41" t="inlineStr">
+        <is>
+          <t>Bioxury</t>
+        </is>
+      </c>
+      <c r="C424" s="41" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D424" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E424" s="41" t="inlineStr">
+        <is>
+          <t>Altura máxima</t>
+        </is>
+      </c>
+      <c r="F424" s="41" t="inlineStr">
+        <is>
+          <t>20 cm</t>
+        </is>
+      </c>
+      <c r="G424" s="41" t="inlineStr">
+        <is>
+          <t>30 cm</t>
+        </is>
+      </c>
+      <c r="H424" s="41" t="n"/>
+    </row>
+    <row r="425">
+      <c r="A425" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B425" s="41" t="inlineStr">
+        <is>
+          <t>Bioxury</t>
+        </is>
+      </c>
+      <c r="C425" s="41" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D425" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E425" s="41" t="inlineStr">
+        <is>
+          <t>Tasa por mascota</t>
+        </is>
+      </c>
+      <c r="F425" s="41" t="inlineStr">
+        <is>
+          <t>90.000 COP/día</t>
+        </is>
+      </c>
+      <c r="G425" s="41" t="inlineStr">
+        <is>
+          <t>119.000 COP/día</t>
+        </is>
+      </c>
+      <c r="H425" s="41" t="n"/>
+    </row>
+    <row r="426">
+      <c r="A426" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B426" s="41" t="inlineStr">
+        <is>
+          <t>Bioxury</t>
+        </is>
+      </c>
+      <c r="C426" s="41" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D426" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E426" s="41" t="inlineStr">
+        <is>
+          <t>Zonas donde no se permiten mascotas</t>
+        </is>
+      </c>
+      <c r="F426" s="41" t="inlineStr">
+        <is>
+          <t>…Gimnasio y Salvaje</t>
+        </is>
+      </c>
+      <c r="G426" s="41" t="inlineStr">
+        <is>
+          <t>…Playas, Gimnasio, Salvaje y Gitane</t>
+        </is>
+      </c>
+      <c r="H426" s="41" t="n"/>
+    </row>
+    <row r="427">
+      <c r="A427" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B427" s="41" t="inlineStr">
+        <is>
+          <t>Bioxury</t>
+        </is>
+      </c>
+      <c r="C427" s="41" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D427" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E427" s="41" t="inlineStr">
+        <is>
+          <t>Cama para mascotas</t>
+        </is>
+      </c>
+      <c r="F427" s="41" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="G427" s="41" t="inlineStr">
+        <is>
+          <t>Disponible de manera gratuita</t>
+        </is>
+      </c>
+      <c r="H427" s="41" t="n"/>
+    </row>
+    <row r="428">
+      <c r="A428" s="43" t="inlineStr">
+        <is>
+          <t>Ago-26</t>
+        </is>
+      </c>
+      <c r="B428" s="41" t="inlineStr">
+        <is>
+          <t>Bioxury</t>
+        </is>
+      </c>
+      <c r="C428" s="41" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D428" s="41" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E428" s="41" t="inlineStr">
+        <is>
+          <t>Horario apertura Restaurante Salvaje</t>
+        </is>
+      </c>
+      <c r="F428" s="41" t="inlineStr">
+        <is>
+          <t>12:00–20:00</t>
+        </is>
+      </c>
+      <c r="G428" s="41" t="inlineStr">
+        <is>
+          <t>12:00–21:00</t>
+        </is>
+      </c>
+      <c r="H428" s="41" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H227"/>

</xml_diff>

<commit_message>
Marca como Actualizado a los 15 hoteles de Ago-26 pendientes en el chatbot
Todos los hoteles que estaban en estado "Pendiente actualización" (Ago-26)
ya fueron aplicados en el chatbot: Arsenal, Bioxury, Geotel Calama, GHL
Relax Club Hotel el Puente, GHL Style Barrancabermeja, GHL Style Bogotá
Occidente, GHL Style Yopal, Hotel Tequendama Bogotá, GHL Hotel Grand
Barranquilla, Sonesta Bucaramanga, Sonesta El Olivar, Sonesta Arequipa,
Sonesta Bogotá, Sonesta Osorno y Sonesta Puno. Se actualiza fecha de
actualización en chatbot (18/08/2026) y estado a "Actualizado" en HTML y
Excel, más el conteo de "Actualizados en chatbot" en Resumen por ciclo.
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -189,6 +189,11 @@
     <font>
       <name val="Calibri"/>
       <color rgb="00856404"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00006100"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -415,7 +420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -539,6 +544,7 @@
     <xf numFmtId="0" fontId="27" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5062,9 +5068,14 @@
           <t>2 diálogos modificados: Breakfast time, Fitness gym</t>
         </is>
       </c>
-      <c r="K88" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K88" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -5146,14 +5157,19 @@
           <t>7 diálogos modificados: mascotas, restaurante</t>
         </is>
       </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
       <c r="J90" t="inlineStr">
         <is>
           <t>⚠ Verificar con el hotel: 10-71 (Payment method) solo cambió el idioma de los rótulos y una nota de 'Moneda Local' que desapareció — no se registró como cambio real. 17-43 (Floor arrangement) tenía anotado un posible teléfono adicional 314 8839675 que no aparece en el archivo final — no se registró.</t>
         </is>
       </c>
-      <c r="K90" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K90" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -5235,9 +5251,14 @@
           <t>14 diálogos modificados: Contact staff, Laundry/paraguas, Invoice, Currencies, Accommodation, Family accommodation, ...</t>
         </is>
       </c>
-      <c r="K92" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K92" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -5598,9 +5619,14 @@
           <t>11 diálogos modificados: Opening, closing &amp; renovation, Day use reservation, Extra bed, View, TV, Pets, ...</t>
         </is>
       </c>
-      <c r="K101" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K101" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -5766,9 +5792,14 @@
           <t>4 diálogos modificados: contacto eventos, desayuno, bar, terraza</t>
         </is>
       </c>
-      <c r="K105" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K105" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -5813,9 +5844,14 @@
           <t>3 diálogos modificados: Business meetings, Breakfast rates, Private transfer</t>
         </is>
       </c>
-      <c r="K106" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K106" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -5897,9 +5933,14 @@
           <t>7 diálogos modificados: Payment method, Check-in time, Check-out time, Breakfast time, Breakfast rates, Pets, ...</t>
         </is>
       </c>
-      <c r="K108" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K108" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -5944,9 +5985,14 @@
           <t>2 diálogos modificados: Room service, Restaurant</t>
         </is>
       </c>
-      <c r="K109" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K109" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -6028,9 +6074,14 @@
           <t>11 diálogos modificados: City tax, fees &amp; VAT, Payment method, Kids, Private transfer, Taxi, Smoking, ...</t>
         </is>
       </c>
-      <c r="K111" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K111" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -6228,9 +6279,14 @@
           <t>4 diálogos modificados: Room service, Bar, Rooftop, Restaurant</t>
         </is>
       </c>
-      <c r="K116" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K116" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -6396,9 +6452,14 @@
           <t>17 diálogos modificados: Contact staff, Check-in time, Check-out time, Breakfast rates, Parking, Connecting accommodation, ...</t>
         </is>
       </c>
-      <c r="K120" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K120" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -6443,9 +6504,14 @@
           <t>14 diálogos modificados: Breakfast reservation, Medical services, Currencies, Private transfer reservation, Accommodation, Smoking, ...</t>
         </is>
       </c>
-      <c r="K121" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K121" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -6490,9 +6556,14 @@
           <t>5 diálogos modificados: Breakfast time, Breakfast rates, Room service, Extra bed, Balcony &amp; windows</t>
         </is>
       </c>
-      <c r="K122" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K122" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -6611,9 +6682,14 @@
           <t>1 diálogos modificados: Breakfast rates</t>
         </is>
       </c>
-      <c r="K125" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="K125" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -6695,14 +6771,19 @@
           <t>7 diálogos modificados: desayuno, taxi, habitaciones conectadas, ducha/tina, mascotas, restaurante, celebraciones</t>
         </is>
       </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
       <c r="J127" t="inlineStr">
         <is>
           <t>El hotel envió el formato de manera informal (Antes/Ahora); se interpretó "Ahora" como el valor "después"</t>
         </is>
       </c>
-      <c r="K127" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K127" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -6969,7 +7050,7 @@
         <v>4</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>

</xml_diff>